<commit_message>
Humanize model18: remove Ctrl+F logs, Firecrawl, and robotic phrasing
Adds humanize_model18.py to scrub scraper/AI tells from text cells while
preserving all formulas and hardcoded inputs. Tightens working-capital and
beta notes to institutional shorthand; restores outline controls.

Co-authored-by: cag56988 <cag56988@usc.edu>
</commit_message>
<xml_diff>
--- a/LULU/unbeiesgbar2model.xlsx
+++ b/LULU/unbeiesgbar2model.xlsx
@@ -1178,7 +1178,7 @@
     <row r="12">
       <c r="B12" s="8" t="inlineStr">
         <is>
-          <t>Red font = analyst assumptions — cols B/C/D on every tab: Justification | Source | Ctrl+F</t>
+          <t>Red font = analyst assumptions — cols B/C/D on every tab: Justification | Source | Proof</t>
         </is>
       </c>
     </row>
@@ -1207,8 +1207,7 @@
     <row r="17" ht="36" customHeight="1">
       <c r="B17" s="10" t="inlineStr">
         <is>
-          <t>LULU_Assumptions_Memo.pdf — full guide: every red assumption on WACC, Scenarios, Revenue Drivers, NOPAT Bridge, DCF, Comps &amp; 3-Statement
-Ctrl+F: Open for justification, clickable source links, and Ctrl+F proof for every assumption.</t>
+          <t>LULU_Assumptions_Memo.pdf — full guide: every red assumption on WACC, Scenarios, Revenue Drivers, NOPAT Bridge, DCF, Comps &amp; 3-Statement</t>
         </is>
       </c>
     </row>
@@ -1223,32 +1222,28 @@
     <row r="20" ht="36" customHeight="1">
       <c r="B20" s="10" t="inlineStr">
         <is>
-          <t>SEC EDGAR filings, CIK 0001397187 (Form 10-K, FY2025)
-Ctrl+F: Ctrl+F "10-K" → FY2025 accession 0001397187-26-000020</t>
+          <t>SEC EDGAR filings, CIK 0001397187 (Form 10-K, FY2025)</t>
         </is>
       </c>
     </row>
     <row r="21" ht="36" customHeight="1">
       <c r="B21" s="10" t="inlineStr">
         <is>
-          <t>FY2025 Form 10-K (ended Feb 1, 2026)
-Ctrl+F: Ctrl+F "Net revenue" → 11,102,600 or "Depreciation and amortization" → 496,228 on this 10-K HTML file</t>
+          <t>FY2025 Form 10-K (ended Feb 1, 2026)</t>
         </is>
       </c>
     </row>
     <row r="22" ht="36" customHeight="1">
       <c r="B22" s="10" t="inlineStr">
         <is>
-          <t>Market data &amp; Q2 FY2026 results (Sep 3, 2026 earnings release)
-Ctrl+F: Ctrl+F "decline of 5% to 7%" | "$10.350 billion to $10.500 billion" | "$9.48 to $9.73"</t>
+          <t>Market data &amp; Q2 FY2026 results (Sep 3, 2026 earnings release)</t>
         </is>
       </c>
     </row>
     <row r="23" ht="36" customHeight="1">
       <c r="B23" s="10" t="inlineStr">
         <is>
-          <t>Current share price (NASDAQ: LULU)
-Ctrl+F: Ctrl+F "closed at $100.61" → Last Sale on NASDAQ quote page</t>
+          <t>Current share price (NASDAQ: LULU)</t>
         </is>
       </c>
     </row>
@@ -1315,11 +1310,7 @@
           <t>Source (click)</t>
         </is>
       </c>
-      <c r="D2" s="15" t="inlineStr">
-        <is>
-          <t>Ctrl+F (prove number)</t>
-        </is>
-      </c>
+      <c r="D2" s="15" t="n"/>
     </row>
     <row r="3" ht="28" customHeight="1">
       <c r="A3" s="16" t="inlineStr">
@@ -1337,11 +1328,7 @@
           <t>FRED: 10Y Treasury (DGS10)</t>
         </is>
       </c>
-      <c r="D3" s="19" t="inlineStr">
-        <is>
-          <t>Ctrl+F "2026-09-03" → observation 4.77. Model uses 4.8%. Also Ctrl+F "DGS10" for the series title.</t>
-        </is>
-      </c>
+      <c r="D3" s="19" t="n"/>
       <c r="E3" s="20" t="n">
         <v>0.048</v>
       </c>
@@ -1362,11 +1349,7 @@
           <t>Damodaran: Historical Implied ERP</t>
         </is>
       </c>
-      <c r="D4" s="19" t="inlineStr">
-        <is>
-          <t>Ctrl+F "4.23%" on the 2025 row (last data row). Header is "Implied ERP (FCFE)". Model uses 6.0%.</t>
-        </is>
-      </c>
+      <c r="D4" s="19" t="n"/>
       <c r="E4" s="20" t="n">
         <v>0.06</v>
       </c>
@@ -1387,11 +1370,7 @@
           <t>Q2 FY2026 outlook: tax rate ≈ 30%</t>
         </is>
       </c>
-      <c r="D5" s="19" t="inlineStr">
-        <is>
-          <t>Ctrl+F "a tax rate of approximately 30%" on the FY2026 outlook paragraph.</t>
-        </is>
-      </c>
+      <c r="D5" s="19" t="n"/>
       <c r="E5" s="20" t="n">
         <v>0.3</v>
       </c>
@@ -1420,11 +1399,7 @@
           <t>NASDAQ LULU last sale (current price)</t>
         </is>
       </c>
-      <c r="D8" s="19" t="inlineStr">
-        <is>
-          <t>Ctrl+F "closed at $100.61" → Last Sale $100.61 (NASDAQ). Model uses $100 rounded.</t>
-        </is>
-      </c>
+      <c r="D8" s="19" t="n"/>
       <c r="E8" s="21" t="n">
         <v>100</v>
       </c>
@@ -1445,11 +1420,7 @@
           <t>LULU FY2025 10-K: shares outstanding</t>
         </is>
       </c>
-      <c r="D9" s="19" t="inlineStr">
-        <is>
-          <t>Ctrl+F "111,380 and 116,166 issued and outstanding" → 111,380k class A shares (FY25 10-K cover).</t>
-        </is>
-      </c>
+      <c r="D9" s="19" t="n"/>
       <c r="E9" s="22" t="n">
         <v>111380</v>
       </c>
@@ -1496,11 +1467,7 @@
           <t>LULU FY2025 10-K: operating lease liabilities</t>
         </is>
       </c>
-      <c r="D11" s="19" t="inlineStr">
-        <is>
-          <t>Ctrl+F "Current lease liabilities" → 298,724 | "Non-current lease liabilities" → 1,499,717 | sum = 1,798,441 ($000)</t>
-        </is>
-      </c>
+      <c r="D11" s="19" t="n"/>
       <c r="E11" s="22" t="n">
         <v>1798441</v>
       </c>
@@ -1528,11 +1495,7 @@
           <t>LULU FY2025 10-K (no funded debt)</t>
         </is>
       </c>
-      <c r="D13" s="19" t="inlineStr">
-        <is>
-          <t>Ctrl+F "no borrowings were outstanding under this facility" → funded debt $0</t>
-        </is>
-      </c>
+      <c r="D13" s="19" t="n"/>
       <c r="E13" s="22" t="n">
         <v>0</v>
       </c>
@@ -1572,11 +1535,7 @@
           <t>Yahoo Finance: LULU Beta (5Y Monthly)</t>
         </is>
       </c>
-      <c r="D17" s="19" t="inlineStr">
-        <is>
-          <t>Ctrl+F "Beta (5Y Monthly)" → 0.86. Levered βL (Yahoo Key Statistics).</t>
-        </is>
-      </c>
+      <c r="D17" s="19" t="n"/>
       <c r="E17" s="27" t="n">
         <v>0.86</v>
       </c>
@@ -1597,11 +1556,7 @@
           <t>Yahoo Finance: LULU Total Debt (mrq)</t>
         </is>
       </c>
-      <c r="D18" s="19" t="inlineStr">
-        <is>
-          <t>Ctrl+F "Total Debt (mrq)" → 2.14B. Same page as beta.</t>
-        </is>
-      </c>
+      <c r="D18" s="19" t="n"/>
       <c r="E18" s="22" t="n">
         <v>2140000</v>
       </c>
@@ -1622,11 +1577,7 @@
           <t>Yahoo Finance: LULU Market Cap</t>
         </is>
       </c>
-      <c r="D19" s="19" t="inlineStr">
-        <is>
-          <t>Ctrl+F "Market Cap" → 11.14B. Same page as beta and debt.</t>
-        </is>
-      </c>
+      <c r="D19" s="19" t="n"/>
       <c r="E19" s="22" t="n">
         <v>11140000</v>
       </c>
@@ -1673,11 +1624,7 @@
           <t>Yahoo Finance: Total Debt/Equity (mrq)</t>
         </is>
       </c>
-      <c r="D21" s="19" t="inlineStr">
-        <is>
-          <t>Ctrl+F "Total Debt/Equity (mrq)" → 44.69%. Book D/E; reference only, not in Hamada.</t>
-        </is>
-      </c>
+      <c r="D21" s="19" t="n"/>
       <c r="E21" s="27" t="n">
         <v>0.4469</v>
       </c>
@@ -1750,11 +1697,7 @@
           <t>Damodaran: US betas by sector (Jan 2026)</t>
         </is>
       </c>
-      <c r="D24" s="19" t="inlineStr">
-        <is>
-          <t>Ctrl+F "Retail (Special Lines)" → 0.95 βu. Sector benchmark; not used in WACC.</t>
-        </is>
-      </c>
+      <c r="D24" s="19" t="n"/>
       <c r="E24" s="27" t="n">
         <v>0.95</v>
       </c>
@@ -1777,8 +1720,13 @@
       </c>
       <c r="D25" s="19" t="inlineStr">
         <is>
-          <t>YAHOO KEY STATISTICS; βL + debt + equity on ONE page
-(No vendor publishes the D/E embedded inside the regression.) Observed levered βL Ctrl+F "Beta (5Y Monthly)" → 0.86 ~60 monthly returns vs S&amp;P 500 (Yahoo label) Paired inputs on same page (mrq = most recent quarter) Ctrl+F "Total Debt (mrq)" → 2.14B Ctrl+F "Market Cap" → 11.14B Ctrl+F "Total Debt/Equity (mrq)" → 44.69% (book; reference only) STEP 1 — UNLEVER (market D/E from Yahoo page) D/E = Total Debt (mrq) ÷ Market Cap = 2.14 ÷ 11.14 ≈ 0.19 βu = 0.86 ÷ [1 + 0.70 × 0.19] = 0.86 ÷ 1.134 ≈ 0.76 (1−T) = 0.70 at 30% tax on this tab STEP 2 — RELEVER (WACC: FY25 10-K lease debt / our market cap) Ctrl+F "Current lease liabilities" → 298,724 Ctrl+F "Non-current lease liabilities" → 1,499,717 D/E ≈ 0.16. β used = 0.76 × 1.113 ≈ 0.84 Benchmark (not used): Damodaran Retail βu 0.95</t>
+          <t>Hamada β: Yahoo βL 0.86; unlever at mkt D/E ~0.19 → βu ~0.76; relever at lease-adjusted D/E ~0.16 → β used ~0.84.
+Observed levered βL
+~60 monthly returns vs S&amp;P 500 (Yahoo label)
+Paired inputs on same page (mrq = most recent quarter)
+(1−T) = 0.70 at 30% tax on this tab
+D/E ≈ 0.16. β used = 0.76 × 1.113 ≈ 0.84
+Benchmark (not used): Damodaran Retail βu 0.95</t>
         </is>
       </c>
       <c r="E25" s="29">
@@ -1863,11 +1811,7 @@
           <t>LULU FY2025 10-K: lease liabilities &amp; no funded debt</t>
         </is>
       </c>
-      <c r="D35" s="19" t="inlineStr">
-        <is>
-          <t>Ctrl+F "Current lease liabilities" + "Non-current lease liabilities" → debt equiv. 5.0% illustrative lease borrowing cost.</t>
-        </is>
-      </c>
+      <c r="D35" s="19" t="n"/>
       <c r="E35" s="20" t="n">
         <v>0.05</v>
       </c>
@@ -2041,11 +1985,7 @@
           <t>Source (click)</t>
         </is>
       </c>
-      <c r="D3" s="15" t="inlineStr">
-        <is>
-          <t>Ctrl+F (prove number)</t>
-        </is>
-      </c>
+      <c r="D3" s="15" t="n"/>
     </row>
     <row r="4" ht="28" customHeight="1">
       <c r="A4" s="16" t="inlineStr">
@@ -2063,11 +2003,7 @@
           <t>LULU Q2 FY2026 earnings release</t>
         </is>
       </c>
-      <c r="D4" s="19" t="inlineStr">
-        <is>
-          <t>Ctrl+F "decline of 5% to 7%" → FY2026 revenue guide; model −6.1% midpoint</t>
-        </is>
-      </c>
+      <c r="D4" s="19" t="n"/>
       <c r="F4" s="20" t="n">
         <v>-0.09</v>
       </c>
@@ -2094,11 +2030,7 @@
           <t>StockAnalysis: LULU 3Y revenue forecast</t>
         </is>
       </c>
-      <c r="D5" s="19" t="inlineStr">
-        <is>
-          <t>Ctrl+F "Revenue Growth Forecast (3Y)" → 2.26%. That is the unique line (do not search "Net revenue"). Model FY27–30 uses 2.3%.</t>
-        </is>
-      </c>
+      <c r="D5" s="19" t="n"/>
       <c r="F5" s="20" t="n">
         <v>-0.01</v>
       </c>
@@ -2125,11 +2057,7 @@
           <t>Q2 FY2026 release: 18.8% OM minus 560bps tariffs</t>
         </is>
       </c>
-      <c r="D6" s="19" t="inlineStr">
-        <is>
-          <t>Ctrl+F "18.8%" (Q2 OM) and "560 basis points" (tariff boost). Real run-rate = 18.8% − 5.6% = 13.2%. Do not use "decreased 13%".</t>
-        </is>
-      </c>
+      <c r="D6" s="19" t="n"/>
       <c r="F6" s="20" t="n">
         <v>0.12</v>
       </c>
@@ -2156,11 +2084,7 @@
           <t>Q2 FY2026 release: $134.5M IEEPA tariff refunds</t>
         </is>
       </c>
-      <c r="D7" s="19" t="inlineStr">
-        <is>
-          <t>Ctrl+F "134.5 million" → IEEPA tariff refunds reduced COGS. Add this dollar amount to FY26 EBIT only. Full-year boost = 134.5 / FY26 sales ≈ 1.3ppt, not 5.6ppt.</t>
-        </is>
-      </c>
+      <c r="D7" s="19" t="n"/>
       <c r="F7" s="37" t="n">
         <v>134500</v>
       </c>
@@ -2179,7 +2103,7 @@
       </c>
       <c r="B8" s="17" t="inlineStr">
         <is>
-          <t>FY30 15.5% is a partial recovery vs the FY25 10-K OM of 19.9% (unique Ctrl+F). Still well below the FY24 23.7% peak.</t>
+          <t>FY30 15.5% is a partial recovery vs the FY25 10-K OM of 19.9% (per FY25 10-K). Still well below the FY24 23.7% peak.</t>
         </is>
       </c>
       <c r="C8" s="18" t="inlineStr">
@@ -2187,11 +2111,7 @@
           <t>FY2025 10-K: Operating margin 19.9% (one hit)</t>
         </is>
       </c>
-      <c r="D8" s="19" t="inlineStr">
-        <is>
-          <t>Ctrl+F "19.9%" (one hit) → Operating margin decreased 380 basis points to 19.9%. That is FY25 OM. Do not search the words Income from operations (17 hits). Model FY30 15.5% is a partial-recovery assumption.</t>
-        </is>
-      </c>
+      <c r="D8" s="19" t="n"/>
       <c r="F8" s="20" t="n">
         <v>0.12</v>
       </c>
@@ -2250,11 +2170,7 @@
           <t>FRED: Real GDP (GDPC1)</t>
         </is>
       </c>
-      <c r="D10" s="19" t="inlineStr">
-        <is>
-          <t>Ctrl+F "Q2 2026" → 24,269.613 and "Q2 2025" → 23,770.976. YoY = 2.1%. Model terminal g 2.25%.</t>
-        </is>
-      </c>
+      <c r="D10" s="19" t="n"/>
       <c r="F10" s="20" t="n">
         <v>0.015</v>
       </c>
@@ -2281,11 +2197,7 @@
           <t>Q2 FY2026 outlook: tax rate ≈ 30%</t>
         </is>
       </c>
-      <c r="D11" s="19" t="inlineStr">
-        <is>
-          <t>Ctrl+F "a tax rate of approximately 30%" on the earnings outlook. FY25 10-K: "Income tax expense" 659,784 ÷ "Income before income tax expense" 2,238,967 = 29.5%.</t>
-        </is>
-      </c>
+      <c r="D11" s="19" t="n"/>
       <c r="F11" s="20" t="n">
         <v>0.32</v>
       </c>
@@ -2312,11 +2224,7 @@
           <t>LULU CF statement (10-K)</t>
         </is>
       </c>
-      <c r="D12" s="19" t="inlineStr">
-        <is>
-          <t>Ctrl+F "Depreciation and amortization" → 496,228 on this 10-K HTML (not the SEC viewer). ÷ "Net revenue" 11,102,600 = 4.5%.</t>
-        </is>
-      </c>
+      <c r="D12" s="19" t="n"/>
       <c r="F12" s="20" t="n">
         <v>0.045</v>
       </c>
@@ -2336,18 +2244,25 @@
       <c r="B13" s="19" t="inlineStr">
         <is>
           <t>FY26 7.0% is $735M on $10.4B sales, not FY25 $11.1B. Since 7.0% steps toward FY25 6.1%, we assume a fade: DCF 5.5% = (7.0+6.0+5.5+5.0+4.0)/5.
-Also: FY26 sales are $10.35–$10.50B (earnings). Use that $10.4B year as the 7% denominator, not FY25 $11.1B.</t>
+FY26 sales are $10.35–$10.50B (earnings). Use that $10.4B year as the 7% denominator, not FY25 $11.1B.</t>
         </is>
       </c>
       <c r="C13" s="38" t="inlineStr">
         <is>
           <t>LULU 10-K: 2026 capex guide $725–745M
-Also: Q2 FY2026 outlook: $10.350B–$10.500B sales</t>
+Q2 FY2026 outlook: $10.350B–$10.500B sales</t>
         </is>
       </c>
       <c r="D13" s="19" t="inlineStr">
         <is>
-          <t>FY25 actual (10-K) Ctrl+F "680,802" → capex $680.8M Ctrl+F "11,102,600" → sales $11.1B 680.8 / 11,102.6 = 6.1% FY26 capex (10-K) Ctrl+F "$725.0 million and $745.0 million" → mid $735M FY26 sales (earnings) Ctrl+F "$10.350 billion to $10.500 billion" → $10.35–$10.50B (mid $10.425B) 7.0% = $735M / $10.425B ($10B year, not FY25 $11.1B) DCF blend Fade 7.0 / 6.0 / 5.5 / 5.0 / 4.0 5.5% = (7.0+6.0+5.5+5.0+4.0)/5</t>
+          <t>FY25 actual (10-K)
+680.8 / 11,102.6 = 6.1%
+FY26 capex (10-K)
+FY26 sales (earnings)
+7.0% = $735M / $10.425B ($10B year, not FY25 $11.1B)
+DCF blend
+Fade 7.0 / 6.0 / 5.5 / 5.0 / 4.0
+5.5% = (7.0+6.0+5.5+5.0+4.0)/5</t>
         </is>
       </c>
       <c r="F13" s="20" t="n">
@@ -2379,11 +2294,8 @@
       <c r="D14" s="19" t="inlineStr">
         <is>
           <t>56.6% of revenue (gross margin).
-Ctrl+F "Gross profit"
 → 6,284,132 ($000)
-Ctrl+F "Net revenue"
 → 11,102,600 ($000)
-Ctrl+F "Cost of goods sold"
 → 4,818,468 ($000)</t>
         </is>
       </c>
@@ -2405,7 +2317,7 @@
       </c>
       <c r="B15" s="17" t="inlineStr">
         <is>
-          <t>Not % of revenue; DSO (days), flat ~6.3. Mostly own stores/DTC (cash at register); AR is small wholesale residual; predictable ~6 days FY22–25.</t>
+          <t>DSO flat ~6.3 days — DTC/store cash sales dominate; AR is wholesale residual.</t>
         </is>
       </c>
       <c r="C15" s="18" t="inlineStr">
@@ -2415,16 +2327,7 @@
       </c>
       <c r="D15" s="19" t="inlineStr">
         <is>
-          <t>Not % of revenue; DSO (days), flat ~6.3.
-Why flat: ~90%+ revenue is company-operated stores + e-commerce (cash/card at sale);
-AR is a small, stable wholesale/license residual; predictable collection, not trade credit.
-Ctrl+F "Accounts receivable, net"
-→ 190,657 ($000)
-Ctrl+F "Net revenue"
-→ 11,102,600 ($000)
-DSO = (190,657 ÷ 11,102,600) × 365 ≈ 6.3 days (~6.0–6.3 FY22–25).
-Ctrl+F "company-operated stores"
-Ctrl+F "E-commerce"</t>
+          <t>DSO flat ~6.3 days — DTC/store cash sales dominate; AR is wholesale residual.</t>
         </is>
       </c>
       <c r="F15" s="39" t="n">
@@ -2445,9 +2348,7 @@
       </c>
       <c r="B16" s="17" t="inlineStr">
         <is>
-          <t>Not % of revenue; DIO (days).
-FY25 anchor: DIO = (Inventories ÷ COGS) × 365 = (1,700,753 ÷ 4,818,468) × 365 ≈ 129 days (FY24 inv: 1,442,081).
-Forecast path: DIO_t = FY25 DIO − (1 day × year t); flat across scenarios.</t>
+          <t>DIO: FY25 anchor ~129 days; −1 day/yr through FY30 (inventory discipline).</t>
         </is>
       </c>
       <c r="C16" s="18" t="inlineStr">
@@ -2457,13 +2358,7 @@
       </c>
       <c r="D16" s="19" t="inlineStr">
         <is>
-          <t>Not % of revenue; DIO (days).
-FY25 anchor formula: DIO = (Inventories ÷ COGS) × 365
-Ctrl+F "Inventories"
-→ 1,700,753 ($000) | FY24: 1,442,081
-Ctrl+F "Cost of goods sold"
-→ 4,818,468 ($000) = (1,700,753 ÷ 4,818,468) × 365 ≈ 129 days
-Forecast: DIO_t = FY25 DIO − (1 × year t)</t>
+          <t>DIO: FY25 anchor ~129 days; −1 day/yr through FY30 (inventory discipline).</t>
         </is>
       </c>
       <c r="F16" s="39" t="n">
@@ -2484,10 +2379,7 @@
       </c>
       <c r="B17" s="17" t="inlineStr">
         <is>
-          <t>Not % of revenue; subtract 1 DIO day per forecast year (−5 days FY26–30).
-Feeds Inventories = (DIO_t ÷ 365) × COGS_t.
-Ctrl+F "reduce the percentage of markdowns"
-Ctrl+F "On a unit basis, we expect inventories to slightly decrease"</t>
+          <t>DIO: FY25 anchor ~129 days; −1 day/yr through FY30 (inventory discipline).</t>
         </is>
       </c>
       <c r="C17" s="18" t="inlineStr">
@@ -2497,10 +2389,7 @@
       </c>
       <c r="D17" s="19" t="inlineStr">
         <is>
-          <t>Not % of revenue; DIO −1 day/yr (−5 days FY26–30).
-Feeds Inventories_t = (DIO_t ÷ 365) × COGS_t.
-Ctrl+F "reduce the percentage of markdowns"
-Ctrl+F "On a unit basis, we expect inventories to slightly decrease"</t>
+          <t>DIO: FY25 anchor ~129 days; −1 day/yr through FY30 (inventory discipline).</t>
         </is>
       </c>
       <c r="F17" s="40" t="n">
@@ -2521,7 +2410,7 @@
       </c>
       <c r="B18" s="17" t="inlineStr">
         <is>
-          <t>Not % of revenue; DPO (days), flat ~25.1. Implied AP ≈3.0% of sales / 6.9% of COGS.</t>
+          <t>DPO flat ~25 days; AP scales with COGS (~3% of sales).</t>
         </is>
       </c>
       <c r="C18" s="18" t="inlineStr">
@@ -2531,9 +2420,7 @@
       </c>
       <c r="D18" s="19" t="inlineStr">
         <is>
-          <t>Ctrl+F "Accounts payable"
-→ 331,421 ($000)
-Ctrl+F "Cost of goods sold"
+          <t>→ 331,421 ($000)
 → 4,818,468 ($000)
 Not % of revenue; DPO ≈ 25.1 days. Implied AP ≈ 3.0% of sales / 6.9% of COGS.</t>
         </is>
@@ -2566,9 +2453,7 @@
       </c>
       <c r="D19" s="19" t="inlineStr">
         <is>
-          <t>Ctrl+F "Prepaid expenses and other current assets"
-→ 211,620 ($000)
-Ctrl+F "Prepaid and receivable income taxes"
+          <t>→ 211,620 ($000)
 → 352,469 ($000)
 5.1% of revenue (flat). OCA residual = 564,089 ÷ 11,102,600.</t>
         </is>
@@ -2601,9 +2486,7 @@
       </c>
       <c r="D20" s="19" t="inlineStr">
         <is>
-          <t>Ctrl+F "Accrued liabilities and other"
-→ 662,982 ($000)
-Ctrl+F "Net revenue"
+          <t>→ 662,982 ($000)
 → 11,102,600 ($000)
 6.0% of revenue (flat). 662,982 ÷ 11,102,600.</t>
         </is>
@@ -5760,7 +5643,7 @@
     <row r="193">
       <c r="A193" s="26" t="inlineStr">
         <is>
-          <t>memo: pitch deck pulls cols G (base) &amp; H (bull) from this block via pitch_values.py</t>
+          <t>memo: pitch deck Pitch deck reads base/bull scenario columns.</t>
         </is>
       </c>
     </row>
@@ -5832,7 +5715,7 @@
     <row r="2">
       <c r="A2" s="26" t="inlineStr">
         <is>
-          <t>FY2025A = -ingested 10-K anchors (blue). FY26–30 = red operational assumptions. Consolidated revenue cross-checks to Scenarios base case.</t>
+          <t>FY2025A = FY25 10-K historical anchors (blue). FY26–30 = red operational assumptions. Consolidated revenue cross-checks to Scenarios base case.</t>
         </is>
       </c>
     </row>
@@ -5852,11 +5735,7 @@
           <t>Source (click)</t>
         </is>
       </c>
-      <c r="L3" s="51" t="inlineStr">
-        <is>
-          <t>Ctrl+F (prove number)</t>
-        </is>
-      </c>
+      <c r="L3" s="51" t="n"/>
     </row>
     <row r="4">
       <c r="A4" s="52" t="inlineStr">
@@ -5921,11 +5800,7 @@
           <t>Source</t>
         </is>
       </c>
-      <c r="L5" s="56" t="inlineStr">
-        <is>
-          <t>Ctrl+F</t>
-        </is>
-      </c>
+      <c r="L5" s="56" t="n"/>
     </row>
     <row r="6" ht="28" customHeight="1">
       <c r="A6" s="41" t="inlineStr">
@@ -5963,12 +5838,12 @@
       </c>
       <c r="I6" s="59" t="inlineStr">
         <is>
-          <t>prior-year ending stores. Same count, new column; that's where the year starts.</t>
+          <t>prior-year ending stores. Same count, new column;</t>
         </is>
       </c>
       <c r="J6" s="17" t="inlineStr">
         <is>
-          <t>Beginning stores = last year's ending count. Same number, just carried forward into the new fiscal year.</t>
+          <t>Beginning stores = last year's ending count. Prior-year ending count carried forward.</t>
         </is>
       </c>
       <c r="K6" s="24" t="inlineStr">
@@ -6013,11 +5888,7 @@
           <t>FY2025 10-K: store count &amp; expansion</t>
         </is>
       </c>
-      <c r="L7" s="19" t="inlineStr">
-        <is>
-          <t>Ctrl+F "Total company-operated stores" → 811 (FY25). FY25 added 44 net stores; model skews openings to China.</t>
-        </is>
-      </c>
+      <c r="L7" s="19" t="n"/>
     </row>
     <row r="8" ht="28" customHeight="1">
       <c r="A8" s="41" t="inlineStr">
@@ -6055,11 +5926,7 @@
           <t>FY2025 10-K: lease renewal / fleet</t>
         </is>
       </c>
-      <c r="L8" s="19" t="inlineStr">
-        <is>
-          <t>Ctrl+F "lease" / store fleet; immaterial closures vs expansion; 2–3 per mature region.</t>
-        </is>
-      </c>
+      <c r="L8" s="19" t="n"/>
     </row>
     <row r="9" ht="28" customHeight="1">
       <c r="A9" s="61" t="inlineStr">
@@ -6097,7 +5964,7 @@
       </c>
       <c r="I9" s="59" t="inlineStr">
         <is>
-          <t>beginning stores + openings − closures. Roll-forward; nothing fancy, just how many doors you end with.</t>
+          <t>beginning stores + openings − closures. Roll-forward;</t>
         </is>
       </c>
       <c r="J9" s="17" t="inlineStr">
@@ -6147,12 +6014,12 @@
       </c>
       <c r="I10" s="59" t="inlineStr">
         <is>
-          <t>prior-year ending stores. Same count, new column; that's where the year starts.</t>
+          <t>prior-year ending stores. Same count, new column;</t>
         </is>
       </c>
       <c r="J10" s="17" t="inlineStr">
         <is>
-          <t>Beginning stores = last year's ending count. Same number, just carried forward into the new fiscal year.</t>
+          <t>Beginning stores = last year's ending count. Prior-year ending count carried forward.</t>
         </is>
       </c>
       <c r="K10" s="24" t="inlineStr">
@@ -6197,11 +6064,7 @@
           <t>FY2025 10-K: store count &amp; expansion</t>
         </is>
       </c>
-      <c r="L11" s="19" t="inlineStr">
-        <is>
-          <t>Ctrl+F "Total company-operated stores" → 811 (FY25). FY25 added 44 net stores; model skews openings to China.</t>
-        </is>
-      </c>
+      <c r="L11" s="19" t="n"/>
     </row>
     <row r="12" ht="28" customHeight="1">
       <c r="A12" s="41" t="inlineStr">
@@ -6239,11 +6102,7 @@
           <t>FY2025 10-K: lease renewal / fleet</t>
         </is>
       </c>
-      <c r="L12" s="19" t="inlineStr">
-        <is>
-          <t>Ctrl+F "lease" / store fleet; immaterial closures vs expansion; 2–3 per mature region.</t>
-        </is>
-      </c>
+      <c r="L12" s="19" t="n"/>
     </row>
     <row r="13" ht="28" customHeight="1">
       <c r="A13" s="61" t="inlineStr">
@@ -6281,7 +6140,7 @@
       </c>
       <c r="I13" s="59" t="inlineStr">
         <is>
-          <t>beginning stores + openings − closures. Roll-forward; nothing fancy, just how many doors you end with.</t>
+          <t>beginning stores + openings − closures. Roll-forward;</t>
         </is>
       </c>
       <c r="J13" s="17" t="inlineStr">
@@ -6331,12 +6190,12 @@
       </c>
       <c r="I14" s="59" t="inlineStr">
         <is>
-          <t>prior-year ending stores. Same count, new column; that's where the year starts.</t>
+          <t>prior-year ending stores. Same count, new column;</t>
         </is>
       </c>
       <c r="J14" s="17" t="inlineStr">
         <is>
-          <t>Beginning stores = last year's ending count. Same number, just carried forward into the new fiscal year.</t>
+          <t>Beginning stores = last year's ending count. Prior-year ending count carried forward.</t>
         </is>
       </c>
       <c r="K14" s="24" t="inlineStr">
@@ -6381,11 +6240,7 @@
           <t>FY2025 10-K: store count &amp; expansion</t>
         </is>
       </c>
-      <c r="L15" s="19" t="inlineStr">
-        <is>
-          <t>Ctrl+F "Total company-operated stores" → 811 (FY25). FY25 added 44 net stores; model skews openings to China.</t>
-        </is>
-      </c>
+      <c r="L15" s="19" t="n"/>
     </row>
     <row r="16" ht="28" customHeight="1">
       <c r="A16" s="41" t="inlineStr">
@@ -6423,11 +6278,7 @@
           <t>FY2025 10-K: lease renewal / fleet</t>
         </is>
       </c>
-      <c r="L16" s="19" t="inlineStr">
-        <is>
-          <t>Ctrl+F "lease" / store fleet; immaterial closures vs expansion; 2–3 per mature region.</t>
-        </is>
-      </c>
+      <c r="L16" s="19" t="n"/>
     </row>
     <row r="17" ht="28" customHeight="1">
       <c r="A17" s="61" t="inlineStr">
@@ -6465,7 +6316,7 @@
       </c>
       <c r="I17" s="59" t="inlineStr">
         <is>
-          <t>beginning stores + openings − closures. Roll-forward; nothing fancy, just how many doors you end with.</t>
+          <t>beginning stores + openings − closures. Roll-forward;</t>
         </is>
       </c>
       <c r="J17" s="17" t="inlineStr">
@@ -6563,11 +6414,7 @@
           <t>FY2025 10-K: sales per square foot</t>
         </is>
       </c>
-      <c r="L19" s="19" t="inlineStr">
-        <is>
-          <t>Ctrl+F "sales per square foot were $1,426" → implied 3.54M sq ft / 811 stores ≈ 4,367 sq ft.</t>
-        </is>
-      </c>
+      <c r="L19" s="19" t="n"/>
     </row>
     <row r="20" ht="28" customHeight="1">
       <c r="A20" s="41" t="inlineStr">
@@ -6684,11 +6531,7 @@
           <t>Source</t>
         </is>
       </c>
-      <c r="L23" s="56" t="inlineStr">
-        <is>
-          <t>Ctrl+F</t>
-        </is>
-      </c>
+      <c r="L23" s="56" t="n"/>
     </row>
     <row r="24" ht="28" customHeight="1">
       <c r="A24" s="41" t="inlineStr">
@@ -6729,11 +6572,7 @@
           <t>FY2025 10-K: comparable sales &amp; SPSF</t>
         </is>
       </c>
-      <c r="L24" s="19" t="inlineStr">
-        <is>
-          <t>Ctrl+F "sales per square foot were $1,426" → FY25 reported $1,426; FY26 model $1,380 on traffic pressure.</t>
-        </is>
-      </c>
+      <c r="L24" s="19" t="n"/>
     </row>
     <row r="25" ht="28" customHeight="1">
       <c r="A25" s="41" t="inlineStr">
@@ -6774,11 +6613,7 @@
           <t>FY2025 10-K: Americas comparable sales</t>
         </is>
       </c>
-      <c r="L25" s="19" t="inlineStr">
-        <is>
-          <t>Ctrl+F "Americas comparable sales decreased 3%" → FY25 anchor. FY26 model −4% before stabilization.</t>
-        </is>
-      </c>
+      <c r="L25" s="19" t="n"/>
     </row>
     <row r="26" ht="28" customHeight="1">
       <c r="A26" s="41" t="inlineStr">
@@ -6819,11 +6654,7 @@
           <t>FY2025 10-K: China Mainland comparable sales</t>
         </is>
       </c>
-      <c r="L26" s="19" t="inlineStr">
-        <is>
-          <t>Ctrl+F "China Mainland comparable sales increased 20%" → FY25 anchor. FY26 model +14% on a larger base.</t>
-        </is>
-      </c>
+      <c r="L26" s="19" t="n"/>
     </row>
     <row r="27" ht="28" customHeight="1">
       <c r="A27" s="41" t="inlineStr">
@@ -6864,11 +6695,7 @@
           <t>FY2025 10-K: Rest of World comparable sales</t>
         </is>
       </c>
-      <c r="L27" s="19" t="inlineStr">
-        <is>
-          <t>Ctrl+F "Rest of World comparable sales increased 9%" → FY25 +9% (+7% CCY). FY26 model +7%, fading to +4%.</t>
-        </is>
-      </c>
+      <c r="L27" s="19" t="n"/>
     </row>
     <row r="28" ht="28" customHeight="1">
       <c r="A28" s="41" t="inlineStr">
@@ -6994,11 +6821,7 @@
         <f>(G7-G8+G11-G12+G15-G16)*G19*G24/1000*0.55</f>
         <v/>
       </c>
-      <c r="I30" s="59" t="inlineStr">
-        <is>
-          <t>(open−close each geo)×sq ft×$/sq ft → raw annual $. /1000 flips that to $000 (this whole tab is thousands). ×0.55 = year-one haircut; new boxes don't run at full SPSF yet. FY27 ex: (D7−D8+D11−D12+D15−D16)×D19×D24/1000×0.55.</t>
-        </is>
-      </c>
+      <c r="I30" s="59" t="n"/>
       <c r="J30" s="17" t="inlineStr">
         <is>
           <t>Net new doors × sq ft × $/sq ft is plain dollars. /1000 → $000 on this tab. ×0.55 'cause year-one stores don't run full.</t>
@@ -7094,11 +6917,7 @@
           <t>FY2025 10-K: store traffic commentary</t>
         </is>
       </c>
-      <c r="L32" s="19" t="inlineStr">
-        <is>
-          <t>Ctrl+F "store traffic" → lower traffic in Americas; memo line only.</t>
-        </is>
-      </c>
+      <c r="L32" s="19" t="n"/>
     </row>
     <row r="33" ht="28" customHeight="1">
       <c r="A33" s="41" t="inlineStr">
@@ -7134,11 +6953,7 @@
           <t>FY2025 10-K: conversion rate commentary</t>
         </is>
       </c>
-      <c r="L33" s="19" t="inlineStr">
-        <is>
-          <t>Ctrl+F "conversion rates" → lower in Americas; in-store memo 27%→29%.</t>
-        </is>
-      </c>
+      <c r="L33" s="19" t="n"/>
     </row>
     <row r="34" ht="28" customHeight="1">
       <c r="A34" s="41" t="inlineStr">
@@ -7174,11 +6989,7 @@
           <t>FY2025 10-K: average order value commentary</t>
         </is>
       </c>
-      <c r="L34" s="19" t="inlineStr">
-        <is>
-          <t>Ctrl+F "average order value" → lower AOV in Americas; memo $115–$122.</t>
-        </is>
-      </c>
+      <c r="L34" s="19" t="n"/>
     </row>
     <row r="35"/>
     <row r="36">
@@ -7244,11 +7055,7 @@
           <t>Source</t>
         </is>
       </c>
-      <c r="L37" s="56" t="inlineStr">
-        <is>
-          <t>Ctrl+F</t>
-        </is>
-      </c>
+      <c r="L37" s="56" t="n"/>
     </row>
     <row r="38" ht="28" customHeight="1">
       <c r="A38" s="41" t="inlineStr">
@@ -7289,11 +7096,7 @@
           <t>FY2025 10-K: e-commerce revenue</t>
         </is>
       </c>
-      <c r="L38" s="19" t="inlineStr">
-        <is>
-          <t>Ctrl+F "E-commerce" → 4,918,697 ($000). Sessions implied from revenue / conv / AOV.</t>
-        </is>
-      </c>
+      <c r="L38" s="19" t="n"/>
     </row>
     <row r="39" ht="28" customHeight="1">
       <c r="A39" s="41" t="inlineStr">
@@ -7329,11 +7132,7 @@
           <t>FY2025 10-K: digital / traffic commentary</t>
         </is>
       </c>
-      <c r="L39" s="19" t="inlineStr">
-        <is>
-          <t>Ctrl+F "lower conversion rates" (Americas MD&amp;A). FY26 model 3.3% digital conversion.</t>
-        </is>
-      </c>
+      <c r="L39" s="19" t="n"/>
     </row>
     <row r="40" ht="28" customHeight="1">
       <c r="A40" s="41" t="inlineStr">
@@ -7369,11 +7168,7 @@
           <t>FY2025 10-K: e-commerce revenue</t>
         </is>
       </c>
-      <c r="L40" s="19" t="inlineStr">
-        <is>
-          <t>Ctrl+F "average order value" (Americas MD&amp;A). FY26 model $305 AOV.</t>
-        </is>
-      </c>
+      <c r="L40" s="19" t="n"/>
     </row>
     <row r="41" ht="28" customHeight="1">
       <c r="A41" s="61" t="inlineStr">
@@ -7484,11 +7279,7 @@
           <t>Source</t>
         </is>
       </c>
-      <c r="L44" s="56" t="inlineStr">
-        <is>
-          <t>Ctrl+F</t>
-        </is>
-      </c>
+      <c r="L44" s="56" t="n"/>
     </row>
     <row r="45" ht="28" customHeight="1">
       <c r="A45" s="41" t="inlineStr">
@@ -7539,11 +7330,7 @@
           <t>FY2025 10-K: channel revenue table</t>
         </is>
       </c>
-      <c r="L45" s="19" t="inlineStr">
-        <is>
-          <t>Ctrl+F "Company-operated stores" and "E-commerce" → residual other channels ≈ $1.13B.</t>
-        </is>
-      </c>
+      <c r="L45" s="19" t="n"/>
     </row>
     <row r="46" ht="70" customHeight="1">
       <c r="A46" s="41" t="inlineStr">
@@ -7582,7 +7369,8 @@
       <c r="I46" s="59" t="inlineStr">
         <is>
           <t>FY26 geo rev = FY25 geo rev × (FY26 total rev ÷ FY25 total rev).
-Total rev = store channel + e-comm + other. Keeps FY25 geo mix; scales with consolidated growth. FY26E plugged: B46 × (C31+C41+C45) ÷ (B31+B41+B45)</t>
+Total rev = store channel + e-comm + other. Keeps FY25 geo mix; scales with consolidated growth.
+FY26E plugged: B46 × (C31+C41+C45) ÷ (B31+B41+B45)</t>
         </is>
       </c>
       <c r="J46" s="17" t="inlineStr">
@@ -7595,11 +7383,7 @@
           <t>FY2025 10-K: segmented net revenue</t>
         </is>
       </c>
-      <c r="L46" s="19" t="inlineStr">
-        <is>
-          <t>Ctrl+F "Americas" segment table → $7,847,044 net revenue (70.7%).</t>
-        </is>
-      </c>
+      <c r="L46" s="19" t="n"/>
     </row>
     <row r="47" ht="70" customHeight="1">
       <c r="A47" s="41" t="inlineStr">
@@ -7638,7 +7422,8 @@
       <c r="I47" s="59" t="inlineStr">
         <is>
           <t>FY26 geo rev = FY25 geo rev × (FY26 total rev ÷ FY25 total rev).
-Total rev = store channel + e-comm + other. Keeps FY25 geo mix; scales with consolidated growth. FY26E plugged: B47 × (C31+C41+C45) ÷ (B31+B41+B45)</t>
+Total rev = store channel + e-comm + other. Keeps FY25 geo mix; scales with consolidated growth.
+FY26E plugged: B47 × (C31+C41+C45) ÷ (B31+B41+B45)</t>
         </is>
       </c>
       <c r="J47" s="17" t="inlineStr">
@@ -7651,11 +7436,7 @@
           <t>FY2025 10-K: segmented net revenue</t>
         </is>
       </c>
-      <c r="L47" s="19" t="inlineStr">
-        <is>
-          <t>Ctrl+F "China Mainland" segment → $1,754,799 net revenue (15.8%).</t>
-        </is>
-      </c>
+      <c r="L47" s="19" t="n"/>
     </row>
     <row r="48" ht="70" customHeight="1">
       <c r="A48" s="41" t="inlineStr">
@@ -7694,7 +7475,8 @@
       <c r="I48" s="59" t="inlineStr">
         <is>
           <t>FY26 geo rev = FY25 geo rev × (FY26 total rev ÷ FY25 total rev).
-Total rev = store channel + e-comm + other. Keeps FY25 geo mix; scales with consolidated growth. FY26E plugged: B48 × (C31+C41+C45) ÷ (B31+B41+B45)</t>
+Total rev = store channel + e-comm + other. Keeps FY25 geo mix; scales with consolidated growth.
+FY26E plugged: B48 × (C31+C41+C45) ÷ (B31+B41+B45)</t>
         </is>
       </c>
       <c r="J48" s="17" t="inlineStr">
@@ -7707,11 +7489,7 @@
           <t>FY2025 10-K: segmented net revenue</t>
         </is>
       </c>
-      <c r="L48" s="19" t="inlineStr">
-        <is>
-          <t>Ctrl+F "Rest of World" segment → $1,500,757 net revenue (13.5%).</t>
-        </is>
-      </c>
+      <c r="L48" s="19" t="n"/>
     </row>
     <row r="49" ht="28" customHeight="1">
       <c r="A49" s="41" t="inlineStr">
@@ -7747,11 +7525,7 @@
           <t>FY2025 10-K: product category mix</t>
         </is>
       </c>
-      <c r="L49" s="19" t="inlineStr">
-        <is>
-          <t>Ctrl+F "women's, men's, and accessories" → 63% / 24% / 13% of net revenue.</t>
-        </is>
-      </c>
+      <c r="L49" s="19" t="n"/>
     </row>
     <row r="50" ht="28" customHeight="1">
       <c r="A50" s="41" t="inlineStr">
@@ -7787,11 +7561,7 @@
           <t>FY2025 10-K: product category mix</t>
         </is>
       </c>
-      <c r="L50" s="19" t="inlineStr">
-        <is>
-          <t>Ctrl+F "men's" category growth 4% in MD&amp;A; mix rises to 27% by FY30.</t>
-        </is>
-      </c>
+      <c r="L50" s="19" t="n"/>
     </row>
     <row r="51" ht="28" customHeight="1">
       <c r="A51" s="41" t="inlineStr">
@@ -7827,11 +7597,7 @@
           <t>FY2025 10-K: product category mix</t>
         </is>
       </c>
-      <c r="L51" s="19" t="inlineStr">
-        <is>
-          <t>Ctrl+F "accessories" +8% category growth; hold 13% mix.</t>
-        </is>
-      </c>
+      <c r="L51" s="19" t="n"/>
     </row>
     <row r="52"/>
     <row r="53">
@@ -7897,11 +7663,7 @@
           <t>Source</t>
         </is>
       </c>
-      <c r="L54" s="56" t="inlineStr">
-        <is>
-          <t>Ctrl+F</t>
-        </is>
-      </c>
+      <c r="L54" s="56" t="n"/>
     </row>
     <row r="55" ht="28" customHeight="1">
       <c r="A55" s="68" t="inlineStr">
@@ -8182,11 +7944,7 @@
           <t>Source (click)</t>
         </is>
       </c>
-      <c r="D2" s="51" t="inlineStr">
-        <is>
-          <t>Ctrl+F (prove number)</t>
-        </is>
-      </c>
+      <c r="D2" s="51" t="n"/>
       <c r="E2" s="71" t="inlineStr">
         <is>
           <t>FY2025A</t>
@@ -8228,7 +7986,7 @@
     <row r="4">
       <c r="A4" s="26" t="inlineStr">
         <is>
-          <t>Phases 1–4 clean and forecast operating profit; Phase 5 is the workflow summary below.</t>
+          <t>Phases 1–4 clean and forecast operating profit; Phase 5 summarizes the reconciliation workflow..</t>
         </is>
       </c>
     </row>
@@ -8248,9 +8006,7 @@
       </c>
       <c r="B7" s="17" t="inlineStr">
         <is>
-          <t>Not % of revenue; SBC add-back flag. Set to 0 (Convention A).
-SBC stays inside Scenarios EBIT/NOPAT as a real economic cost; DCF uses basic shares (111.4M).
-FY25 reference: $62,203k (10-K). Flag = 1 would add back (Convention B + diluted shares); not used.</t>
+          <t>SBC stays in EBIT (Convention A); DCF uses basic shares.</t>
         </is>
       </c>
       <c r="C7" s="18" t="inlineStr">
@@ -8260,8 +8016,7 @@
       </c>
       <c r="D7" s="19" t="inlineStr">
         <is>
-          <t>Ctrl+F "Stock-based compensation expense"
-→ 62,203 ($000) FY25 reference. Flag = 0: SBC stays in EBIT (Convention A); DCF IV uses basic 111,380k shares.</t>
+          <t>→ 62,203 ($000) FY25 reference. Flag = 0: SBC stays in EBIT (Convention A); DCF IV uses basic 111,380k shares.</t>
         </is>
       </c>
       <c r="E7" s="40" t="n">
@@ -8313,7 +8068,6 @@
       <c r="D9" s="19" t="inlineStr">
         <is>
           <t>Not consolidated EBIT margin; EBIT ÷ store revenue only (cf. Scenarios 13.2%–15.5%).
-Ctrl+F "Company-operated stores"
 → 5,049,744 ($000) net revenue
 × 18.6% margin assumption → store EBIT ≈ 939,252 ($000)</t>
         </is>
@@ -8360,7 +8114,6 @@
       <c r="D10" s="19" t="inlineStr">
         <is>
           <t>Not consolidated EBIT margin; EBIT ÷ e-commerce revenue only (cf. Scenarios 13.2%–15.5%).
-Ctrl+F "E-commerce"
 → 4,918,697 ($000) net revenue
 × 23.6% margin assumption → e-comm EBIT ≈ 1,160,812 ($000)</t>
         </is>
@@ -8407,7 +8160,6 @@
       <c r="D11" s="19" t="inlineStr">
         <is>
           <t>Not consolidated EBIT margin; EBIT ÷ other-channel revenue only (cf. Scenarios 13.2%–15.5%).
-Ctrl+F "Net revenue" → 11,102,600
 Minus stores + e-comm → other channels ≈ 1,134,159 ($000)
 × 9.1% margin assumption → other EBIT ≈ 103,209 ($000)</t>
         </is>
@@ -8447,11 +8199,7 @@
           <t>Q2 FY2026 outlook: tax rate ≈ 30%</t>
         </is>
       </c>
-      <c r="D12" s="19" t="inlineStr">
-        <is>
-          <t>Ctrl+F "a tax rate of approximately 30%" → terminal marginal rate for t_operating glide path.</t>
-        </is>
-      </c>
+      <c r="D12" s="19" t="n"/>
       <c r="E12" s="20" t="n">
         <v>0.3</v>
       </c>
@@ -8479,7 +8227,7 @@
       </c>
       <c r="B13" s="17" t="inlineStr">
         <is>
-          <t>Not % of revenue; amortization period (years) if R&amp;D/software is capitalized. LULU: no separate R&amp;D cap.</t>
+          <t>amortization period (years) if R&amp;D/software is capitalized.</t>
         </is>
       </c>
       <c r="C13" s="24" t="inlineStr">
@@ -8535,11 +8283,7 @@
           <t>LULU FY2025 10-K: Income from operations</t>
         </is>
       </c>
-      <c r="D16" s="19" t="inlineStr">
-        <is>
-          <t>Ctrl+F "Income from operations" → 2,210,615 ($000). Forecast links to Scenarios EBIT.</t>
-        </is>
-      </c>
+      <c r="D16" s="19" t="n"/>
       <c r="E16" s="74" t="n">
         <v>2210615</v>
       </c>
@@ -8580,11 +8324,7 @@
           <t>LULU FY2025 10-K: amortization of intangible assets</t>
         </is>
       </c>
-      <c r="D17" s="19" t="inlineStr">
-        <is>
-          <t>Ctrl+F "Amortization of intangible assets" → other operating expense run-rate (add-back).</t>
-        </is>
-      </c>
+      <c r="D17" s="19" t="n"/>
       <c r="E17" s="74" t="n">
         <v>6961</v>
       </c>
@@ -8620,11 +8360,7 @@
           <t>LULU FY2025 10-K: restructuring charges</t>
         </is>
       </c>
-      <c r="D18" s="19" t="inlineStr">
-        <is>
-          <t>Ctrl+F "restructuring" → none material in FY25 10-K.</t>
-        </is>
-      </c>
+      <c r="D18" s="19" t="n"/>
       <c r="E18" s="74" t="n">
         <v>0</v>
       </c>
@@ -8692,9 +8428,7 @@
       </c>
       <c r="B20" s="17" t="inlineStr">
         <is>
-          <t>Not % of revenue; SBC add-back flag. Set to 0 (Convention A).
-SBC stays inside Scenarios EBIT/NOPAT as a real economic cost; DCF uses basic shares (111.4M).
-FY25 reference: $62,203k (10-K). Flag = 1 would add back (Convention B + diluted shares); not used.</t>
+          <t>SBC stays in EBIT (Convention A); DCF uses basic shares.</t>
         </is>
       </c>
       <c r="C20" s="18" t="inlineStr">
@@ -8704,8 +8438,7 @@
       </c>
       <c r="D20" s="19" t="inlineStr">
         <is>
-          <t>Ctrl+F "Stock-based compensation expense"
-→ 62,203 ($000) FY25 reference. Flag = 0: SBC stays in EBIT (Convention A); DCF IV uses basic 111,380k shares.</t>
+          <t>→ 62,203 ($000) FY25 reference. Flag = 0: SBC stays in EBIT (Convention A); DCF IV uses basic 111,380k shares.</t>
         </is>
       </c>
       <c r="E20" s="75">
@@ -8789,7 +8522,7 @@
       </c>
       <c r="B23" s="17" t="inlineStr">
         <is>
-          <t>Not % of revenue; implied lease interest ($1,028k FY25). Reclass from rent to unlevered EBIT; scales with revenue in forecast.</t>
+          <t>implied lease interest ($1,028k FY25).</t>
         </is>
       </c>
       <c r="C23" s="18" t="inlineStr">
@@ -8799,8 +8532,7 @@
       </c>
       <c r="D23" s="19" t="inlineStr">
         <is>
-          <t>Ctrl+F "Interest paid on lease liabilities"
-→ 1,028 ($000) supplemental cash-flow disclosure. Reclass to unlevered EBIT.</t>
+          <t>→ 1,028 ($000) supplemental cash-flow disclosure. Reclass to unlevered EBIT.</t>
         </is>
       </c>
       <c r="E23" s="74" t="n">
@@ -8963,7 +8695,7 @@
       </c>
       <c r="B28" s="17" t="inlineStr">
         <is>
-          <t>Not % of revenue; store-channel revenue from Revenue Drivers tab.</t>
+          <t>store-channel revenue from Revenue Drivers tab.</t>
         </is>
       </c>
       <c r="C28" s="18" t="inlineStr">
@@ -9008,7 +8740,7 @@
       </c>
       <c r="B29" s="17" t="inlineStr">
         <is>
-          <t>Not % of revenue; e-commerce revenue from Revenue Drivers tab.</t>
+          <t>e-commerce revenue from Revenue Drivers tab.</t>
         </is>
       </c>
       <c r="C29" s="18" t="inlineStr">
@@ -9053,7 +8785,7 @@
       </c>
       <c r="B30" s="17" t="inlineStr">
         <is>
-          <t>Not % of revenue; wholesale/license/outlet revenue from Revenue Drivers tab.</t>
+          <t>wholesale/license/outlet revenue from Revenue Drivers tab.</t>
         </is>
       </c>
       <c r="C30" s="18" t="inlineStr">
@@ -9112,7 +8844,6 @@
       <c r="D31" s="19" t="inlineStr">
         <is>
           <t>Not consolidated EBIT margin; store EBIT ÷ store revenue only.
-Ctrl+F "Company-operated stores"
 → 5,049,744 ($000)
 EBIT = Rev × 18.6% → ≈ 939,252 ($000)</t>
         </is>
@@ -9163,7 +8894,6 @@
       <c r="D32" s="19" t="inlineStr">
         <is>
           <t>Not consolidated EBIT margin; e-commerce EBIT ÷ e-commerce revenue only.
-Ctrl+F "E-commerce"
 → 4,918,697 ($000)
 EBIT = Rev × 23.6% → ≈ 1,160,812 ($000)</t>
         </is>
@@ -9425,10 +9155,7 @@
       </c>
       <c r="D39" s="19" t="inlineStr">
         <is>
-          <t>t_operating = (tax + interest×30%) ÷ (EBT + interest).
-Ctrl+F "Income tax expense" → 659,784
-Ctrl+F "Income before income tax expense" → 2,238,967
-Ctrl+F "Interest paid on lease liabilities" → 1,028</t>
+          <t>t_operating = (tax + interest×30%) ÷ (EBT + interest).</t>
         </is>
       </c>
       <c r="E39" s="77" t="n">
@@ -9543,7 +9270,7 @@
     <row r="43">
       <c r="A43" s="73" t="inlineStr">
         <is>
-          <t>Phase 5 — workflow (execution steps)</t>
+          <t>Phase 5 — Reconciliation (execution steps)</t>
         </is>
       </c>
     </row>
@@ -9835,11 +9562,7 @@
           <t>Source (click)</t>
         </is>
       </c>
-      <c r="D2" s="78" t="inlineStr">
-        <is>
-          <t>Ctrl+F (prove number)</t>
-        </is>
-      </c>
+      <c r="D2" s="78" t="n"/>
       <c r="E2" s="71" t="inlineStr">
         <is>
           <t>FY2025A</t>
@@ -9882,7 +9605,7 @@
       </c>
       <c r="M2" s="78" t="inlineStr">
         <is>
-          <t>Alt. Ctrl+F</t>
+          <t>Alt. source</t>
         </is>
       </c>
     </row>
@@ -9892,11 +9615,7 @@
           <t>Forecast drivers linked to Scenarios tab → Base case (column G)</t>
         </is>
       </c>
-      <c r="C3" s="19" t="inlineStr">
-        <is>
-          <t>Ctrl+F "Net revenue" → 11,102,600 or "Depreciation and amortization" → 496,228 on this 10-K HTML file</t>
-        </is>
-      </c>
+      <c r="C3" s="19" t="n"/>
       <c r="E3" s="83" t="inlineStr">
         <is>
           <t>10-K</t>
@@ -9911,20 +9630,17 @@
     <row r="4" ht="36" customHeight="1">
       <c r="A4" s="38" t="inlineStr">
         <is>
-          <t>Full Assumptions Guide (PDF)
-Ctrl+F: Every red assumption on every tab — justification, source link, Ctrl+F proof.</t>
+          <t>Full Assumptions Guide (PDF)</t>
         </is>
       </c>
       <c r="C4" s="85" t="inlineStr">
         <is>
-          <t>NOPAT Bridge tab
-Ctrl+F: 5-phase EBIT normalization → normalized NOPAT (base case).</t>
+          <t>NOPAT Bridge tab</t>
         </is>
       </c>
       <c r="D4" s="85" t="inlineStr">
         <is>
-          <t>Revenue Drivers tab
-Ctrl+F: Bottom-up store / DTC / category schedule (FY26–30).</t>
+          <t>Revenue Drivers tab</t>
         </is>
       </c>
     </row>
@@ -9971,21 +9687,16 @@
       <c r="B6" s="19" t="inlineStr">
         <is>
           <t>−6.1% FY2026 revenue growth matches company guidance midpoint of −5% to −7% after Q2 FY2026 print.
-Also: 2.3% FY27–30 growth matches StockAnalysis Revenue Growth Forecast (3Y) of 2.26%; next-year consensus is +2.64%.</t>
+2.3% FY27–30 growth matches StockAnalysis Revenue Growth Forecast (3Y) of 2.26%; next-year consensus is +2.64%.</t>
         </is>
       </c>
       <c r="C6" s="38" t="inlineStr">
         <is>
           <t>LULU Q2 FY2026 earnings release
-Also: StockAnalysis: LULU 3Y revenue forecast</t>
-        </is>
-      </c>
-      <c r="D6" s="19" t="inlineStr">
-        <is>
-          <t>Ctrl+F "decline of 5% to 7%" → FY2026 revenue guide; model −6.1% midpoint
-Also: Ctrl+F "Revenue Growth Forecast (3Y)" → 2.26%. That is the unique line (do not search "Net revenue"). Model FY27–30 uses 2.3%.</t>
-        </is>
-      </c>
+StockAnalysis: LULU 3Y revenue forecast</t>
+        </is>
+      </c>
+      <c r="D6" s="19" t="n"/>
       <c r="F6" s="32">
         <f>F5/E5-1</f>
         <v/>
@@ -10026,11 +9737,8 @@
       <c r="D7" s="19" t="inlineStr">
         <is>
           <t>56.6% of revenue (gross margin).
-Ctrl+F "Gross profit"
 → 6,284,132 ($000)
-Ctrl+F "Net revenue"
 → 11,102,600 ($000)
-Ctrl+F "Cost of goods sold"
 → 4,818,468 ($000)</t>
         </is>
       </c>
@@ -10101,21 +9809,16 @@
       <c r="B9" s="19" t="inlineStr">
         <is>
           <t>13.2% is the real/run-rate OM: Q2 18.8% minus 560bps of tariff refunds. FY26 then adds the $134.5M refund once on top.
-Also: FY30 15.5% is a partial recovery vs the FY25 10-K OM of 19.9% (unique Ctrl+F). Still well below the FY24 23.7% peak.</t>
+FY30 15.5% is a partial recovery vs the FY25 10-K OM of 19.9% (per FY25 10-K). Still well below the FY24 23.7% peak.</t>
         </is>
       </c>
       <c r="C9" s="38" t="inlineStr">
         <is>
           <t>Q2 FY2026 release: 18.8% OM minus 560bps tariffs
-Also: FY2025 10-K: Operating margin 19.9% (one hit)</t>
-        </is>
-      </c>
-      <c r="D9" s="19" t="inlineStr">
-        <is>
-          <t>Ctrl+F "18.8%" (Q2 OM) and "560 basis points" (tariff boost). Real run-rate = 18.8% − 5.6% = 13.2%. Do not use "decreased 13%".
-Also: Ctrl+F "19.9%" (one hit) → Operating margin decreased 380 basis points to 19.9%. That is FY25 OM. Do not search the words Income from operations (17 hits). Model FY30 15.5% is a partial-recovery assumption.</t>
-        </is>
-      </c>
+FY2025 10-K: Operating margin 19.9% (one hit)</t>
+        </is>
+      </c>
+      <c r="D9" s="19" t="n"/>
       <c r="F9" s="32">
         <f>Scenarios!G40</f>
         <v/>
@@ -10157,11 +9860,7 @@
           <t>Q2 FY2026 release: $134.5M IEEPA tariff refunds</t>
         </is>
       </c>
-      <c r="D10" s="19" t="inlineStr">
-        <is>
-          <t>Ctrl+F "134.5 million" → IEEPA tariff refunds reduced COGS. Add this dollar amount to FY26 EBIT only. Full-year boost = 134.5 / FY26 sales ≈ 1.3ppt, not 5.6ppt.</t>
-        </is>
-      </c>
+      <c r="D10" s="19" t="n"/>
       <c r="E10" s="74" t="n">
         <v>0</v>
       </c>
@@ -10320,11 +10019,7 @@
           <t>LULU CF statement (10-K)</t>
         </is>
       </c>
-      <c r="D15" s="19" t="inlineStr">
-        <is>
-          <t>Ctrl+F "Depreciation and amortization" → 496,228 on this 10-K HTML (not the SEC viewer). ÷ "Net revenue" 11,102,600 = 4.5%.</t>
-        </is>
-      </c>
+      <c r="D15" s="19" t="n"/>
       <c r="F15" s="20">
         <f>Scenarios!$G$12</f>
         <v/>
@@ -10386,18 +10081,25 @@
       <c r="B17" s="19" t="inlineStr">
         <is>
           <t>FY26 7.0% is $735M on $10.4B sales, not FY25 $11.1B. Since 7.0% steps toward FY25 6.1%, we assume a fade: DCF 5.5% = (7.0+6.0+5.5+5.0+4.0)/5.
-Also: FY26 sales are $10.35–$10.50B (earnings). Use that $10.4B year as the 7% denominator, not FY25 $11.1B.</t>
+FY26 sales are $10.35–$10.50B (earnings). Use that $10.4B year as the 7% denominator, not FY25 $11.1B.</t>
         </is>
       </c>
       <c r="C17" s="38" t="inlineStr">
         <is>
           <t>LULU 10-K: 2026 capex guide $725–745M
-Also: Q2 FY2026 outlook: $10.350B–$10.500B sales</t>
+Q2 FY2026 outlook: $10.350B–$10.500B sales</t>
         </is>
       </c>
       <c r="D17" s="19" t="inlineStr">
         <is>
-          <t>FY25 actual (10-K) Ctrl+F "680,802" → capex $680.8M Ctrl+F "11,102,600" → sales $11.1B 680.8 / 11,102.6 = 6.1% FY26 capex (10-K) Ctrl+F "$725.0 million and $745.0 million" → mid $735M FY26 sales (earnings) Ctrl+F "$10.350 billion to $10.500 billion" → $10.35–$10.50B (mid $10.425B) 7.0% = $735M / $10.425B ($10B year, not FY25 $11.1B) DCF blend Fade 7.0 / 6.0 / 5.5 / 5.0 / 4.0 5.5% = (7.0+6.0+5.5+5.0+4.0)/5</t>
+          <t>FY25 actual (10-K)
+680.8 / 11,102.6 = 6.1%
+FY26 capex (10-K)
+FY26 sales (earnings)
+7.0% = $735M / $10.425B ($10B year, not FY25 $11.1B)
+DCF blend
+Fade 7.0 / 6.0 / 5.5 / 5.0 / 4.0
+5.5% = (7.0+6.0+5.5+5.0+4.0)/5</t>
         </is>
       </c>
       <c r="F17" s="20">
@@ -10467,7 +10169,7 @@
       </c>
       <c r="B20" s="17" t="inlineStr">
         <is>
-          <t>Not % of revenue; DSO (days), flat ~6.3. Mostly own stores/DTC (cash at register); AR is small wholesale residual; predictable ~6 days FY22–25.</t>
+          <t>DSO flat ~6.3 days — DTC/store cash sales dominate; AR is wholesale residual.</t>
         </is>
       </c>
       <c r="C20" s="18" t="inlineStr">
@@ -10477,16 +10179,7 @@
       </c>
       <c r="D20" s="19" t="inlineStr">
         <is>
-          <t>Not % of revenue; DSO (days), flat ~6.3.
-Why flat: ~90%+ revenue is company-operated stores + e-commerce (cash/card at sale);
-AR is a small, stable wholesale/license residual; predictable collection, not trade credit.
-Ctrl+F "Accounts receivable, net"
-→ 190,657 ($000)
-Ctrl+F "Net revenue"
-→ 11,102,600 ($000)
-DSO = (190,657 ÷ 11,102,600) × 365 ≈ 6.3 days (~6.0–6.3 FY22–25).
-Ctrl+F "company-operated stores"
-Ctrl+F "E-commerce"</t>
+          <t>DSO flat ~6.3 days — DTC/store cash sales dominate; AR is wholesale residual.</t>
         </is>
       </c>
       <c r="E20" s="88" t="n">
@@ -10537,9 +10230,7 @@
         <is>
           <t>Implied ~1.7% of revenue (= 190,657 ÷ 11,102,600); not a direct % plug.
 AR_t = (DSO ÷ 365) × Revenue_t. DSO flat because own-store/DTC dominates; AR scales predictably with sales.
-Ctrl+F "Accounts receivable, net"
 → 190,657 ($000)
-Ctrl+F "Net revenue"
 → 11,102,600 ($000)</t>
         </is>
       </c>
@@ -10579,34 +10270,18 @@
       </c>
       <c r="B22" s="19" t="inlineStr">
         <is>
-          <t>Not % of revenue; DIO (days).
-FY25 anchor: DIO = (Inventories ÷ COGS) × 365 = (1,700,753 ÷ 4,818,468) × 365 ≈ 129 days (FY24 inv: 1,442,081).
-Forecast path: DIO_t = FY25 DIO − (1 day × year t); flat across scenarios.
-Also: Not % of revenue; subtract 1 DIO day per forecast year (−5 days FY26–30).
-Feeds Inventories = (DIO_t ÷ 365) × COGS_t.
-Ctrl+F "reduce the percentage of markdowns"
-Ctrl+F "On a unit basis, we expect inventories to slightly decrease"</t>
+          <t>DIO: FY25 anchor ~129 days; −1 day/yr through FY30 (inventory discipline).</t>
         </is>
       </c>
       <c r="C22" s="38" t="inlineStr">
         <is>
           <t>LULU FY2025 10-K: Inventories &amp; COGS
-Also: LULU FY2025 10-K: inventory &amp; markdown outlook</t>
+LULU FY2025 10-K: inventory &amp; markdown outlook</t>
         </is>
       </c>
       <c r="D22" s="19" t="inlineStr">
         <is>
-          <t>Not % of revenue; DIO (days).
-FY25 anchor formula: DIO = (Inventories ÷ COGS) × 365
-Ctrl+F "Inventories"
-→ 1,700,753 ($000) | FY24: 1,442,081
-Ctrl+F "Cost of goods sold"
-→ 4,818,468 ($000) = (1,700,753 ÷ 4,818,468) × 365 ≈ 129 days
-Forecast: DIO_t = FY25 DIO − (1 × year t)
-Also: Not % of revenue; DIO −1 day/yr (−5 days FY26–30).
-Feeds Inventories_t = (DIO_t ÷ 365) × COGS_t.
-Ctrl+F "reduce the percentage of markdowns"
-Ctrl+F "On a unit basis, we expect inventories to slightly decrease"</t>
+          <t>DIO: FY25 anchor ~129 days; −1 day/yr through FY30 (inventory discipline).</t>
         </is>
       </c>
       <c r="E22" s="88" t="n">
@@ -10645,13 +10320,7 @@
       </c>
       <c r="B23" s="17" t="inlineStr">
         <is>
-          <t>Not % of revenue; $ balance (not a direct % plug).
-Inventories_t = (DIO_t ÷ 365) × COGS_t
-COGS_t = Revenue_t × (1 − GM%). FY25 check: (129 ÷ 365) × 4,818,468 ≈ 1,700,753.
-Ctrl+F "Inventories"
-→ 1,700,753 ($000)
-Ctrl+F "Cost of goods sold"
-→ 4,818,468 ($000)</t>
+          <t>$ balance (not a direct % plug).</t>
         </is>
       </c>
       <c r="C23" s="18" t="inlineStr">
@@ -10661,13 +10330,7 @@
       </c>
       <c r="D23" s="19" t="inlineStr">
         <is>
-          <t>Not % of revenue; Inventories_t = (DIO_t ÷ 365) × COGS_t.
-COGS_t = Revenue_t × (1 − GM%).
-Ctrl+F "Inventories"
-→ 1,700,753 ($000)
-Ctrl+F "Cost of goods sold"
-→ 4,818,468 ($000)
-FY25 proof: (129 ÷ 365) × 4,818,468 ≈ 1,700,753</t>
+          <t>DIO: FY25 anchor ~129 days; −1 day/yr through FY30 (inventory discipline).</t>
         </is>
       </c>
       <c r="E23" s="74" t="n">
@@ -10706,7 +10369,7 @@
       </c>
       <c r="B24" s="17" t="inlineStr">
         <is>
-          <t>Not % of revenue; DPO (days), flat ~25.1. Implied AP ≈3.0% of sales / 6.9% of COGS.</t>
+          <t>DPO flat ~25 days; AP scales with COGS (~3% of sales).</t>
         </is>
       </c>
       <c r="C24" s="18" t="inlineStr">
@@ -10716,9 +10379,7 @@
       </c>
       <c r="D24" s="19" t="inlineStr">
         <is>
-          <t>Ctrl+F "Accounts payable"
-→ 331,421 ($000)
-Ctrl+F "Cost of goods sold"
+          <t>→ 331,421 ($000)
 → 4,818,468 ($000)
 Not % of revenue; DPO ≈ 25.1 days. Implied AP ≈ 3.0% of sales / 6.9% of COGS.</t>
         </is>
@@ -10769,9 +10430,7 @@
       </c>
       <c r="D25" s="19" t="inlineStr">
         <is>
-          <t>Ctrl+F "Accounts payable"
-→ 331,421 ($000)
-Ctrl+F "Net revenue"
+          <t>→ 331,421 ($000)
 → 11,102,600 ($000)
 Implied ~3.0% of revenue (= 331,421 ÷ 11,102,600); forecast via DPO×COGS.</t>
         </is>
@@ -10822,9 +10481,7 @@
       </c>
       <c r="D26" s="19" t="inlineStr">
         <is>
-          <t>Ctrl+F "Prepaid expenses and other current assets"
-→ 211,620 ($000)
-Ctrl+F "Prepaid and receivable income taxes"
+          <t>→ 211,620 ($000)
 → 352,469 ($000)
 5.1% of revenue (flat). OCA residual = 564,089 ÷ 11,102,600.</t>
         </is>
@@ -10871,9 +10528,7 @@
       </c>
       <c r="D27" s="19" t="inlineStr">
         <is>
-          <t>Ctrl+F "Prepaid expenses and other current assets"
-→ 211,620 ($000)
-Ctrl+F "Prepaid and receivable income taxes"
+          <t>→ 211,620 ($000)
 → 352,469 ($000)
 5.1% of revenue (flat). OCA residual = 564,089 ÷ 11,102,600.</t>
         </is>
@@ -10924,9 +10579,7 @@
       </c>
       <c r="D28" s="19" t="inlineStr">
         <is>
-          <t>Ctrl+F "Accrued liabilities and other"
-→ 662,982 ($000)
-Ctrl+F "Net revenue"
+          <t>→ 662,982 ($000)
 → 11,102,600 ($000)
 6.0% of revenue (flat). 662,982 ÷ 11,102,600.</t>
         </is>
@@ -10973,9 +10626,7 @@
       </c>
       <c r="D29" s="19" t="inlineStr">
         <is>
-          <t>Ctrl+F "Accrued liabilities and other"
-→ 662,982 ($000)
-Ctrl+F "Net revenue"
+          <t>→ 662,982 ($000)
 → 11,102,600 ($000)
 6.0% of revenue (flat). 662,982 ÷ 11,102,600.</t>
         </is>
@@ -11160,7 +10811,7 @@
       </c>
       <c r="B33" s="17" t="inlineStr">
         <is>
-          <t>Not % of revenue; $ change in NWC year-over-year. Prior-year NWC minus current-year NWC for the FCF bridge.</t>
+          <t>$ change in NWC year-over-year.</t>
         </is>
       </c>
       <c r="C33" s="18" t="inlineStr">
@@ -11170,9 +10821,7 @@
       </c>
       <c r="D33" s="19" t="inlineStr">
         <is>
-          <t>Not % of revenue; $ change year-over-year.
-FY26: revenue −6.1% + DIO −1 day → NWC falls → ΔNWC positive (WC release).
-FY27–30: revenue +2.3%/yr → AR &amp; inventory rebuild → ΔNWC negative (WC build).</t>
+          <t>$ change year-over-year.</t>
         </is>
       </c>
       <c r="F33" s="25">
@@ -11362,11 +11011,7 @@
           <t>FRED: Real GDP (GDPC1)</t>
         </is>
       </c>
-      <c r="D43" s="19" t="inlineStr">
-        <is>
-          <t>Ctrl+F "Q2 2026" → 24,269.613 and "Q2 2025" → 23,770.976. YoY = 2.1%. Model terminal g 2.25%.</t>
-        </is>
-      </c>
+      <c r="D43" s="19" t="n"/>
       <c r="E43" s="32">
         <f>Scenarios!$G$10</f>
         <v/>
@@ -11449,11 +11094,7 @@
           <t>10-K</t>
         </is>
       </c>
-      <c r="D50" s="19" t="inlineStr">
-        <is>
-          <t>Ctrl+F "Cash and cash equivalents" → 1,807,202 ($000) FY2025</t>
-        </is>
-      </c>
+      <c r="D50" s="19" t="n"/>
       <c r="E50" s="74" t="n">
         <v>1807202</v>
       </c>
@@ -11474,11 +11115,7 @@
           <t>LULU FY2025 10-K: operating lease liabilities</t>
         </is>
       </c>
-      <c r="D51" s="19" t="inlineStr">
-        <is>
-          <t>Ctrl+F "Current lease liabilities" → 298,724 | "Non-current lease liabilities" → 1,499,717 | sum 1,798,441 ($000). Funded debt: "no borrowings were outstanding"</t>
-        </is>
-      </c>
+      <c r="D51" s="19" t="n"/>
       <c r="E51" s="74" t="n">
         <v>-1798441</v>
       </c>
@@ -11519,11 +11156,7 @@
           <t>10-K</t>
         </is>
       </c>
-      <c r="D55" s="19" t="inlineStr">
-        <is>
-          <t>Ctrl+F "111,380 and 116,166 issued and outstanding" → 111,380k class A (FY25 10-K cover)</t>
-        </is>
-      </c>
+      <c r="D55" s="19" t="n"/>
       <c r="E55" s="74" t="n">
         <v>111380</v>
       </c>
@@ -11554,11 +11187,7 @@
           <t>NASDAQ</t>
         </is>
       </c>
-      <c r="D57" s="19" t="inlineStr">
-        <is>
-          <t>Ctrl+F "closed at $100.61" → Last Sale on NASDAQ quote page</t>
-        </is>
-      </c>
+      <c r="D57" s="19" t="n"/>
       <c r="E57" s="97" t="n">
         <v>100</v>
       </c>
@@ -11968,7 +11597,7 @@
       </c>
       <c r="D82" s="19" t="inlineStr">
         <is>
-          <t>No peer Ctrl+F. This cell = Gordon TV / FY30 EBITDA = (UFCF/EBITDA)×(1+g)/(WACC−g). WACC and g are sourced on those rows.</t>
+          <t>No peer print. This cell = Gordon TV / FY30 EBITDA = (UFCF/EBITDA)×(1+g)/(WACC−g). WACC and g are sourced on those rows.</t>
         </is>
       </c>
       <c r="E82" s="94">
@@ -12176,11 +11805,7 @@
           <t>FRED: Real GDP (GDPC1)</t>
         </is>
       </c>
-      <c r="D98" s="19" t="inlineStr">
-        <is>
-          <t>Ctrl+F "GDPC1" → bounds terminal-g sensitivity grid 1.5%–3.0%</t>
-        </is>
-      </c>
+      <c r="D98" s="19" t="n"/>
       <c r="F98" s="109" t="n">
         <v>0.015</v>
       </c>
@@ -12395,7 +12020,7 @@
       </c>
       <c r="D104" s="19" t="inlineStr">
         <is>
-          <t>Scenarios tab → Ctrl+F "WACC" and "Terminal growth" rows (base-case inputs)</t>
+          <t>Scenarios tab → WACC and terminal growth rows rows (base-case inputs)</t>
         </is>
       </c>
       <c r="L104" s="95" t="inlineStr">
@@ -12403,11 +12028,7 @@
           <t>FRED: Real GDP (GDPC1)</t>
         </is>
       </c>
-      <c r="M104" s="19" t="inlineStr">
-        <is>
-          <t>Ctrl+F "GDPC1" → bounds terminal-g sensitivity grid 1.5%–3.0%</t>
-        </is>
-      </c>
+      <c r="M104" s="19" t="n"/>
     </row>
   </sheetData>
   <hyperlinks>
@@ -12524,11 +12145,7 @@
           <t>Source (click)</t>
         </is>
       </c>
-      <c r="D2" s="15" t="inlineStr">
-        <is>
-          <t>Ctrl+F (prove number)</t>
-        </is>
-      </c>
+      <c r="D2" s="15" t="n"/>
     </row>
     <row r="3">
       <c r="A3" s="14" t="inlineStr">
@@ -12548,11 +12165,7 @@
           <t>10-K</t>
         </is>
       </c>
-      <c r="D4" s="19" t="inlineStr">
-        <is>
-          <t>Ctrl+F "Net revenue" → 11,102,600 ($000) in FY2025 column</t>
-        </is>
-      </c>
+      <c r="D4" s="19" t="n"/>
       <c r="E4" s="74" t="n">
         <v>11102600</v>
       </c>
@@ -12595,11 +12208,7 @@
           <t>Release</t>
         </is>
       </c>
-      <c r="D7" s="19" t="inlineStr">
-        <is>
-          <t>Ctrl+F "$9.48 to $9.73" → FY2026 diluted EPS guidance; model midpoint $9.61</t>
-        </is>
-      </c>
+      <c r="D7" s="19" t="n"/>
       <c r="E7" s="97" t="n">
         <v>9.609999999999999</v>
       </c>
@@ -12615,11 +12224,7 @@
           <t>10-K</t>
         </is>
       </c>
-      <c r="D8" s="19" t="inlineStr">
-        <is>
-          <t>Ctrl+F "Cash and cash equivalents" → 1,807,202 ($000) FY2025</t>
-        </is>
-      </c>
+      <c r="D8" s="19" t="n"/>
       <c r="E8" s="74" t="n">
         <v>1807202</v>
       </c>
@@ -12635,11 +12240,7 @@
           <t>10-K</t>
         </is>
       </c>
-      <c r="D9" s="19" t="inlineStr">
-        <is>
-          <t>Ctrl+F "111,380 and 116,166 issued and outstanding" → 111,380k class A (FY25 10-K cover)</t>
-        </is>
-      </c>
+      <c r="D9" s="19" t="n"/>
       <c r="E9" s="74" t="n">
         <v>111380</v>
       </c>
@@ -12655,11 +12256,7 @@
           <t>NASDAQ</t>
         </is>
       </c>
-      <c r="D10" s="19" t="inlineStr">
-        <is>
-          <t>Ctrl+F "closed at $100.61" → Last Sale on NASDAQ quote page</t>
-        </is>
-      </c>
+      <c r="D10" s="19" t="n"/>
       <c r="E10" s="97" t="n">
         <v>100</v>
       </c>
@@ -12731,11 +12328,7 @@
           <t>Source</t>
         </is>
       </c>
-      <c r="D18" s="113" t="inlineStr">
-        <is>
-          <t>Ctrl+F / proof</t>
-        </is>
-      </c>
+      <c r="D18" s="113" t="n"/>
       <c r="E18" s="114" t="inlineStr">
         <is>
           <t>EV/EBITDA</t>
@@ -13108,7 +12701,7 @@
     <row r="31">
       <c r="A31" s="14" t="inlineStr">
         <is>
-          <t>ALO YOGA BUILD — no source prints EV/EBITDA (: Reuters + Forbes)</t>
+          <t>ALO YOGA BUILD — no source prints EV/EBITDA (Reuters + Forbes)</t>
         </is>
       </c>
     </row>
@@ -13127,22 +12720,16 @@
       </c>
       <c r="B33" s="19" t="inlineStr">
         <is>
-          <t>Reuters: about $10 billion Moelis ask for Color Image. 2026 follow-up: no deal announced. Ask, not a print.
-Also: Reuters June 2026: no deal was announced on the 2023 process. The $10bn is still an ask.</t>
+          <t>Reuters: about $10 billion Moelis ask for Color Image. 2026 follow-up: no deal announced. Ask, not a print.</t>
         </is>
       </c>
       <c r="C33" s="38" t="inlineStr">
         <is>
           <t>Reuters: Alo parent $10bn Moelis ask
-Also: Reuters: Alo 2023 process; no deal</t>
-        </is>
-      </c>
-      <c r="D33" s="19" t="inlineStr">
-        <is>
-          <t>Ctrl+F "at about $10 billion" and "hired investment bank Moelis". That is the 2023 ask, not a closed EV.
-Also: Ctrl+F "roughly $10 billion" and "No deal was announced". Still an ask.</t>
-        </is>
-      </c>
+Reuters: Alo 2023 process; no deal</t>
+        </is>
+      </c>
+      <c r="D33" s="19" t="n"/>
       <c r="E33" s="117" t="n">
         <v>10</v>
       </c>
@@ -13163,11 +12750,7 @@
           <t>Forbes: Color Image nearly $2bn sales</t>
         </is>
       </c>
-      <c r="D34" s="19" t="inlineStr">
-        <is>
-          <t>Ctrl+F "nearly $2 billion". Forbes estimate for Color Image parent (Alo + Bella+Canvas), not Alo-only EBITDA.</t>
-        </is>
-      </c>
+      <c r="D34" s="19" t="n"/>
       <c r="E34" s="117" t="n">
         <v>2</v>
       </c>
@@ -13190,7 +12773,7 @@
       </c>
       <c r="D35" s="19" t="inlineStr">
         <is>
-          <t>No Ctrl+F for EV/EBITDA — found none on Reuters or Forbes. This cell is E33 / E34 (ask ÷ parent sales). Not the TV.</t>
+          <t>This cell is E33 / E34 (ask ÷ parent sales). Not the TV.</t>
         </is>
       </c>
       <c r="E35" s="118">
@@ -13216,7 +12799,7 @@
       </c>
       <c r="D36" s="19" t="inlineStr">
         <is>
-          <t>No Ctrl+F. Reuters, Forbes, and PitchBook do not print Alo EV/EBITDA.</t>
+          <t>Reuters, Forbes, and PitchBook do not print Alo EV/EBITDA.</t>
         </is>
       </c>
       <c r="E36" s="119" t="inlineStr">
@@ -13406,11 +12989,7 @@
           <t>Source</t>
         </is>
       </c>
-      <c r="D56" s="113" t="inlineStr">
-        <is>
-          <t>Ctrl+F</t>
-        </is>
-      </c>
+      <c r="D56" s="113" t="n"/>
       <c r="E56" s="114" t="inlineStr">
         <is>
           <t>Low mult.</t>
@@ -13452,8 +13031,8 @@
       </c>
       <c r="D57" s="19" t="inlineStr">
         <is>
-          <t>Lo: Ctrl+F "EV / EBITDA" → LULU trough ~5x; football-field floor 5.0x
-Hi: Ctrl+F "EV / EBITDA" → 7.95. Football-field cap 8.0x (Deckers). Not the selected exit.</t>
+          <t>Lo:.0x
+Hi:.95. Football-field cap 8.0x (Deckers). Not the selected exit.</t>
         </is>
       </c>
       <c r="E57" s="120" t="n">
@@ -13489,7 +13068,7 @@
       </c>
       <c r="D58" s="19" t="inlineStr">
         <is>
-          <t>No peer Ctrl+F. This cell = Gordon TV / FY30 EBITDA = (UFCF/EBITDA)×(1+g)/(WACC−g). WACC and g are sourced on those rows.</t>
+          <t>No peer print. This cell = Gordon TV / FY30 EBITDA = (UFCF/EBITDA)×(1+g)/(WACC−g). WACC and g are sourced on those rows.</t>
         </is>
       </c>
       <c r="E58" s="118">
@@ -13521,8 +13100,8 @@
       </c>
       <c r="D59" s="19" t="inlineStr">
         <is>
-          <t>Lo: Ctrl+F "Forward PE" → LULU ~12.3x; low-case multiple assumption 10.0x
-Hi: Ctrl+F "Forward PE" → NKE peer benchmark; high-case assumption 18.0x</t>
+          <t>Lo:.3x; low-case multiple assumption 10.0x
+Hi:.0x</t>
         </is>
       </c>
       <c r="E59" s="120" t="n">
@@ -13577,11 +13156,7 @@
           <t>NASDAQ</t>
         </is>
       </c>
-      <c r="D62" s="19" t="inlineStr">
-        <is>
-          <t>Ctrl+F "closed at $100.61" → Last Sale on NASDAQ quote page</t>
-        </is>
-      </c>
+      <c r="D62" s="19" t="n"/>
       <c r="E62" s="125" t="n">
         <v>100</v>
       </c>

</xml_diff>

<commit_message>
Sanitize Excel text: remove em dashes, arrows, bullets, Unicode symbols
Replace en/em dashes, arrows, middle dots, beta/Delta glyphs, and subscripts
with plain ASCII in text cells only; formulas unchanged.

Co-authored-by: cag56988 <cag56988@usc.edu>
</commit_message>
<xml_diff>
--- a/LULU/unbeiesgbar2model.xlsx
+++ b/LULU/unbeiesgbar2model.xlsx
@@ -1141,7 +1141,7 @@
     <row r="5">
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>FY2025A – FY2030E | US$ thousands</t>
+          <t>FY2025A - FY2030E | US$ thousands</t>
         </is>
       </c>
     </row>
@@ -1157,7 +1157,7 @@
     <row r="9">
       <c r="B9" s="5" t="inlineStr">
         <is>
-          <t>Tabs: WACC · Scenarios · Revenue Drivers · NOPAT Bridge · DCF · Comps</t>
+          <t>Tabs: WACC / Scenarios / Revenue Drivers / NOPAT Bridge / DCF / Comps</t>
         </is>
       </c>
     </row>
@@ -1181,7 +1181,11 @@
       <c r="B16" s="5" t="n"/>
     </row>
     <row r="17" ht="36" customHeight="1">
-      <c r="B17" s="10" t="n"/>
+      <c r="B17" s="10" t="inlineStr">
+        <is>
+          <t>LULU_Assumptions_Memo.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="18"/>
     <row r="19">
@@ -1370,14 +1374,14 @@
     <row r="15">
       <c r="A15" s="14" t="inlineStr">
         <is>
-          <t>Beta (unlever → relever)</t>
+          <t>Beta (unlever to relever)</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="16" t="inlineStr">
         <is>
-          <t>Observed Beta (5Y Monthly) — levered βL</t>
+          <t>Observed Beta (5Y Monthly) - levered betaL</t>
         </is>
       </c>
       <c r="B16" s="27" t="n">
@@ -1397,7 +1401,7 @@
     <row r="18" ht="28" customHeight="1">
       <c r="A18" s="16" t="inlineStr">
         <is>
-          <t>Yahoo Market Cap (same page as βL)</t>
+          <t>Yahoo Market Cap (same page as betaL)</t>
         </is>
       </c>
       <c r="B18" s="22" t="n">
@@ -1407,7 +1411,7 @@
     <row r="19" ht="28" customHeight="1">
       <c r="A19" s="16" t="inlineStr">
         <is>
-          <t>D/E for unlever (Yahoo debt mrq ÷ Yahoo market cap)</t>
+          <t>D/E for unlever (Yahoo debt mrq / Yahoo market cap)</t>
         </is>
       </c>
       <c r="B19" s="28">
@@ -1418,7 +1422,7 @@
     <row r="20" ht="28" customHeight="1">
       <c r="A20" s="16" t="inlineStr">
         <is>
-          <t>Yahoo book D/E (mrq) — reference only</t>
+          <t>Yahoo book D/E (mrq) - reference only</t>
         </is>
       </c>
       <c r="B20" s="27" t="n">
@@ -1428,7 +1432,7 @@
     <row r="21" ht="28" customHeight="1">
       <c r="A21" s="16" t="inlineStr">
         <is>
-          <t>Unlevered βu</t>
+          <t>Unlevered betau</t>
         </is>
       </c>
       <c r="B21" s="28">
@@ -1450,7 +1454,7 @@
     <row r="23" ht="28" customHeight="1">
       <c r="A23" s="16" t="inlineStr">
         <is>
-          <t>Sector βu benchmark (Damodaran Special Lines) — not used</t>
+          <t>Sector betau benchmark (Damodaran Special Lines) - not used</t>
         </is>
       </c>
       <c r="B23" s="27" t="n">
@@ -1481,7 +1485,7 @@
     <row r="27">
       <c r="A27" s="23" t="inlineStr">
         <is>
-          <t>Cost of equity = rf + β × ERP</t>
+          <t>Cost of equity = rf + beta x ERP</t>
         </is>
       </c>
       <c r="B27" s="30">
@@ -1638,7 +1642,7 @@
     <row r="5" ht="28" customHeight="1">
       <c r="A5" s="16" t="inlineStr">
         <is>
-          <t>FY2027–FY2030E revenue growth (avg)</t>
+          <t>FY2027-FY2030E revenue growth (avg)</t>
         </is>
       </c>
       <c r="C5" s="20" t="n">
@@ -1799,7 +1803,7 @@
     <row r="15" ht="150" customHeight="1">
       <c r="A15" s="16" t="inlineStr">
         <is>
-          <t>DSO (days) — flat vs FY25</t>
+          <t>DSO (days) - flat vs FY25</t>
         </is>
       </c>
       <c r="C15" s="39" t="n">
@@ -1847,7 +1851,7 @@
     <row r="18" ht="84" customHeight="1">
       <c r="A18" s="16" t="inlineStr">
         <is>
-          <t>DPO (days) — flat vs FY25</t>
+          <t>DPO (days) - flat vs FY25</t>
         </is>
       </c>
       <c r="C18" s="39" t="n">
@@ -1935,7 +1939,7 @@
     <row r="25">
       <c r="A25" s="41" t="inlineStr">
         <is>
-          <t>Revenue – year 1</t>
+          <t>Revenue - year 1</t>
         </is>
       </c>
       <c r="C25" s="42">
@@ -1954,7 +1958,7 @@
     <row r="26">
       <c r="A26" s="41" t="inlineStr">
         <is>
-          <t>Revenue – year 2</t>
+          <t>Revenue - year 2</t>
         </is>
       </c>
       <c r="C26" s="42">
@@ -1973,7 +1977,7 @@
     <row r="27">
       <c r="A27" s="41" t="inlineStr">
         <is>
-          <t>Revenue – year 3</t>
+          <t>Revenue - year 3</t>
         </is>
       </c>
       <c r="C27" s="42">
@@ -1992,7 +1996,7 @@
     <row r="28">
       <c r="A28" s="41" t="inlineStr">
         <is>
-          <t>Revenue – year 4</t>
+          <t>Revenue - year 4</t>
         </is>
       </c>
       <c r="C28" s="42">
@@ -2011,7 +2015,7 @@
     <row r="29">
       <c r="A29" s="41" t="inlineStr">
         <is>
-          <t>Revenue – year 5</t>
+          <t>Revenue - year 5</t>
         </is>
       </c>
       <c r="C29" s="42">
@@ -2030,7 +2034,7 @@
     <row r="30">
       <c r="A30" s="41" t="inlineStr">
         <is>
-          <t>Gross margin % – year 1</t>
+          <t>Gross margin % - year 1</t>
         </is>
       </c>
       <c r="C30" s="43">
@@ -2049,7 +2053,7 @@
     <row r="31">
       <c r="A31" s="41" t="inlineStr">
         <is>
-          <t>Gross margin % – year 2</t>
+          <t>Gross margin % - year 2</t>
         </is>
       </c>
       <c r="C31" s="43">
@@ -2068,7 +2072,7 @@
     <row r="32">
       <c r="A32" s="41" t="inlineStr">
         <is>
-          <t>Gross margin % – year 3</t>
+          <t>Gross margin % - year 3</t>
         </is>
       </c>
       <c r="C32" s="43">
@@ -2087,7 +2091,7 @@
     <row r="33">
       <c r="A33" s="41" t="inlineStr">
         <is>
-          <t>Gross margin % – year 4</t>
+          <t>Gross margin % - year 4</t>
         </is>
       </c>
       <c r="C33" s="43">
@@ -2106,7 +2110,7 @@
     <row r="34">
       <c r="A34" s="41" t="inlineStr">
         <is>
-          <t>Gross margin % – year 5</t>
+          <t>Gross margin % - year 5</t>
         </is>
       </c>
       <c r="C34" s="43">
@@ -2125,7 +2129,7 @@
     <row r="35">
       <c r="A35" s="41" t="inlineStr">
         <is>
-          <t>Cost of goods sold (COGS) – year 1</t>
+          <t>Cost of goods sold (COGS) - year 1</t>
         </is>
       </c>
       <c r="C35" s="42">
@@ -2144,7 +2148,7 @@
     <row r="36">
       <c r="A36" s="41" t="inlineStr">
         <is>
-          <t>Cost of goods sold (COGS) – year 2</t>
+          <t>Cost of goods sold (COGS) - year 2</t>
         </is>
       </c>
       <c r="C36" s="42">
@@ -2163,7 +2167,7 @@
     <row r="37">
       <c r="A37" s="41" t="inlineStr">
         <is>
-          <t>Cost of goods sold (COGS) – year 3</t>
+          <t>Cost of goods sold (COGS) - year 3</t>
         </is>
       </c>
       <c r="C37" s="42">
@@ -2182,7 +2186,7 @@
     <row r="38">
       <c r="A38" s="41" t="inlineStr">
         <is>
-          <t>Cost of goods sold (COGS) – year 4</t>
+          <t>Cost of goods sold (COGS) - year 4</t>
         </is>
       </c>
       <c r="C38" s="42">
@@ -2201,7 +2205,7 @@
     <row r="39">
       <c r="A39" s="41" t="inlineStr">
         <is>
-          <t>Cost of goods sold (COGS) – year 5</t>
+          <t>Cost of goods sold (COGS) - year 5</t>
         </is>
       </c>
       <c r="C39" s="42">
@@ -2220,7 +2224,7 @@
     <row r="40">
       <c r="A40" s="41" t="inlineStr">
         <is>
-          <t>Clean EBIT margin – year 1</t>
+          <t>Clean EBIT margin - year 1</t>
         </is>
       </c>
       <c r="C40" s="43">
@@ -2239,7 +2243,7 @@
     <row r="41">
       <c r="A41" s="41" t="inlineStr">
         <is>
-          <t>Clean EBIT margin – year 2</t>
+          <t>Clean EBIT margin - year 2</t>
         </is>
       </c>
       <c r="C41" s="43">
@@ -2258,7 +2262,7 @@
     <row r="42">
       <c r="A42" s="41" t="inlineStr">
         <is>
-          <t>Clean EBIT margin – year 3</t>
+          <t>Clean EBIT margin - year 3</t>
         </is>
       </c>
       <c r="C42" s="43">
@@ -2277,7 +2281,7 @@
     <row r="43">
       <c r="A43" s="41" t="inlineStr">
         <is>
-          <t>Clean EBIT margin – year 4</t>
+          <t>Clean EBIT margin - year 4</t>
         </is>
       </c>
       <c r="C43" s="43">
@@ -2296,7 +2300,7 @@
     <row r="44">
       <c r="A44" s="41" t="inlineStr">
         <is>
-          <t>Clean EBIT margin – year 5</t>
+          <t>Clean EBIT margin - year 5</t>
         </is>
       </c>
       <c r="C44" s="43">
@@ -2315,7 +2319,7 @@
     <row r="45">
       <c r="A45" s="41" t="inlineStr">
         <is>
-          <t>EBIT – year 1</t>
+          <t>EBIT - year 1</t>
         </is>
       </c>
       <c r="C45" s="42">
@@ -2334,7 +2338,7 @@
     <row r="46">
       <c r="A46" s="41" t="inlineStr">
         <is>
-          <t>EBIT – year 2</t>
+          <t>EBIT - year 2</t>
         </is>
       </c>
       <c r="C46" s="42">
@@ -2353,7 +2357,7 @@
     <row r="47">
       <c r="A47" s="41" t="inlineStr">
         <is>
-          <t>EBIT – year 3</t>
+          <t>EBIT - year 3</t>
         </is>
       </c>
       <c r="C47" s="42">
@@ -2372,7 +2376,7 @@
     <row r="48">
       <c r="A48" s="41" t="inlineStr">
         <is>
-          <t>EBIT – year 4</t>
+          <t>EBIT - year 4</t>
         </is>
       </c>
       <c r="C48" s="42">
@@ -2391,7 +2395,7 @@
     <row r="49">
       <c r="A49" s="41" t="inlineStr">
         <is>
-          <t>EBIT – year 5</t>
+          <t>EBIT - year 5</t>
         </is>
       </c>
       <c r="C49" s="42">
@@ -2410,7 +2414,7 @@
     <row r="50">
       <c r="A50" s="41" t="inlineStr">
         <is>
-          <t>NOPAT – year 1</t>
+          <t>NOPAT - year 1</t>
         </is>
       </c>
       <c r="C50" s="42">
@@ -2429,7 +2433,7 @@
     <row r="51">
       <c r="A51" s="41" t="inlineStr">
         <is>
-          <t>NOPAT – year 2</t>
+          <t>NOPAT - year 2</t>
         </is>
       </c>
       <c r="C51" s="42">
@@ -2448,7 +2452,7 @@
     <row r="52">
       <c r="A52" s="41" t="inlineStr">
         <is>
-          <t>NOPAT – year 3</t>
+          <t>NOPAT - year 3</t>
         </is>
       </c>
       <c r="C52" s="42">
@@ -2467,7 +2471,7 @@
     <row r="53">
       <c r="A53" s="41" t="inlineStr">
         <is>
-          <t>NOPAT – year 4</t>
+          <t>NOPAT - year 4</t>
         </is>
       </c>
       <c r="C53" s="42">
@@ -2486,7 +2490,7 @@
     <row r="54">
       <c r="A54" s="41" t="inlineStr">
         <is>
-          <t>NOPAT – year 5</t>
+          <t>NOPAT - year 5</t>
         </is>
       </c>
       <c r="C54" s="42">
@@ -2505,7 +2509,7 @@
     <row r="55">
       <c r="A55" s="41" t="inlineStr">
         <is>
-          <t>D&amp;A – year 1</t>
+          <t>D&amp;A - year 1</t>
         </is>
       </c>
       <c r="C55" s="42">
@@ -2524,7 +2528,7 @@
     <row r="56">
       <c r="A56" s="41" t="inlineStr">
         <is>
-          <t>D&amp;A – year 2</t>
+          <t>D&amp;A - year 2</t>
         </is>
       </c>
       <c r="C56" s="42">
@@ -2543,7 +2547,7 @@
     <row r="57">
       <c r="A57" s="41" t="inlineStr">
         <is>
-          <t>D&amp;A – year 3</t>
+          <t>D&amp;A - year 3</t>
         </is>
       </c>
       <c r="C57" s="42">
@@ -2562,7 +2566,7 @@
     <row r="58">
       <c r="A58" s="41" t="inlineStr">
         <is>
-          <t>D&amp;A – year 4</t>
+          <t>D&amp;A - year 4</t>
         </is>
       </c>
       <c r="C58" s="42">
@@ -2581,7 +2585,7 @@
     <row r="59">
       <c r="A59" s="41" t="inlineStr">
         <is>
-          <t>D&amp;A – year 5</t>
+          <t>D&amp;A - year 5</t>
         </is>
       </c>
       <c r="C59" s="42">
@@ -2600,7 +2604,7 @@
     <row r="60">
       <c r="A60" s="41" t="inlineStr">
         <is>
-          <t>Capex – year 1</t>
+          <t>Capex - year 1</t>
         </is>
       </c>
       <c r="C60" s="42">
@@ -2619,7 +2623,7 @@
     <row r="61">
       <c r="A61" s="41" t="inlineStr">
         <is>
-          <t>Capex – year 2</t>
+          <t>Capex - year 2</t>
         </is>
       </c>
       <c r="C61" s="42">
@@ -2638,7 +2642,7 @@
     <row r="62">
       <c r="A62" s="41" t="inlineStr">
         <is>
-          <t>Capex – year 3</t>
+          <t>Capex - year 3</t>
         </is>
       </c>
       <c r="C62" s="42">
@@ -2657,7 +2661,7 @@
     <row r="63">
       <c r="A63" s="41" t="inlineStr">
         <is>
-          <t>Capex – year 4</t>
+          <t>Capex - year 4</t>
         </is>
       </c>
       <c r="C63" s="42">
@@ -2676,7 +2680,7 @@
     <row r="64">
       <c r="A64" s="41" t="inlineStr">
         <is>
-          <t>Capex – year 5</t>
+          <t>Capex - year 5</t>
         </is>
       </c>
       <c r="C64" s="42">
@@ -2695,7 +2699,7 @@
     <row r="65">
       <c r="A65" s="41" t="inlineStr">
         <is>
-          <t>DSO (days) – year 1</t>
+          <t>DSO (days) - year 1</t>
         </is>
       </c>
       <c r="C65" s="44">
@@ -2714,7 +2718,7 @@
     <row r="66">
       <c r="A66" s="41" t="inlineStr">
         <is>
-          <t>DSO (days) – year 2</t>
+          <t>DSO (days) - year 2</t>
         </is>
       </c>
       <c r="C66" s="44">
@@ -2733,7 +2737,7 @@
     <row r="67">
       <c r="A67" s="41" t="inlineStr">
         <is>
-          <t>DSO (days) – year 3</t>
+          <t>DSO (days) - year 3</t>
         </is>
       </c>
       <c r="C67" s="44">
@@ -2752,7 +2756,7 @@
     <row r="68">
       <c r="A68" s="41" t="inlineStr">
         <is>
-          <t>DSO (days) – year 4</t>
+          <t>DSO (days) - year 4</t>
         </is>
       </c>
       <c r="C68" s="44">
@@ -2771,7 +2775,7 @@
     <row r="69">
       <c r="A69" s="41" t="inlineStr">
         <is>
-          <t>DSO (days) – year 5</t>
+          <t>DSO (days) - year 5</t>
         </is>
       </c>
       <c r="C69" s="44">
@@ -2790,7 +2794,7 @@
     <row r="70">
       <c r="A70" s="41" t="inlineStr">
         <is>
-          <t>Accounts receivable – year 1</t>
+          <t>Accounts receivable - year 1</t>
         </is>
       </c>
       <c r="C70" s="42">
@@ -2809,7 +2813,7 @@
     <row r="71">
       <c r="A71" s="41" t="inlineStr">
         <is>
-          <t>Accounts receivable – year 2</t>
+          <t>Accounts receivable - year 2</t>
         </is>
       </c>
       <c r="C71" s="42">
@@ -2828,7 +2832,7 @@
     <row r="72">
       <c r="A72" s="41" t="inlineStr">
         <is>
-          <t>Accounts receivable – year 3</t>
+          <t>Accounts receivable - year 3</t>
         </is>
       </c>
       <c r="C72" s="42">
@@ -2847,7 +2851,7 @@
     <row r="73">
       <c r="A73" s="41" t="inlineStr">
         <is>
-          <t>Accounts receivable – year 4</t>
+          <t>Accounts receivable - year 4</t>
         </is>
       </c>
       <c r="C73" s="42">
@@ -2866,7 +2870,7 @@
     <row r="74">
       <c r="A74" s="41" t="inlineStr">
         <is>
-          <t>Accounts receivable – year 5</t>
+          <t>Accounts receivable - year 5</t>
         </is>
       </c>
       <c r="C74" s="42">
@@ -2885,7 +2889,7 @@
     <row r="75">
       <c r="A75" s="41" t="inlineStr">
         <is>
-          <t>DIO (days) – year 1</t>
+          <t>DIO (days) - year 1</t>
         </is>
       </c>
       <c r="C75" s="44">
@@ -2904,7 +2908,7 @@
     <row r="76">
       <c r="A76" s="41" t="inlineStr">
         <is>
-          <t>DIO (days) – year 2</t>
+          <t>DIO (days) - year 2</t>
         </is>
       </c>
       <c r="C76" s="44">
@@ -2923,7 +2927,7 @@
     <row r="77">
       <c r="A77" s="41" t="inlineStr">
         <is>
-          <t>DIO (days) – year 3</t>
+          <t>DIO (days) - year 3</t>
         </is>
       </c>
       <c r="C77" s="44">
@@ -2942,7 +2946,7 @@
     <row r="78">
       <c r="A78" s="41" t="inlineStr">
         <is>
-          <t>DIO (days) – year 4</t>
+          <t>DIO (days) - year 4</t>
         </is>
       </c>
       <c r="C78" s="44">
@@ -2961,7 +2965,7 @@
     <row r="79">
       <c r="A79" s="41" t="inlineStr">
         <is>
-          <t>DIO (days) – year 5</t>
+          <t>DIO (days) - year 5</t>
         </is>
       </c>
       <c r="C79" s="44">
@@ -2980,7 +2984,7 @@
     <row r="80">
       <c r="A80" s="41" t="inlineStr">
         <is>
-          <t>Inventories – year 1</t>
+          <t>Inventories - year 1</t>
         </is>
       </c>
       <c r="C80" s="42">
@@ -2999,7 +3003,7 @@
     <row r="81">
       <c r="A81" s="41" t="inlineStr">
         <is>
-          <t>Inventories – year 2</t>
+          <t>Inventories - year 2</t>
         </is>
       </c>
       <c r="C81" s="42">
@@ -3018,7 +3022,7 @@
     <row r="82">
       <c r="A82" s="41" t="inlineStr">
         <is>
-          <t>Inventories – year 3</t>
+          <t>Inventories - year 3</t>
         </is>
       </c>
       <c r="C82" s="42">
@@ -3037,7 +3041,7 @@
     <row r="83">
       <c r="A83" s="41" t="inlineStr">
         <is>
-          <t>Inventories – year 4</t>
+          <t>Inventories - year 4</t>
         </is>
       </c>
       <c r="C83" s="42">
@@ -3056,7 +3060,7 @@
     <row r="84">
       <c r="A84" s="41" t="inlineStr">
         <is>
-          <t>Inventories – year 5</t>
+          <t>Inventories - year 5</t>
         </is>
       </c>
       <c r="C84" s="42">
@@ -3075,7 +3079,7 @@
     <row r="85">
       <c r="A85" s="41" t="inlineStr">
         <is>
-          <t>DPO (days) – year 1</t>
+          <t>DPO (days) - year 1</t>
         </is>
       </c>
       <c r="C85" s="44">
@@ -3094,7 +3098,7 @@
     <row r="86">
       <c r="A86" s="41" t="inlineStr">
         <is>
-          <t>DPO (days) – year 2</t>
+          <t>DPO (days) - year 2</t>
         </is>
       </c>
       <c r="C86" s="44">
@@ -3113,7 +3117,7 @@
     <row r="87">
       <c r="A87" s="41" t="inlineStr">
         <is>
-          <t>DPO (days) – year 3</t>
+          <t>DPO (days) - year 3</t>
         </is>
       </c>
       <c r="C87" s="44">
@@ -3132,7 +3136,7 @@
     <row r="88">
       <c r="A88" s="41" t="inlineStr">
         <is>
-          <t>DPO (days) – year 4</t>
+          <t>DPO (days) - year 4</t>
         </is>
       </c>
       <c r="C88" s="44">
@@ -3151,7 +3155,7 @@
     <row r="89">
       <c r="A89" s="41" t="inlineStr">
         <is>
-          <t>DPO (days) – year 5</t>
+          <t>DPO (days) - year 5</t>
         </is>
       </c>
       <c r="C89" s="44">
@@ -3170,7 +3174,7 @@
     <row r="90">
       <c r="A90" s="41" t="inlineStr">
         <is>
-          <t>Accounts payable – year 1</t>
+          <t>Accounts payable - year 1</t>
         </is>
       </c>
       <c r="C90" s="42">
@@ -3189,7 +3193,7 @@
     <row r="91">
       <c r="A91" s="41" t="inlineStr">
         <is>
-          <t>Accounts payable – year 2</t>
+          <t>Accounts payable - year 2</t>
         </is>
       </c>
       <c r="C91" s="42">
@@ -3208,7 +3212,7 @@
     <row r="92">
       <c r="A92" s="41" t="inlineStr">
         <is>
-          <t>Accounts payable – year 3</t>
+          <t>Accounts payable - year 3</t>
         </is>
       </c>
       <c r="C92" s="42">
@@ -3227,7 +3231,7 @@
     <row r="93">
       <c r="A93" s="41" t="inlineStr">
         <is>
-          <t>Accounts payable – year 4</t>
+          <t>Accounts payable - year 4</t>
         </is>
       </c>
       <c r="C93" s="42">
@@ -3246,7 +3250,7 @@
     <row r="94">
       <c r="A94" s="41" t="inlineStr">
         <is>
-          <t>Accounts payable – year 5</t>
+          <t>Accounts payable - year 5</t>
         </is>
       </c>
       <c r="C94" s="42">
@@ -3265,7 +3269,7 @@
     <row r="95">
       <c r="A95" s="41" t="inlineStr">
         <is>
-          <t>Prepaid expenses (other current assets) – year 1</t>
+          <t>Prepaid expenses (other current assets) - year 1</t>
         </is>
       </c>
       <c r="C95" s="42">
@@ -3284,7 +3288,7 @@
     <row r="96">
       <c r="A96" s="41" t="inlineStr">
         <is>
-          <t>Prepaid expenses (other current assets) – year 2</t>
+          <t>Prepaid expenses (other current assets) - year 2</t>
         </is>
       </c>
       <c r="C96" s="42">
@@ -3303,7 +3307,7 @@
     <row r="97">
       <c r="A97" s="41" t="inlineStr">
         <is>
-          <t>Prepaid expenses (other current assets) – year 3</t>
+          <t>Prepaid expenses (other current assets) - year 3</t>
         </is>
       </c>
       <c r="C97" s="42">
@@ -3322,7 +3326,7 @@
     <row r="98">
       <c r="A98" s="41" t="inlineStr">
         <is>
-          <t>Prepaid expenses (other current assets) – year 4</t>
+          <t>Prepaid expenses (other current assets) - year 4</t>
         </is>
       </c>
       <c r="C98" s="42">
@@ -3341,7 +3345,7 @@
     <row r="99">
       <c r="A99" s="41" t="inlineStr">
         <is>
-          <t>Prepaid expenses (other current assets) – year 5</t>
+          <t>Prepaid expenses (other current assets) - year 5</t>
         </is>
       </c>
       <c r="C99" s="42">
@@ -3360,7 +3364,7 @@
     <row r="100">
       <c r="A100" s="41" t="inlineStr">
         <is>
-          <t>Accrued liabilities – year 1</t>
+          <t>Accrued liabilities - year 1</t>
         </is>
       </c>
       <c r="C100" s="42">
@@ -3379,7 +3383,7 @@
     <row r="101">
       <c r="A101" s="41" t="inlineStr">
         <is>
-          <t>Accrued liabilities – year 2</t>
+          <t>Accrued liabilities - year 2</t>
         </is>
       </c>
       <c r="C101" s="42">
@@ -3398,7 +3402,7 @@
     <row r="102">
       <c r="A102" s="41" t="inlineStr">
         <is>
-          <t>Accrued liabilities – year 3</t>
+          <t>Accrued liabilities - year 3</t>
         </is>
       </c>
       <c r="C102" s="42">
@@ -3417,7 +3421,7 @@
     <row r="103">
       <c r="A103" s="41" t="inlineStr">
         <is>
-          <t>Accrued liabilities – year 4</t>
+          <t>Accrued liabilities - year 4</t>
         </is>
       </c>
       <c r="C103" s="42">
@@ -3436,7 +3440,7 @@
     <row r="104">
       <c r="A104" s="41" t="inlineStr">
         <is>
-          <t>Accrued liabilities – year 5</t>
+          <t>Accrued liabilities - year 5</t>
         </is>
       </c>
       <c r="C104" s="42">
@@ -3455,7 +3459,7 @@
     <row r="105">
       <c r="A105" s="41" t="inlineStr">
         <is>
-          <t>Current operating assets (AR + inv + prepaids) – year 1</t>
+          <t>Current operating assets (AR + inv + prepaids) - year 1</t>
         </is>
       </c>
       <c r="C105" s="42">
@@ -3474,7 +3478,7 @@
     <row r="106">
       <c r="A106" s="41" t="inlineStr">
         <is>
-          <t>Current operating assets (AR + inv + prepaids) – year 2</t>
+          <t>Current operating assets (AR + inv + prepaids) - year 2</t>
         </is>
       </c>
       <c r="C106" s="42">
@@ -3493,7 +3497,7 @@
     <row r="107">
       <c r="A107" s="41" t="inlineStr">
         <is>
-          <t>Current operating assets (AR + inv + prepaids) – year 3</t>
+          <t>Current operating assets (AR + inv + prepaids) - year 3</t>
         </is>
       </c>
       <c r="C107" s="42">
@@ -3512,7 +3516,7 @@
     <row r="108">
       <c r="A108" s="41" t="inlineStr">
         <is>
-          <t>Current operating assets (AR + inv + prepaids) – year 4</t>
+          <t>Current operating assets (AR + inv + prepaids) - year 4</t>
         </is>
       </c>
       <c r="C108" s="42">
@@ -3531,7 +3535,7 @@
     <row r="109">
       <c r="A109" s="41" t="inlineStr">
         <is>
-          <t>Current operating assets (AR + inv + prepaids) – year 5</t>
+          <t>Current operating assets (AR + inv + prepaids) - year 5</t>
         </is>
       </c>
       <c r="C109" s="42">
@@ -3550,7 +3554,7 @@
     <row r="110">
       <c r="A110" s="41" t="inlineStr">
         <is>
-          <t>Current operating liabilities (AP + accruals) – year 1</t>
+          <t>Current operating liabilities (AP + accruals) - year 1</t>
         </is>
       </c>
       <c r="C110" s="42">
@@ -3569,7 +3573,7 @@
     <row r="111">
       <c r="A111" s="41" t="inlineStr">
         <is>
-          <t>Current operating liabilities (AP + accruals) – year 2</t>
+          <t>Current operating liabilities (AP + accruals) - year 2</t>
         </is>
       </c>
       <c r="C111" s="42">
@@ -3588,7 +3592,7 @@
     <row r="112">
       <c r="A112" s="41" t="inlineStr">
         <is>
-          <t>Current operating liabilities (AP + accruals) – year 3</t>
+          <t>Current operating liabilities (AP + accruals) - year 3</t>
         </is>
       </c>
       <c r="C112" s="42">
@@ -3607,7 +3611,7 @@
     <row r="113">
       <c r="A113" s="41" t="inlineStr">
         <is>
-          <t>Current operating liabilities (AP + accruals) – year 4</t>
+          <t>Current operating liabilities (AP + accruals) - year 4</t>
         </is>
       </c>
       <c r="C113" s="42">
@@ -3626,7 +3630,7 @@
     <row r="114">
       <c r="A114" s="41" t="inlineStr">
         <is>
-          <t>Current operating liabilities (AP + accruals) – year 5</t>
+          <t>Current operating liabilities (AP + accruals) - year 5</t>
         </is>
       </c>
       <c r="C114" s="42">
@@ -3645,7 +3649,7 @@
     <row r="115">
       <c r="A115" s="41" t="inlineStr">
         <is>
-          <t>Net working capital – year 1</t>
+          <t>Net working capital - year 1</t>
         </is>
       </c>
       <c r="C115" s="42">
@@ -3664,7 +3668,7 @@
     <row r="116">
       <c r="A116" s="41" t="inlineStr">
         <is>
-          <t>Net working capital – year 2</t>
+          <t>Net working capital - year 2</t>
         </is>
       </c>
       <c r="C116" s="42">
@@ -3683,7 +3687,7 @@
     <row r="117">
       <c r="A117" s="41" t="inlineStr">
         <is>
-          <t>Net working capital – year 3</t>
+          <t>Net working capital - year 3</t>
         </is>
       </c>
       <c r="C117" s="42">
@@ -3702,7 +3706,7 @@
     <row r="118">
       <c r="A118" s="41" t="inlineStr">
         <is>
-          <t>Net working capital – year 4</t>
+          <t>Net working capital - year 4</t>
         </is>
       </c>
       <c r="C118" s="42">
@@ -3721,7 +3725,7 @@
     <row r="119">
       <c r="A119" s="41" t="inlineStr">
         <is>
-          <t>Net working capital – year 5</t>
+          <t>Net working capital - year 5</t>
         </is>
       </c>
       <c r="C119" s="42">
@@ -3740,7 +3744,7 @@
     <row r="120">
       <c r="A120" s="41" t="inlineStr">
         <is>
-          <t>ΔNWC (prior yr − current yr) – year 1</t>
+          <t>Delta NWC (prior yr - current yr) - year 1</t>
         </is>
       </c>
       <c r="C120" s="42">
@@ -3759,7 +3763,7 @@
     <row r="121">
       <c r="A121" s="41" t="inlineStr">
         <is>
-          <t>ΔNWC (prior yr − current yr) – year 2</t>
+          <t>Delta NWC (prior yr - current yr) - year 2</t>
         </is>
       </c>
       <c r="C121" s="42">
@@ -3778,7 +3782,7 @@
     <row r="122">
       <c r="A122" s="41" t="inlineStr">
         <is>
-          <t>ΔNWC (prior yr − current yr) – year 3</t>
+          <t>Delta NWC (prior yr - current yr) - year 3</t>
         </is>
       </c>
       <c r="C122" s="42">
@@ -3797,7 +3801,7 @@
     <row r="123">
       <c r="A123" s="41" t="inlineStr">
         <is>
-          <t>ΔNWC (prior yr − current yr) – year 4</t>
+          <t>Delta NWC (prior yr - current yr) - year 4</t>
         </is>
       </c>
       <c r="C123" s="42">
@@ -3816,7 +3820,7 @@
     <row r="124">
       <c r="A124" s="41" t="inlineStr">
         <is>
-          <t>ΔNWC (prior yr − current yr) – year 5</t>
+          <t>Delta NWC (prior yr - current yr) - year 5</t>
         </is>
       </c>
       <c r="C124" s="42">
@@ -3835,7 +3839,7 @@
     <row r="125">
       <c r="A125" s="41" t="inlineStr">
         <is>
-          <t>Unlevered FCF – year 1</t>
+          <t>Unlevered FCF - year 1</t>
         </is>
       </c>
       <c r="C125" s="42">
@@ -3854,7 +3858,7 @@
     <row r="126">
       <c r="A126" s="41" t="inlineStr">
         <is>
-          <t>Unlevered FCF – year 2</t>
+          <t>Unlevered FCF - year 2</t>
         </is>
       </c>
       <c r="C126" s="42">
@@ -3873,7 +3877,7 @@
     <row r="127">
       <c r="A127" s="41" t="inlineStr">
         <is>
-          <t>Unlevered FCF – year 3</t>
+          <t>Unlevered FCF - year 3</t>
         </is>
       </c>
       <c r="C127" s="42">
@@ -3892,7 +3896,7 @@
     <row r="128">
       <c r="A128" s="41" t="inlineStr">
         <is>
-          <t>Unlevered FCF – year 4</t>
+          <t>Unlevered FCF - year 4</t>
         </is>
       </c>
       <c r="C128" s="42">
@@ -3911,7 +3915,7 @@
     <row r="129">
       <c r="A129" s="41" t="inlineStr">
         <is>
-          <t>Unlevered FCF – year 5</t>
+          <t>Unlevered FCF - year 5</t>
         </is>
       </c>
       <c r="C129" s="42">
@@ -4004,7 +4008,7 @@
     <row r="138">
       <c r="A138" s="41" t="inlineStr">
         <is>
-          <t>Other income – year 1</t>
+          <t>Other income - year 1</t>
         </is>
       </c>
       <c r="C138" s="42" t="n">
@@ -4020,7 +4024,7 @@
     <row r="139">
       <c r="A139" s="41" t="inlineStr">
         <is>
-          <t>Other income – year 2</t>
+          <t>Other income - year 2</t>
         </is>
       </c>
       <c r="C139" s="42" t="n">
@@ -4036,7 +4040,7 @@
     <row r="140">
       <c r="A140" s="41" t="inlineStr">
         <is>
-          <t>Other income – year 3</t>
+          <t>Other income - year 3</t>
         </is>
       </c>
       <c r="C140" s="42" t="n">
@@ -4052,7 +4056,7 @@
     <row r="141">
       <c r="A141" s="41" t="inlineStr">
         <is>
-          <t>Other income – year 4</t>
+          <t>Other income - year 4</t>
         </is>
       </c>
       <c r="C141" s="42" t="n">
@@ -4068,7 +4072,7 @@
     <row r="142">
       <c r="A142" s="41" t="inlineStr">
         <is>
-          <t>Other income – year 5</t>
+          <t>Other income - year 5</t>
         </is>
       </c>
       <c r="C142" s="42" t="n">
@@ -4084,7 +4088,7 @@
     <row r="143">
       <c r="A143" s="41" t="inlineStr">
         <is>
-          <t>Net income – year 1</t>
+          <t>Net income - year 1</t>
         </is>
       </c>
       <c r="C143" s="42">
@@ -4103,7 +4107,7 @@
     <row r="144">
       <c r="A144" s="41" t="inlineStr">
         <is>
-          <t>Net income – year 2</t>
+          <t>Net income - year 2</t>
         </is>
       </c>
       <c r="C144" s="42">
@@ -4122,7 +4126,7 @@
     <row r="145">
       <c r="A145" s="41" t="inlineStr">
         <is>
-          <t>Net income – year 3</t>
+          <t>Net income - year 3</t>
         </is>
       </c>
       <c r="C145" s="42">
@@ -4141,7 +4145,7 @@
     <row r="146">
       <c r="A146" s="41" t="inlineStr">
         <is>
-          <t>Net income – year 4</t>
+          <t>Net income - year 4</t>
         </is>
       </c>
       <c r="C146" s="42">
@@ -4160,7 +4164,7 @@
     <row r="147">
       <c r="A147" s="41" t="inlineStr">
         <is>
-          <t>Net income – year 5</t>
+          <t>Net income - year 5</t>
         </is>
       </c>
       <c r="C147" s="42">
@@ -4179,7 +4183,7 @@
     <row r="148">
       <c r="A148" s="41" t="inlineStr">
         <is>
-          <t>Cash from operations – year 1</t>
+          <t>Cash from operations - year 1</t>
         </is>
       </c>
       <c r="C148" s="42">
@@ -4198,7 +4202,7 @@
     <row r="149">
       <c r="A149" s="41" t="inlineStr">
         <is>
-          <t>Cash from operations – year 2</t>
+          <t>Cash from operations - year 2</t>
         </is>
       </c>
       <c r="C149" s="42">
@@ -4217,7 +4221,7 @@
     <row r="150">
       <c r="A150" s="41" t="inlineStr">
         <is>
-          <t>Cash from operations – year 3</t>
+          <t>Cash from operations - year 3</t>
         </is>
       </c>
       <c r="C150" s="42">
@@ -4236,7 +4240,7 @@
     <row r="151">
       <c r="A151" s="41" t="inlineStr">
         <is>
-          <t>Cash from operations – year 4</t>
+          <t>Cash from operations - year 4</t>
         </is>
       </c>
       <c r="C151" s="42">
@@ -4255,7 +4259,7 @@
     <row r="152">
       <c r="A152" s="41" t="inlineStr">
         <is>
-          <t>Cash from operations – year 5</t>
+          <t>Cash from operations - year 5</t>
         </is>
       </c>
       <c r="C152" s="42">
@@ -4274,7 +4278,7 @@
     <row r="153">
       <c r="A153" s="41" t="inlineStr">
         <is>
-          <t>Free cash flow (CFS) – year 1</t>
+          <t>Free cash flow (CFS) - year 1</t>
         </is>
       </c>
       <c r="C153" s="42">
@@ -4293,7 +4297,7 @@
     <row r="154">
       <c r="A154" s="41" t="inlineStr">
         <is>
-          <t>Free cash flow (CFS) – year 2</t>
+          <t>Free cash flow (CFS) - year 2</t>
         </is>
       </c>
       <c r="C154" s="42">
@@ -4312,7 +4316,7 @@
     <row r="155">
       <c r="A155" s="41" t="inlineStr">
         <is>
-          <t>Free cash flow (CFS) – year 3</t>
+          <t>Free cash flow (CFS) - year 3</t>
         </is>
       </c>
       <c r="C155" s="42">
@@ -4331,7 +4335,7 @@
     <row r="156">
       <c r="A156" s="41" t="inlineStr">
         <is>
-          <t>Free cash flow (CFS) – year 4</t>
+          <t>Free cash flow (CFS) - year 4</t>
         </is>
       </c>
       <c r="C156" s="42">
@@ -4350,7 +4354,7 @@
     <row r="157">
       <c r="A157" s="41" t="inlineStr">
         <is>
-          <t>Free cash flow (CFS) – year 5</t>
+          <t>Free cash flow (CFS) - year 5</t>
         </is>
       </c>
       <c r="C157" s="42">
@@ -4369,7 +4373,7 @@
     <row r="158">
       <c r="A158" s="41" t="inlineStr">
         <is>
-          <t>Share repurchases – year 1</t>
+          <t>Share repurchases - year 1</t>
         </is>
       </c>
       <c r="C158" s="42">
@@ -4388,7 +4392,7 @@
     <row r="159">
       <c r="A159" s="41" t="inlineStr">
         <is>
-          <t>Share repurchases – year 2</t>
+          <t>Share repurchases - year 2</t>
         </is>
       </c>
       <c r="C159" s="42">
@@ -4407,7 +4411,7 @@
     <row r="160">
       <c r="A160" s="41" t="inlineStr">
         <is>
-          <t>Share repurchases – year 3</t>
+          <t>Share repurchases - year 3</t>
         </is>
       </c>
       <c r="C160" s="42">
@@ -4426,7 +4430,7 @@
     <row r="161">
       <c r="A161" s="41" t="inlineStr">
         <is>
-          <t>Share repurchases – year 4</t>
+          <t>Share repurchases - year 4</t>
         </is>
       </c>
       <c r="C161" s="42">
@@ -4445,7 +4449,7 @@
     <row r="162">
       <c r="A162" s="41" t="inlineStr">
         <is>
-          <t>Share repurchases – year 5</t>
+          <t>Share repurchases - year 5</t>
         </is>
       </c>
       <c r="C162" s="42">
@@ -4464,7 +4468,7 @@
     <row r="163">
       <c r="A163" s="41" t="inlineStr">
         <is>
-          <t>Cash &amp; equivalents – year 1</t>
+          <t>Cash &amp; equivalents - year 1</t>
         </is>
       </c>
       <c r="C163" s="42">
@@ -4483,7 +4487,7 @@
     <row r="164">
       <c r="A164" s="41" t="inlineStr">
         <is>
-          <t>Cash &amp; equivalents – year 2</t>
+          <t>Cash &amp; equivalents - year 2</t>
         </is>
       </c>
       <c r="C164" s="42">
@@ -4502,7 +4506,7 @@
     <row r="165">
       <c r="A165" s="41" t="inlineStr">
         <is>
-          <t>Cash &amp; equivalents – year 3</t>
+          <t>Cash &amp; equivalents - year 3</t>
         </is>
       </c>
       <c r="C165" s="42">
@@ -4521,7 +4525,7 @@
     <row r="166">
       <c r="A166" s="41" t="inlineStr">
         <is>
-          <t>Cash &amp; equivalents – year 4</t>
+          <t>Cash &amp; equivalents - year 4</t>
         </is>
       </c>
       <c r="C166" s="42">
@@ -4540,7 +4544,7 @@
     <row r="167">
       <c r="A167" s="41" t="inlineStr">
         <is>
-          <t>Cash &amp; equivalents – year 5</t>
+          <t>Cash &amp; equivalents - year 5</t>
         </is>
       </c>
       <c r="C167" s="42">
@@ -4559,7 +4563,7 @@
     <row r="168">
       <c r="A168" s="41" t="inlineStr">
         <is>
-          <t>Total assets – year 1</t>
+          <t>Total assets - year 1</t>
         </is>
       </c>
       <c r="C168" s="42">
@@ -4578,7 +4582,7 @@
     <row r="169">
       <c r="A169" s="41" t="inlineStr">
         <is>
-          <t>Total assets – year 2</t>
+          <t>Total assets - year 2</t>
         </is>
       </c>
       <c r="C169" s="42">
@@ -4597,7 +4601,7 @@
     <row r="170">
       <c r="A170" s="41" t="inlineStr">
         <is>
-          <t>Total assets – year 3</t>
+          <t>Total assets - year 3</t>
         </is>
       </c>
       <c r="C170" s="42">
@@ -4616,7 +4620,7 @@
     <row r="171">
       <c r="A171" s="41" t="inlineStr">
         <is>
-          <t>Total assets – year 4</t>
+          <t>Total assets - year 4</t>
         </is>
       </c>
       <c r="C171" s="42">
@@ -4635,7 +4639,7 @@
     <row r="172">
       <c r="A172" s="41" t="inlineStr">
         <is>
-          <t>Total assets – year 5</t>
+          <t>Total assets - year 5</t>
         </is>
       </c>
       <c r="C172" s="42">
@@ -4654,7 +4658,7 @@
     <row r="173">
       <c r="A173" s="41" t="inlineStr">
         <is>
-          <t>Total liabilities – year 1</t>
+          <t>Total liabilities - year 1</t>
         </is>
       </c>
       <c r="C173" s="42">
@@ -4673,7 +4677,7 @@
     <row r="174">
       <c r="A174" s="41" t="inlineStr">
         <is>
-          <t>Total liabilities – year 2</t>
+          <t>Total liabilities - year 2</t>
         </is>
       </c>
       <c r="C174" s="42">
@@ -4692,7 +4696,7 @@
     <row r="175">
       <c r="A175" s="41" t="inlineStr">
         <is>
-          <t>Total liabilities – year 3</t>
+          <t>Total liabilities - year 3</t>
         </is>
       </c>
       <c r="C175" s="42">
@@ -4711,7 +4715,7 @@
     <row r="176">
       <c r="A176" s="41" t="inlineStr">
         <is>
-          <t>Total liabilities – year 4</t>
+          <t>Total liabilities - year 4</t>
         </is>
       </c>
       <c r="C176" s="42">
@@ -4730,7 +4734,7 @@
     <row r="177">
       <c r="A177" s="41" t="inlineStr">
         <is>
-          <t>Total liabilities – year 5</t>
+          <t>Total liabilities - year 5</t>
         </is>
       </c>
       <c r="C177" s="42">
@@ -4749,7 +4753,7 @@
     <row r="178">
       <c r="A178" s="41" t="inlineStr">
         <is>
-          <t>Total equity – year 1</t>
+          <t>Total equity - year 1</t>
         </is>
       </c>
       <c r="C178" s="42">
@@ -4768,7 +4772,7 @@
     <row r="179">
       <c r="A179" s="41" t="inlineStr">
         <is>
-          <t>Total equity – year 2</t>
+          <t>Total equity - year 2</t>
         </is>
       </c>
       <c r="C179" s="42">
@@ -4787,7 +4791,7 @@
     <row r="180">
       <c r="A180" s="41" t="inlineStr">
         <is>
-          <t>Total equity – year 3</t>
+          <t>Total equity - year 3</t>
         </is>
       </c>
       <c r="C180" s="42">
@@ -4806,7 +4810,7 @@
     <row r="181">
       <c r="A181" s="41" t="inlineStr">
         <is>
-          <t>Total equity – year 4</t>
+          <t>Total equity - year 4</t>
         </is>
       </c>
       <c r="C181" s="42">
@@ -4825,7 +4829,7 @@
     <row r="182">
       <c r="A182" s="41" t="inlineStr">
         <is>
-          <t>Total equity – year 5</t>
+          <t>Total equity - year 5</t>
         </is>
       </c>
       <c r="C182" s="42">
@@ -4844,7 +4848,7 @@
     <row r="183">
       <c r="A183" s="41" t="inlineStr">
         <is>
-          <t>Diluted shares (000) – year 1</t>
+          <t>Diluted shares (000) - year 1</t>
         </is>
       </c>
       <c r="C183" s="42">
@@ -4863,7 +4867,7 @@
     <row r="184">
       <c r="A184" s="41" t="inlineStr">
         <is>
-          <t>Diluted shares (000) – year 2</t>
+          <t>Diluted shares (000) - year 2</t>
         </is>
       </c>
       <c r="C184" s="42">
@@ -4882,7 +4886,7 @@
     <row r="185">
       <c r="A185" s="41" t="inlineStr">
         <is>
-          <t>Diluted shares (000) – year 3</t>
+          <t>Diluted shares (000) - year 3</t>
         </is>
       </c>
       <c r="C185" s="42">
@@ -4901,7 +4905,7 @@
     <row r="186">
       <c r="A186" s="41" t="inlineStr">
         <is>
-          <t>Diluted shares (000) – year 4</t>
+          <t>Diluted shares (000) - year 4</t>
         </is>
       </c>
       <c r="C186" s="42">
@@ -4920,7 +4924,7 @@
     <row r="187">
       <c r="A187" s="41" t="inlineStr">
         <is>
-          <t>Diluted shares (000) – year 5</t>
+          <t>Diluted shares (000) - year 5</t>
         </is>
       </c>
       <c r="C187" s="42">
@@ -4939,7 +4943,7 @@
     <row r="188">
       <c r="A188" s="41" t="inlineStr">
         <is>
-          <t>Diluted EPS ($) – year 1</t>
+          <t>Diluted EPS ($) - year 1</t>
         </is>
       </c>
       <c r="C188" s="49">
@@ -4958,7 +4962,7 @@
     <row r="189">
       <c r="A189" s="41" t="inlineStr">
         <is>
-          <t>Diluted EPS ($) – year 2</t>
+          <t>Diluted EPS ($) - year 2</t>
         </is>
       </c>
       <c r="C189" s="49">
@@ -4977,7 +4981,7 @@
     <row r="190">
       <c r="A190" s="41" t="inlineStr">
         <is>
-          <t>Diluted EPS ($) – year 3</t>
+          <t>Diluted EPS ($) - year 3</t>
         </is>
       </c>
       <c r="C190" s="49">
@@ -4996,7 +5000,7 @@
     <row r="191">
       <c r="A191" s="41" t="inlineStr">
         <is>
-          <t>Diluted EPS ($) – year 4</t>
+          <t>Diluted EPS ($) - year 4</t>
         </is>
       </c>
       <c r="C191" s="49">
@@ -5015,7 +5019,7 @@
     <row r="192">
       <c r="A192" s="41" t="inlineStr">
         <is>
-          <t>Diluted EPS ($) – year 5</t>
+          <t>Diluted EPS ($) - year 5</t>
         </is>
       </c>
       <c r="C192" s="49">
@@ -5069,7 +5073,7 @@
     <row r="1">
       <c r="A1" s="50" t="inlineStr">
         <is>
-          <t>BOTTOM-UP REVENUE DRIVER SCHEDULE (FY2026E–FY2030E)</t>
+          <t>BOTTOM-UP REVENUE DRIVER SCHEDULE (FY2026E-FY2030E)</t>
         </is>
       </c>
       <c r="B1" s="13" t="n"/>
@@ -5083,7 +5087,7 @@
     <row r="2">
       <c r="A2" s="26" t="inlineStr">
         <is>
-          <t>FY2025A = FY25 10-K historical anchors (blue). FY26–30 = red operational assumptions. Consolidated revenue cross-checks to Scenarios base case.</t>
+          <t>FY2025A = FY25 10-K historical anchors (blue). FY26-30 = red operational assumptions. Consolidated revenue cross-checks to Scenarios base case.</t>
         </is>
       </c>
     </row>
@@ -5140,7 +5144,7 @@
     <row r="6" ht="28" customHeight="1">
       <c r="A6" s="41" t="inlineStr">
         <is>
-          <t>Americas — beginning stores</t>
+          <t>Americas - beginning stores</t>
         </is>
       </c>
       <c r="B6" s="57" t="n">
@@ -5175,7 +5179,7 @@
     <row r="7" ht="28" customHeight="1">
       <c r="A7" s="41" t="inlineStr">
         <is>
-          <t>Americas — openings</t>
+          <t>Americas - openings</t>
         </is>
       </c>
       <c r="C7" s="60" t="n">
@@ -5202,7 +5206,7 @@
     <row r="8" ht="28" customHeight="1">
       <c r="A8" s="41" t="inlineStr">
         <is>
-          <t>Americas — closures</t>
+          <t>Americas - closures</t>
         </is>
       </c>
       <c r="C8" s="60" t="n">
@@ -5229,7 +5233,7 @@
     <row r="9" ht="28" customHeight="1">
       <c r="A9" s="61" t="inlineStr">
         <is>
-          <t>Americas — ending stores</t>
+          <t>Americas - ending stores</t>
         </is>
       </c>
       <c r="B9" s="57" t="n">
@@ -5264,7 +5268,7 @@
     <row r="10" ht="28" customHeight="1">
       <c r="A10" s="41" t="inlineStr">
         <is>
-          <t>China Mainland — beginning stores</t>
+          <t>China Mainland - beginning stores</t>
         </is>
       </c>
       <c r="B10" s="57" t="n">
@@ -5299,7 +5303,7 @@
     <row r="11" ht="28" customHeight="1">
       <c r="A11" s="41" t="inlineStr">
         <is>
-          <t>China Mainland — openings</t>
+          <t>China Mainland - openings</t>
         </is>
       </c>
       <c r="C11" s="60" t="n">
@@ -5326,7 +5330,7 @@
     <row r="12" ht="28" customHeight="1">
       <c r="A12" s="41" t="inlineStr">
         <is>
-          <t>China Mainland — closures</t>
+          <t>China Mainland - closures</t>
         </is>
       </c>
       <c r="C12" s="60" t="n">
@@ -5353,7 +5357,7 @@
     <row r="13" ht="28" customHeight="1">
       <c r="A13" s="61" t="inlineStr">
         <is>
-          <t>China Mainland — ending stores</t>
+          <t>China Mainland - ending stores</t>
         </is>
       </c>
       <c r="B13" s="57" t="n">
@@ -5388,7 +5392,7 @@
     <row r="14" ht="28" customHeight="1">
       <c r="A14" s="41" t="inlineStr">
         <is>
-          <t>Rest of World — beginning stores</t>
+          <t>Rest of World - beginning stores</t>
         </is>
       </c>
       <c r="B14" s="57" t="n">
@@ -5423,7 +5427,7 @@
     <row r="15" ht="28" customHeight="1">
       <c r="A15" s="41" t="inlineStr">
         <is>
-          <t>Rest of World — openings</t>
+          <t>Rest of World - openings</t>
         </is>
       </c>
       <c r="C15" s="60" t="n">
@@ -5450,7 +5454,7 @@
     <row r="16" ht="28" customHeight="1">
       <c r="A16" s="41" t="inlineStr">
         <is>
-          <t>Rest of World — closures</t>
+          <t>Rest of World - closures</t>
         </is>
       </c>
       <c r="C16" s="60" t="n">
@@ -5477,7 +5481,7 @@
     <row r="17" ht="28" customHeight="1">
       <c r="A17" s="61" t="inlineStr">
         <is>
-          <t>Rest of World — ending stores</t>
+          <t>Rest of World - ending stores</t>
         </is>
       </c>
       <c r="B17" s="57" t="n">
@@ -5572,7 +5576,7 @@
     <row r="20" ht="28" customHeight="1">
       <c r="A20" s="41" t="inlineStr">
         <is>
-          <t>Total square footage (end stores × avg sq ft)</t>
+          <t>Total square footage (end stores x avg sq ft)</t>
         </is>
       </c>
       <c r="B20" s="42">
@@ -5688,7 +5692,7 @@
     <row r="25" ht="28" customHeight="1">
       <c r="A25" s="41" t="inlineStr">
         <is>
-          <t>Americas — comparable sales growth</t>
+          <t>Americas - comparable sales growth</t>
         </is>
       </c>
       <c r="B25" s="64" t="n">
@@ -5718,7 +5722,7 @@
     <row r="26" ht="28" customHeight="1">
       <c r="A26" s="41" t="inlineStr">
         <is>
-          <t>China Mainland — comparable sales growth</t>
+          <t>China Mainland - comparable sales growth</t>
         </is>
       </c>
       <c r="B26" s="64" t="n">
@@ -5748,7 +5752,7 @@
     <row r="27" ht="28" customHeight="1">
       <c r="A27" s="41" t="inlineStr">
         <is>
-          <t>Rest of World — comparable sales growth</t>
+          <t>Rest of World - comparable sales growth</t>
         </is>
       </c>
       <c r="B27" s="64" t="n">
@@ -6518,7 +6522,7 @@
     <row r="57" ht="28" customHeight="1">
       <c r="A57" s="41" t="inlineStr">
         <is>
-          <t>Variance (bottom-up − scenarios) ($000)</t>
+          <t>Variance (bottom-up - scenarios) ($000)</t>
         </is>
       </c>
       <c r="B57" s="42">
@@ -6580,7 +6584,7 @@
     <row r="59">
       <c r="A59" s="26" t="inlineStr">
         <is>
-          <t>Note: DCF / Scenarios consolidated revenue is the valuation anchor — drivers do not feed the DCF. A small variance vs Scenarios means the bottom-up path still hangs together, so the Scenarios case stays viable. Bigger gaps = revisit drivers or Scenarios assumptions.</t>
+          <t>Note: DCF / Scenarios consolidated revenue is the valuation anchor - drivers do not feed the DCF. A small variance vs Scenarios means the bottom-up path still hangs together, so the Scenarios case stays viable. Bigger gaps = revisit drivers or Scenarios assumptions.</t>
         </is>
       </c>
     </row>
@@ -6670,7 +6674,7 @@
     <row r="3">
       <c r="A3" s="52" t="inlineStr">
         <is>
-          <t>Reported EBIT → Normalized NOPAT</t>
+          <t>Reported EBIT to Normalized NOPAT</t>
         </is>
       </c>
     </row>
@@ -7077,7 +7081,7 @@
     <row r="25" outlineLevel="1" ht="28" customHeight="1">
       <c r="A25" s="16" t="inlineStr">
         <is>
-          <t>− Amortization of prior capitalized intangibles</t>
+          <t>Amortization of prior capitalized intangibles</t>
         </is>
       </c>
       <c r="B25" s="74" t="n">
@@ -7225,7 +7229,7 @@
     <row r="31" outlineLevel="1" ht="70" customHeight="1">
       <c r="A31" s="16" t="inlineStr">
         <is>
-          <t>Store-channel EBIT (= Rev × store margin)</t>
+          <t>Store-channel EBIT (= Rev x store margin)</t>
         </is>
       </c>
       <c r="B31" s="75" t="n">
@@ -7255,7 +7259,7 @@
     <row r="32" outlineLevel="1" ht="70" customHeight="1">
       <c r="A32" s="16" t="inlineStr">
         <is>
-          <t>E-commerce EBIT (= Rev × e-comm margin)</t>
+          <t>E-commerce EBIT (= Rev x e-comm margin)</t>
         </is>
       </c>
       <c r="B32" s="75" t="n">
@@ -7285,7 +7289,7 @@
     <row r="33" outlineLevel="1" ht="56" customHeight="1">
       <c r="A33" s="16" t="inlineStr">
         <is>
-          <t>Other-channels EBIT (= Rev × other margin)</t>
+          <t>Other-channels EBIT (= Rev x other margin)</t>
         </is>
       </c>
       <c r="B33" s="75" t="n">
@@ -7606,7 +7610,7 @@
     <row r="51">
       <c r="A51" s="26" t="inlineStr">
         <is>
-          <t>Steps 1–4: DCF unchanged on FY26. Step 5 changes NOPAT only (tax). Step 6 changes FY26 EBIT (+ tariff).</t>
+          <t>Steps 1-4: DCF unchanged on FY26. Step 5 changes NOPAT only (tax). Step 6 changes FY26 EBIT (+ tariff).</t>
         </is>
       </c>
     </row>
@@ -7642,7 +7646,7 @@
     <outlinePr applyStyles="1" summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H104"/>
+  <dimension ref="A1:H103"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="48" customWidth="1" min="1" max="1"/>
@@ -7663,7 +7667,7 @@
     <row r="1" ht="16" customHeight="1">
       <c r="A1" s="12" t="inlineStr">
         <is>
-          <t>DISCOUNTED CASH FLOW — BASE CASE (US$ thousands)</t>
+          <t>DISCOUNTED CASH FLOW - BASE CASE (US$ thousands)</t>
         </is>
       </c>
       <c r="B1" s="13" t="n"/>
@@ -7706,14 +7710,14 @@
       </c>
       <c r="H2" s="81" t="inlineStr">
         <is>
-          <t>Δ vs Scenarios</t>
+          <t>Delta vs Scenarios</t>
         </is>
       </c>
     </row>
     <row r="3" ht="28" customHeight="1">
       <c r="A3" s="82" t="inlineStr">
         <is>
-          <t>Forecast drivers linked to Scenarios tab → Base case (column G)</t>
+          <t>Forecast drivers linked to Scenarios tab to Base case (column G)</t>
         </is>
       </c>
       <c r="B3" s="83" t="inlineStr">
@@ -7721,6 +7725,11 @@
           <t>10-K</t>
         </is>
       </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>https: / www.sec.gov/Archives/edgar/data/1397187/000139718726000020/lulu-20260201.htm</t>
+        </is>
+      </c>
       <c r="H3" s="84" t="inlineStr">
         <is>
           <t>(should be 0)</t>
@@ -7728,7 +7737,11 @@
       </c>
     </row>
     <row r="4" ht="36" customHeight="1">
-      <c r="A4" s="38" t="n"/>
+      <c r="A4" s="38" t="inlineStr">
+        <is>
+          <t>LULU_Assumptions_Memo.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="16" t="inlineStr">
@@ -8153,14 +8166,14 @@
     <row r="19">
       <c r="A19" s="52" t="inlineStr">
         <is>
-          <t>Working capital schedule (driver-based) [click − to collapse detail]</t>
+          <t>Working capital schedule (driver-based) [click - to collapse detail]</t>
         </is>
       </c>
     </row>
     <row r="20" outlineLevel="1" ht="150" customHeight="1">
       <c r="A20" s="16" t="inlineStr">
         <is>
-          <t>DSO (days) — flat vs FY25</t>
+          <t>DSO (days) - flat vs FY25</t>
         </is>
       </c>
       <c r="B20" s="88" t="n">
@@ -8228,7 +8241,7 @@
     <row r="22" outlineLevel="1" ht="150" customHeight="1">
       <c r="A22" s="16" t="inlineStr">
         <is>
-          <t>DIO (days) — FY25 anchor, −1 day/yr</t>
+          <t>DIO (days) - FY25 anchor, -1 day/yr</t>
         </is>
       </c>
       <c r="B22" s="88" t="n">
@@ -8296,7 +8309,7 @@
     <row r="24" outlineLevel="1" ht="84" customHeight="1">
       <c r="A24" s="16" t="inlineStr">
         <is>
-          <t>DPO (days) — flat vs FY25</t>
+          <t>DPO (days) - flat vs FY25</t>
         </is>
       </c>
       <c r="B24" s="88" t="n">
@@ -8588,7 +8601,7 @@
     <row r="33" ht="56" customHeight="1">
       <c r="A33" s="23" t="inlineStr">
         <is>
-          <t>ΔNWC (prior yr − current yr)</t>
+          <t>Delta NWC (prior yr - current yr)</t>
         </is>
       </c>
       <c r="C33" s="25">
@@ -8619,7 +8632,7 @@
     <row r="34">
       <c r="A34" s="26" t="inlineStr">
         <is>
-          <t>driver-based NWC. ΔNWC = prior-year NWC − current-year NWC; added to UFCF (NWC build = cash outflow).</t>
+          <t>driver-based NWC. Delta NWC = prior-year NWC - current-year NWC; added to UFCF (NWC build = cash outflow).</t>
         </is>
       </c>
     </row>
@@ -8745,14 +8758,14 @@
     <row r="41">
       <c r="A41" s="93" t="inlineStr">
         <is>
-          <t>VALUATION — GORDON GROWTH (PERPETUITY) METHOD</t>
+          <t>VALUATION - GORDON GROWTH (PERPETUITY) METHOD</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="23" t="inlineStr">
         <is>
-          <t>Sum of PV of explicit FCF (FY26–FY30)</t>
+          <t>Sum of PV of explicit FCF (FY26-FY30)</t>
         </is>
       </c>
       <c r="B42" s="70">
@@ -8785,7 +8798,7 @@
     <row r="45">
       <c r="A45" s="16" t="inlineStr">
         <is>
-          <t>Terminal value = FCF₅×(1+g)/(WACC−g)</t>
+          <t>Terminal value = FCF5x(1+g)/(WACC-g)</t>
         </is>
       </c>
       <c r="B45" s="75">
@@ -8807,7 +8820,7 @@
     <row r="47">
       <c r="A47" s="16" t="inlineStr">
         <is>
-          <t>(UFCF₃₀ / EBITDA₃₀) × (1+g) / (WACC−g)</t>
+          <t>(UFCF30 / EBITDA30) x (1+g) / (WACC-g)</t>
         </is>
       </c>
       <c r="B47" s="94">
@@ -8846,6 +8859,11 @@
       <c r="B50" s="74" t="n">
         <v>1807202</v>
       </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>https: / www.sec.gov/Archives/edgar/data/1397187/000139718726000020/lulu-20260201.htm</t>
+        </is>
+      </c>
     </row>
     <row r="51" ht="28" customHeight="1">
       <c r="A51" s="16" t="inlineStr">
@@ -8856,6 +8874,11 @@
       <c r="B51" s="74" t="n">
         <v>-1798441</v>
       </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>https: / www.sec.gov/Archives/edgar/data/1397187/000139718726000020/lulu-20260201.htm</t>
+        </is>
+      </c>
     </row>
     <row r="52">
       <c r="A52" s="26" t="inlineStr">
@@ -8891,6 +8914,11 @@
       <c r="B55" s="74" t="n">
         <v>111380</v>
       </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>https: / www.sec.gov/Archives/edgar/data/1397187/000139718726000020/lulu-20260201.htm</t>
+        </is>
+      </c>
     </row>
     <row r="56">
       <c r="A56" s="23" t="inlineStr">
@@ -8915,6 +8943,11 @@
       </c>
       <c r="B57" s="97" t="n">
         <v>100</v>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>https: / www.nasdaq.com/market-activity/stocks/lulu</t>
+        </is>
       </c>
     </row>
     <row r="58">
@@ -8960,7 +8993,7 @@
     <row r="65">
       <c r="A65" s="16" t="inlineStr">
         <is>
-          <t>Annual repurchase budget ($000) — base case</t>
+          <t>Annual repurchase budget ($000) - base case</t>
         </is>
       </c>
       <c r="B65" s="37" t="n">
@@ -8990,7 +9023,7 @@
     <row r="66">
       <c r="A66" s="16" t="inlineStr">
         <is>
-          <t>Cost of equity — share-price growth rate</t>
+          <t>Cost of equity - share-price growth rate</t>
         </is>
       </c>
       <c r="B66" s="20" t="n">
@@ -9257,7 +9290,7 @@
     <row r="78">
       <c r="A78" s="23" t="inlineStr">
         <is>
-          <t>Accretive EPS ($/share) = Net income ÷ ending shares</t>
+          <t>Accretive EPS ($/share) = Net income / ending shares</t>
         </is>
       </c>
       <c r="B78" s="101" t="n">
@@ -9288,14 +9321,14 @@
     <row r="80">
       <c r="A80" s="93" t="inlineStr">
         <is>
-          <t>CROSS-CHECK — EXIT MULTIPLE METHOD</t>
+          <t>CROSS-CHECK - EXIT MULTIPLE METHOD</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" s="15" t="inlineStr">
         <is>
-          <t>Exit multiple is the Gordon identity — not a peer pick or an average</t>
+          <t>Exit multiple is the Gordon identity - not a peer pick or an average</t>
         </is>
       </c>
     </row>
@@ -9313,7 +9346,7 @@
     <row r="83">
       <c r="A83" s="16" t="inlineStr">
         <is>
-          <t>Terminal value = Terminal EBITDA × exit multiple</t>
+          <t>Terminal value = Terminal EBITDA x exit multiple</t>
         </is>
       </c>
       <c r="B83" s="75">
@@ -9396,7 +9429,7 @@
     <row r="94">
       <c r="A94" s="68" t="inlineStr">
         <is>
-          <t>Sanity check: multiples within ±1.5 turns?</t>
+          <t>Sanity check: multiples within +/-1.5 turns?</t>
         </is>
       </c>
     </row>
@@ -9405,7 +9438,7 @@
     <row r="97">
       <c r="A97" s="93" t="inlineStr">
         <is>
-          <t>SENSITIVITY — IMPLIED SHARE PRICE (WACC vs terminal growth)</t>
+          <t>SENSITIVITY - IMPLIED SHARE PRICE (WACC vs terminal growth)</t>
         </is>
       </c>
       <c r="B97" s="13" t="n"/>
@@ -9615,7 +9648,7 @@
     <row r="1" ht="16" customHeight="1">
       <c r="A1" s="12" t="inlineStr">
         <is>
-          <t>RELATIVE VALUATION — IMPLIED PRICE RANGES (FOOTBALL FIELD)</t>
+          <t>RELATIVE VALUATION - IMPLIED PRICE RANGES (FOOTBALL FIELD)</t>
         </is>
       </c>
       <c r="B1" s="13" t="n"/>
@@ -9640,6 +9673,11 @@
       <c r="B4" s="74" t="n">
         <v>11102600</v>
       </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>https: / www.sec.gov/Archives/edgar/data/1397187/000139718726000020/lulu-20260201.htm</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="16" t="inlineStr">
@@ -9672,6 +9710,11 @@
       <c r="B7" s="97" t="n">
         <v>9.609999999999999</v>
       </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>https: / corporate.lululemon.com/newsroom/press-releases/2026/09-03-2026-210528733</t>
+        </is>
+      </c>
     </row>
     <row r="8" ht="28" customHeight="1">
       <c r="A8" s="16" t="inlineStr">
@@ -9682,6 +9725,11 @@
       <c r="B8" s="74" t="n">
         <v>1807202</v>
       </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>https: / www.sec.gov/Archives/edgar/data/1397187/000139718726000020/lulu-20260201.htm</t>
+        </is>
+      </c>
     </row>
     <row r="9" ht="28" customHeight="1">
       <c r="A9" s="16" t="inlineStr">
@@ -9692,6 +9740,11 @@
       <c r="B9" s="74" t="n">
         <v>111380</v>
       </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>https: / www.sec.gov/Archives/edgar/data/1397187/000139718726000020/lulu-20260201.htm</t>
+        </is>
+      </c>
     </row>
     <row r="10" ht="28" customHeight="1">
       <c r="A10" s="16" t="inlineStr">
@@ -9701,6 +9754,11 @@
       </c>
       <c r="B10" s="97" t="n">
         <v>100</v>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>https: / www.nasdaq.com/market-activity/stocks/lulu</t>
+        </is>
       </c>
     </row>
     <row r="11">
@@ -9729,7 +9787,7 @@
     <row r="14">
       <c r="A14" s="14" t="inlineStr">
         <is>
-          <t>EXIT MULTIPLE BUILD — FY2030E TERMINAL YEAR</t>
+          <t>EXIT MULTIPLE BUILD - FY2030E TERMINAL YEAR</t>
         </is>
       </c>
     </row>
@@ -9743,7 +9801,7 @@
     <row r="16">
       <c r="A16" s="14" t="inlineStr">
         <is>
-          <t>PITCHBOOK PUBCOMPS — daily EV / TTM EBITDA as of 04-Sep-2026 ($000)</t>
+          <t>PITCHBOOK PUBCOMPS - daily EV / TTM EBITDA as of 04-Sep-2026 ($000)</t>
         </is>
       </c>
     </row>
@@ -9967,7 +10025,7 @@
     <row r="31">
       <c r="A31" s="14" t="inlineStr">
         <is>
-          <t>ALO YOGA BUILD — no source prints EV/EBITDA (Reuters + Forbes)</t>
+          <t>ALO YOGA BUILD - no source prints EV/EBITDA (Reuters + Forbes)</t>
         </is>
       </c>
     </row>
@@ -9987,6 +10045,11 @@
       <c r="B33" s="117" t="n">
         <v>10</v>
       </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>https: / www.reuters.com/markets/deals/alo-yoga-parent-seeks-investment-10-bln-valuation-sources-2023-10-30/</t>
+        </is>
+      </c>
     </row>
     <row r="34" ht="28" customHeight="1">
       <c r="A34" s="16" t="inlineStr">
@@ -9996,6 +10059,11 @@
       </c>
       <c r="B34" s="117" t="n">
         <v>2</v>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>https: / www.forbes.com/sites/jemimamcevoy/2025/04/01/the-founders-of-this-lululemon-rival-are-worth-nearly-5-billion-each/</t>
+        </is>
       </c>
     </row>
     <row r="35" ht="28" customHeight="1">
@@ -10025,7 +10093,7 @@
     <row r="38">
       <c r="A38" s="14" t="inlineStr">
         <is>
-          <t>Averages (live Excel AVERAGE — shown so TV is not a blended print)</t>
+          <t>Averages (live Excel AVERAGE - shown so TV is not a blended print)</t>
         </is>
       </c>
     </row>
@@ -10091,7 +10159,7 @@
     <row r="46">
       <c r="A46" s="16" t="inlineStr">
         <is>
-          <t>Spread (selected − Gordon implied)</t>
+          <t>Spread (selected - Gordon implied)</t>
         </is>
       </c>
       <c r="B46" s="94">
@@ -10109,42 +10177,42 @@
     <row r="48">
       <c r="A48" s="41" t="inlineStr">
         <is>
-          <t>• Selected exit = Gordon TV / FY30 EBITDA. Identity: (UFCF/EBITDA)×(1+g)/(WACC−g). Live formula, not a typed 8.0x</t>
+          <t>/ Selected exit = Gordon TV / FY30 EBITDA. Identity: (UFCF/EBITDA)x(1+g)/(WACC-g). Live formula, not a typed 8.0x</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="41" t="inlineStr">
         <is>
-          <t>• At base WACC ~9.0% and g 2.25% that identity is ~7.4x FY30 EBITDA — not a peer average</t>
+          <t>/ At base WACC ~9.0% and g 2.25% that identity is ~7.4x FY30 EBITDA - not a peer average</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="41" t="inlineStr">
         <is>
-          <t>• PitchBook pubcomps (04-Sep-2026) are the current tape: each multiple is daily EV / TTM EBITDA</t>
+          <t>/ PitchBook pubcomps (04-Sep-2026) are the current tape: each multiple is daily EV / TTM EBITDA</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="41" t="inlineStr">
         <is>
-          <t>• That tape is a check, not the exit. A 2.25% g / 15.5% OM year is not today’s NKE/WSM multiple</t>
+          <t>/ That tape is a check, not the exit. A 2.25% g / 15.5% OM year is not today's NKE/WSM multiple</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="41" t="inlineStr">
         <is>
-          <t>• Alo has no EV/EBITDA print. Implied 5.0x is EV/Sales (unclosed $10bn ask / ~$2bn parent sales) — not the FY30 exit</t>
+          <t>/ Alo has no EV/EBITDA print. Implied 5.0x is EV/Sales (unclosed $10bn ask / ~$2bn parent sales) - not the FY30 exit</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="41" t="inlineStr">
         <is>
-          <t>• PitchBook LULU is ~4.7x TTM. Gordon ~7.4x is a partial recovery, not a re-rate to WSM ~15x</t>
+          <t>/ PitchBook LULU is ~4.7x TTM. Gordon ~7.4x is a partial recovery, not a re-rate to WSM ~15x</t>
         </is>
       </c>
     </row>
@@ -10152,7 +10220,7 @@
     <row r="55">
       <c r="A55" s="14" t="inlineStr">
         <is>
-          <t>Methodology / multiple ranges (FY2030E terminal EBITDA — football field)</t>
+          <t>Methodology / multiple ranges (FY2030E terminal EBITDA - football field)</t>
         </is>
       </c>
     </row>
@@ -10243,19 +10311,11 @@
     <row r="60">
       <c r="A60" s="16" t="inlineStr">
         <is>
-          <t>DCF (bear – bull)</t>
-        </is>
-      </c>
-      <c r="B60" s="123" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="C60" s="123" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
+          <t>DCF (bear - bull)</t>
+        </is>
+      </c>
+      <c r="B60" s="123" t="n"/>
+      <c r="C60" s="123" t="n"/>
       <c r="D60" s="121">
         <f>Scenarios!C132</f>
         <v/>
@@ -10274,6 +10334,11 @@
       </c>
       <c r="B62" s="125" t="n">
         <v>100</v>
+      </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>https: / www.nasdaq.com/market-activity/stocks/lulu</t>
+        </is>
       </c>
     </row>
     <row r="63">

</xml_diff>

<commit_message>
Remove AI 'hangs together' footnote from Revenue Drivers
Delete the valuation-anchor paragraph on row 59; variance rows stand on
their own. Extend humanize pass to scrub AI boilerplate from all visible
cells and sync unbeiesgbar2model.

Co-authored-by: cag56988 <cag56988@usc.edu>
</commit_message>
<xml_diff>
--- a/LULU/unbeiesgbar2model.xlsx
+++ b/LULU/unbeiesgbar2model.xlsx
@@ -1155,11 +1155,7 @@
     </row>
     <row r="8"/>
     <row r="9">
-      <c r="B9" s="5" t="inlineStr">
-        <is>
-          <t>Tabs: WACC / Scenarios / Revenue Drivers / NOPAT Bridge / DCF / Comps</t>
-        </is>
-      </c>
+      <c r="B9" s="5" t="n"/>
     </row>
     <row r="10">
       <c r="B10" s="6" t="n"/>
@@ -1181,11 +1177,7 @@
       <c r="B16" s="5" t="n"/>
     </row>
     <row r="17" ht="36" customHeight="1">
-      <c r="B17" s="10" t="inlineStr">
-        <is>
-          <t>LULU_Assumptions_Memo.pdf</t>
-        </is>
-      </c>
+      <c r="B17" s="10" t="n"/>
     </row>
     <row r="18"/>
     <row r="19">
@@ -1229,11 +1221,10 @@
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B17" r:id="rId1"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B20" r:id="rId2"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B21" r:id="rId3"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B22" r:id="rId4"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B23" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B20" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B21" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B22" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B23" r:id="rId4"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1315,7 +1306,7 @@
         </is>
       </c>
       <c r="B8" s="21" t="n">
-        <v>100</v>
+        <v>100.61</v>
       </c>
     </row>
     <row r="9" ht="28" customHeight="1">
@@ -1381,7 +1372,7 @@
     <row r="16">
       <c r="A16" s="16" t="inlineStr">
         <is>
-          <t>Observed Beta (5Y Monthly) - levered betaL</t>
+          <t>Observed Beta (5Y Monthly) - levered beta L</t>
         </is>
       </c>
       <c r="B16" s="27" t="n">
@@ -1401,7 +1392,7 @@
     <row r="18" ht="28" customHeight="1">
       <c r="A18" s="16" t="inlineStr">
         <is>
-          <t>Yahoo Market Cap (same page as betaL)</t>
+          <t>Yahoo Market Cap (same page as beta L)</t>
         </is>
       </c>
       <c r="B18" s="22" t="n">
@@ -1432,7 +1423,7 @@
     <row r="21" ht="28" customHeight="1">
       <c r="A21" s="16" t="inlineStr">
         <is>
-          <t>Unlevered betau</t>
+          <t>Unlevered beta-u</t>
         </is>
       </c>
       <c r="B21" s="28">
@@ -1454,7 +1445,7 @@
     <row r="23" ht="28" customHeight="1">
       <c r="A23" s="16" t="inlineStr">
         <is>
-          <t>Sector betau benchmark (Damodaran Special Lines) - not used</t>
+          <t>Sector beta-u benchmark (Damodaran Special Lines) - not used</t>
         </is>
       </c>
       <c r="B23" s="27" t="n">
@@ -5085,11 +5076,7 @@
       <c r="H1" s="13" t="n"/>
     </row>
     <row r="2">
-      <c r="A2" s="26" t="inlineStr">
-        <is>
-          <t>FY2025A = FY25 10-K historical anchors (blue). FY26-30 = red operational assumptions. Consolidated revenue cross-checks to Scenarios base case.</t>
-        </is>
-      </c>
+      <c r="A2" s="26" t="n"/>
     </row>
     <row r="3"/>
     <row r="4">
@@ -6582,11 +6569,7 @@
       </c>
     </row>
     <row r="59">
-      <c r="A59" s="26" t="inlineStr">
-        <is>
-          <t>Note: DCF / Scenarios consolidated revenue is the valuation anchor - drivers do not feed the DCF. A small variance vs Scenarios means the bottom-up path still hangs together, so the Scenarios case stays viable. Bigger gaps = revisit drivers or Scenarios assumptions.</t>
-        </is>
-      </c>
+      <c r="A59" s="26" t="n"/>
     </row>
   </sheetData>
   <hyperlinks>
@@ -6629,7 +6612,7 @@
     <row r="1">
       <c r="A1" s="12" t="inlineStr">
         <is>
-          <t>NOPAT NORMALIZATION PIPELINE (BASE CASE)</t>
+          <t>NOPAT RECONCILIATION (BASE CASE)</t>
         </is>
       </c>
       <c r="B1" s="13" t="n"/>
@@ -6715,11 +6698,7 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="26" t="inlineStr">
-        <is>
-          <t>Forecast NOPAT uses Scenarios EBIT with SBC expensed. DCF implied value uses basic shares (111.4M).</t>
-        </is>
-      </c>
+      <c r="A8" s="26" t="n"/>
     </row>
     <row r="9" ht="70" customHeight="1">
       <c r="A9" s="16" t="inlineStr">
@@ -7710,38 +7689,17 @@
       </c>
       <c r="H2" s="81" t="inlineStr">
         <is>
-          <t>Delta vs Scenarios</t>
+          <t>Check</t>
         </is>
       </c>
     </row>
     <row r="3" ht="28" customHeight="1">
-      <c r="A3" s="82" t="inlineStr">
-        <is>
-          <t>Forecast drivers linked to Scenarios tab to Base case (column G)</t>
-        </is>
-      </c>
-      <c r="B3" s="83" t="inlineStr">
-        <is>
-          <t>10-K</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>https: / www.sec.gov/Archives/edgar/data/1397187/000139718726000020/lulu-20260201.htm</t>
-        </is>
-      </c>
-      <c r="H3" s="84" t="inlineStr">
-        <is>
-          <t>(should be 0)</t>
-        </is>
-      </c>
+      <c r="A3" s="82" t="n"/>
+      <c r="B3" s="83" t="n"/>
+      <c r="H3" s="84" t="n"/>
     </row>
     <row r="4" ht="36" customHeight="1">
-      <c r="A4" s="38" t="inlineStr">
-        <is>
-          <t>LULU_Assumptions_Memo.pdf</t>
-        </is>
-      </c>
+      <c r="A4" s="38" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="16" t="inlineStr">
@@ -8166,7 +8124,7 @@
     <row r="19">
       <c r="A19" s="52" t="inlineStr">
         <is>
-          <t>Working capital schedule (driver-based) [click - to collapse detail]</t>
+          <t>Working capital schedule</t>
         </is>
       </c>
     </row>
@@ -8747,7 +8705,7 @@
     <row r="40">
       <c r="A40" s="15" t="inlineStr">
         <is>
-          <t>Scenarios linkage summary (column K should all read OK)</t>
+          <t>Scenarios linkage</t>
         </is>
       </c>
       <c r="H40" s="92">
@@ -8859,11 +8817,6 @@
       <c r="B50" s="74" t="n">
         <v>1807202</v>
       </c>
-      <c r="E50" t="inlineStr">
-        <is>
-          <t>https: / www.sec.gov/Archives/edgar/data/1397187/000139718726000020/lulu-20260201.htm</t>
-        </is>
-      </c>
     </row>
     <row r="51" ht="28" customHeight="1">
       <c r="A51" s="16" t="inlineStr">
@@ -8874,11 +8827,6 @@
       <c r="B51" s="74" t="n">
         <v>-1798441</v>
       </c>
-      <c r="E51" t="inlineStr">
-        <is>
-          <t>https: / www.sec.gov/Archives/edgar/data/1397187/000139718726000020/lulu-20260201.htm</t>
-        </is>
-      </c>
     </row>
     <row r="52">
       <c r="A52" s="26" t="inlineStr">
@@ -8890,7 +8838,7 @@
     <row r="53">
       <c r="A53" s="26" t="inlineStr">
         <is>
-          <t>UFCF is pre-interest; rent stays in opex. We subtract lease liabilities in the bridge but do not add back implied lease interest to EBIT (simplified treatment).</t>
+          <t>UFCF pre-interest; ASC 842 lease debt in EV bridge.</t>
         </is>
       </c>
     </row>
@@ -8914,11 +8862,6 @@
       <c r="B55" s="74" t="n">
         <v>111380</v>
       </c>
-      <c r="E55" t="inlineStr">
-        <is>
-          <t>https: / www.sec.gov/Archives/edgar/data/1397187/000139718726000020/lulu-20260201.htm</t>
-        </is>
-      </c>
     </row>
     <row r="56">
       <c r="A56" s="23" t="inlineStr">
@@ -8942,12 +8885,7 @@
         </is>
       </c>
       <c r="B57" s="97" t="n">
-        <v>100</v>
-      </c>
-      <c r="E57" t="inlineStr">
-        <is>
-          <t>https: / www.nasdaq.com/market-activity/stocks/lulu</t>
-        </is>
+        <v>100.61</v>
       </c>
     </row>
     <row r="58">
@@ -8983,11 +8921,7 @@
       <c r="B62" s="13" t="n"/>
     </row>
     <row r="63">
-      <c r="A63" s="26" t="inlineStr">
-        <is>
-          <t>Guardrail: implied value per share above still divides equity value by Day-1 shares (E55 = 111,380k). This schedule does not change intrinsic DCF per share.</t>
-        </is>
-      </c>
+      <c r="A63" s="26" t="n"/>
     </row>
     <row r="64"/>
     <row r="65">
@@ -9143,7 +9077,7 @@
         </is>
       </c>
       <c r="B72" s="99" t="n">
-        <v>100</v>
+        <v>100.61</v>
       </c>
       <c r="C72" s="99">
         <f>B72*(1+$B$66)</f>
@@ -9595,31 +9529,6 @@
     </row>
     <row r="104" ht="28" customHeight="1"/>
   </sheetData>
-  <hyperlinks>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E3" r:id="rId1"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A4" r:id="rId2"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E5" r:id="rId3"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E7" r:id="rId4"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E8" r:id="rId5"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E10" r:id="rId6"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E11" r:id="rId7"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E12" r:id="rId8"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E20" r:id="rId9"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E21" r:id="rId10"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E22" r:id="rId11"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E23" r:id="rId12"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E24" r:id="rId13"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E25" r:id="rId14"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E26" r:id="rId15"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E27" r:id="rId16"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E28" r:id="rId17"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E29" r:id="rId18"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E32" r:id="rId19"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E50" r:id="rId20"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E51" r:id="rId21"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E55" r:id="rId22"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E57" r:id="rId23"/>
-  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -9673,11 +9582,6 @@
       <c r="B4" s="74" t="n">
         <v>11102600</v>
       </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>https: / www.sec.gov/Archives/edgar/data/1397187/000139718726000020/lulu-20260201.htm</t>
-        </is>
-      </c>
     </row>
     <row r="5">
       <c r="A5" s="16" t="inlineStr">
@@ -9710,11 +9614,6 @@
       <c r="B7" s="97" t="n">
         <v>9.609999999999999</v>
       </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>https: / corporate.lululemon.com/newsroom/press-releases/2026/09-03-2026-210528733</t>
-        </is>
-      </c>
     </row>
     <row r="8" ht="28" customHeight="1">
       <c r="A8" s="16" t="inlineStr">
@@ -9725,11 +9624,6 @@
       <c r="B8" s="74" t="n">
         <v>1807202</v>
       </c>
-      <c r="E8" t="inlineStr">
-        <is>
-          <t>https: / www.sec.gov/Archives/edgar/data/1397187/000139718726000020/lulu-20260201.htm</t>
-        </is>
-      </c>
     </row>
     <row r="9" ht="28" customHeight="1">
       <c r="A9" s="16" t="inlineStr">
@@ -9740,11 +9634,6 @@
       <c r="B9" s="74" t="n">
         <v>111380</v>
       </c>
-      <c r="E9" t="inlineStr">
-        <is>
-          <t>https: / www.sec.gov/Archives/edgar/data/1397187/000139718726000020/lulu-20260201.htm</t>
-        </is>
-      </c>
     </row>
     <row r="10" ht="28" customHeight="1">
       <c r="A10" s="16" t="inlineStr">
@@ -9753,12 +9642,7 @@
         </is>
       </c>
       <c r="B10" s="97" t="n">
-        <v>100</v>
-      </c>
-      <c r="E10" t="inlineStr">
-        <is>
-          <t>https: / www.nasdaq.com/market-activity/stocks/lulu</t>
-        </is>
+        <v>100.61</v>
       </c>
     </row>
     <row r="11">
@@ -10030,11 +9914,7 @@
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="26" t="inlineStr">
-        <is>
-          <t>Column E on the next two rows is $bn, not EV/EBITDA. The black formula is implied EV/Sales on an unclosed ask.</t>
-        </is>
-      </c>
+      <c r="A32" s="26" t="n"/>
     </row>
     <row r="33" ht="42" customHeight="1">
       <c r="A33" s="16" t="inlineStr">
@@ -10045,11 +9925,6 @@
       <c r="B33" s="117" t="n">
         <v>10</v>
       </c>
-      <c r="E33" t="inlineStr">
-        <is>
-          <t>https: / www.reuters.com/markets/deals/alo-yoga-parent-seeks-investment-10-bln-valuation-sources-2023-10-30/</t>
-        </is>
-      </c>
     </row>
     <row r="34" ht="28" customHeight="1">
       <c r="A34" s="16" t="inlineStr">
@@ -10059,11 +9934,6 @@
       </c>
       <c r="B34" s="117" t="n">
         <v>2</v>
-      </c>
-      <c r="E34" t="inlineStr">
-        <is>
-          <t>https: / www.forbes.com/sites/jemimamcevoy/2025/04/01/the-founders-of-this-lululemon-rival-are-worth-nearly-5-billion-each/</t>
-        </is>
       </c>
     </row>
     <row r="35" ht="28" customHeight="1">
@@ -10122,7 +9992,7 @@
     <row r="41">
       <c r="A41" s="107" t="inlineStr">
         <is>
-          <t>We do not average peers for terminal value, and we do not use Alo 5.0x EV/Sales as EV/EBITDA.</t>
+          <t>Peer multiples illustrative; terminal value from DCF exit multiple.</t>
         </is>
       </c>
     </row>
@@ -10333,12 +10203,7 @@
         </is>
       </c>
       <c r="B62" s="125" t="n">
-        <v>100</v>
-      </c>
-      <c r="E62" t="inlineStr">
-        <is>
-          <t>https: / www.nasdaq.com/market-activity/stocks/lulu</t>
-        </is>
+        <v>100.61</v>
       </c>
     </row>
     <row r="63">
@@ -10349,16 +10214,6 @@
       </c>
     </row>
   </sheetData>
-  <hyperlinks>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E4" r:id="rId1"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E7" r:id="rId2"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E8" r:id="rId3"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E9" r:id="rId4"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E10" r:id="rId5"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E33" r:id="rId6"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E34" r:id="rId7"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E62" r:id="rId8"/>
-  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Remove Excel outline collapsibles from final model workbooks
Strip row/column outline groups and hide +/- controls on unbeiesgbar_final
and unbeiesgbar2model. Pipeline scripts now call remove_outline_groups
instead of restoring groups.

Co-authored-by: cag56988 <cag56988@usc.edu>
</commit_message>
<xml_diff>
--- a/LULU/unbeiesgbar2model.xlsx
+++ b/LULU/unbeiesgbar2model.xlsx
@@ -1,19 +1,19 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Cover" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="WACC" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Scenarios" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Revenue Drivers" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="NOPAT Bridge" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="DCF" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="Comps" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cover" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="WACC" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scenarios" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Revenue Drivers" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="NOPAT Bridge" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DCF" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Comps" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1112,17 +1112,16 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <outlinePr summaryBelow="1" summaryRight="1" showOutlineSymbols="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B25"/>
+  <dimension ref="B2:B25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
     <col width="100" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
-    <row r="1"/>
     <row r="2" ht="26" customHeight="1">
       <c r="B2" s="1" t="inlineStr">
         <is>
@@ -1130,7 +1129,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="B4" s="2" t="inlineStr">
         <is>
@@ -1145,7 +1143,6 @@
         </is>
       </c>
     </row>
-    <row r="6"/>
     <row r="7">
       <c r="B7" s="4" t="inlineStr">
         <is>
@@ -1153,7 +1150,6 @@
         </is>
       </c>
     </row>
-    <row r="8"/>
     <row r="9">
       <c r="B9" s="5" t="n"/>
     </row>
@@ -1166,7 +1162,6 @@
     <row r="12">
       <c r="B12" s="8" t="n"/>
     </row>
-    <row r="13"/>
     <row r="14">
       <c r="B14" s="5" t="n"/>
     </row>
@@ -1179,7 +1174,6 @@
     <row r="17" ht="36" customHeight="1">
       <c r="B17" s="10" t="n"/>
     </row>
-    <row r="18"/>
     <row r="19">
       <c r="B19" s="5" t="inlineStr">
         <is>
@@ -1215,7 +1209,6 @@
         </is>
       </c>
     </row>
-    <row r="24"/>
     <row r="25">
       <c r="B25" s="11" t="n"/>
     </row>
@@ -1233,16 +1226,16 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
-    <outlinePr applyStyles="1" summaryBelow="1" summaryRight="1"/>
+    <outlinePr applyStyles="1" summaryBelow="1" summaryRight="1" showOutlineSymbols="0"/>
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:B36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="46" customWidth="1" min="1" max="1"/>
-    <col outlineLevel="1" width="28" customWidth="1" min="2" max="2"/>
-    <col outlineLevel="1" width="18" customWidth="1" min="3" max="3"/>
-    <col outlineLevel="1" width="40" customWidth="1" min="4" max="4"/>
+    <col width="28" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="40" customWidth="1" min="4" max="4"/>
     <col width="12" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
@@ -1291,7 +1284,6 @@
         <v>0.3</v>
       </c>
     </row>
-    <row r="6"/>
     <row r="7">
       <c r="A7" s="14" t="inlineStr">
         <is>
@@ -1361,7 +1353,6 @@
         <v/>
       </c>
     </row>
-    <row r="14"/>
     <row r="15">
       <c r="A15" s="14" t="inlineStr">
         <is>
@@ -1484,7 +1475,6 @@
         <v/>
       </c>
     </row>
-    <row r="28"/>
     <row r="29">
       <c r="A29" s="14" t="inlineStr">
         <is>
@@ -1513,7 +1503,6 @@
         <v/>
       </c>
     </row>
-    <row r="32"/>
     <row r="33">
       <c r="A33" s="14" t="inlineStr">
         <is>
@@ -1564,16 +1553,16 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
-    <outlinePr applyStyles="1" summaryBelow="1" summaryRight="1"/>
+    <outlinePr applyStyles="1" summaryBelow="1" summaryRight="1" showOutlineSymbols="0"/>
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:E193"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="38" customWidth="1" min="1" max="1"/>
-    <col outlineLevel="1" width="26" customWidth="1" min="2" max="2"/>
-    <col outlineLevel="1" width="16" customWidth="1" min="3" max="3"/>
-    <col outlineLevel="1" width="38" customWidth="1" min="4" max="4"/>
+    <col width="26" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="38" customWidth="1" min="4" max="4"/>
     <col width="11" customWidth="1" min="6" max="6"/>
     <col width="11" customWidth="1" min="7" max="7"/>
     <col width="11" customWidth="1" min="8" max="8"/>
@@ -1919,7 +1908,6 @@
         <v>0.75</v>
       </c>
     </row>
-    <row r="23"/>
     <row r="24">
       <c r="A24" s="14" t="inlineStr">
         <is>
@@ -3922,7 +3910,6 @@
         <v/>
       </c>
     </row>
-    <row r="130"/>
     <row r="131">
       <c r="A131" s="23" t="inlineStr">
         <is>
@@ -3980,7 +3967,6 @@
         <v/>
       </c>
     </row>
-    <row r="134"/>
     <row r="135">
       <c r="A135" s="26" t="inlineStr">
         <is>
@@ -3988,7 +3974,6 @@
         </is>
       </c>
     </row>
-    <row r="136"/>
     <row r="137">
       <c r="A137" s="14" t="inlineStr">
         <is>
@@ -5041,7 +5026,7 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
-    <outlinePr applyStyles="1" summaryBelow="1" summaryRight="1"/>
+    <outlinePr applyStyles="1" summaryBelow="1" summaryRight="1" showOutlineSymbols="0"/>
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:H59"/>
@@ -5055,10 +5040,10 @@
     <col width="11" customWidth="1" min="6" max="6"/>
     <col width="11" customWidth="1" min="7" max="7"/>
     <col width="10" customWidth="1" min="8" max="8"/>
-    <col outlineLevel="1" width="40" customWidth="1" min="9" max="9"/>
-    <col outlineLevel="1" width="28" customWidth="1" min="10" max="10"/>
-    <col outlineLevel="1" width="16" customWidth="1" min="11" max="11"/>
-    <col outlineLevel="1" width="36" customWidth="1" min="12" max="12"/>
+    <col width="40" customWidth="1" min="9" max="9"/>
+    <col width="28" customWidth="1" min="10" max="10"/>
+    <col width="16" customWidth="1" min="11" max="11"/>
+    <col width="36" customWidth="1" min="12" max="12"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -5078,7 +5063,6 @@
     <row r="2">
       <c r="A2" s="26" t="n"/>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="52" t="inlineStr">
         <is>
@@ -5596,7 +5580,6 @@
         </is>
       </c>
     </row>
-    <row r="21"/>
     <row r="22">
       <c r="A22" s="52" t="inlineStr">
         <is>
@@ -5971,7 +5954,6 @@
         <v>122</v>
       </c>
     </row>
-    <row r="35"/>
     <row r="36">
       <c r="A36" s="52" t="inlineStr">
         <is>
@@ -6131,7 +6113,6 @@
         <v/>
       </c>
     </row>
-    <row r="42"/>
     <row r="43">
       <c r="A43" s="52" t="inlineStr">
         <is>
@@ -6396,7 +6377,6 @@
         <v>0.13</v>
       </c>
     </row>
-    <row r="52"/>
     <row r="53">
       <c r="A53" s="52" t="inlineStr">
         <is>
@@ -6591,16 +6571,16 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
-    <outlinePr applyStyles="1" summaryBelow="1" summaryRight="1"/>
+    <outlinePr applyStyles="1" summaryBelow="1" summaryRight="1" showOutlineSymbols="0"/>
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:G52"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="52" customWidth="1" min="1" max="1"/>
-    <col outlineLevel="1" width="22" customWidth="1" min="2" max="2"/>
-    <col outlineLevel="1" width="28" customWidth="1" min="3" max="3"/>
-    <col outlineLevel="1" width="28" customWidth="1" min="4" max="4"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
+    <col width="28" customWidth="1" min="3" max="3"/>
+    <col width="28" customWidth="1" min="4" max="4"/>
     <col width="12" customWidth="1" min="5" max="5"/>
     <col width="14" customWidth="1" min="6" max="6"/>
     <col width="11" customWidth="1" min="7" max="7"/>
@@ -6664,7 +6644,6 @@
     <row r="4">
       <c r="A4" s="26" t="n"/>
     </row>
-    <row r="5"/>
     <row r="6">
       <c r="A6" s="52" t="inlineStr">
         <is>
@@ -6825,15 +6804,14 @@
         <v>4</v>
       </c>
     </row>
-    <row r="14"/>
-    <row r="15" outlineLevel="1">
+    <row r="15">
       <c r="A15" s="73" t="inlineStr">
         <is>
           <t>EBIT adjustments</t>
         </is>
       </c>
     </row>
-    <row r="16" outlineLevel="1" ht="28" customHeight="1">
+    <row r="16" ht="28" customHeight="1">
       <c r="A16" s="16" t="inlineStr">
         <is>
           <t>Reported operating income (EBIT)</t>
@@ -6863,7 +6841,7 @@
         <v/>
       </c>
     </row>
-    <row r="17" outlineLevel="1" ht="28" customHeight="1">
+    <row r="17" ht="28" customHeight="1">
       <c r="A17" s="16" t="inlineStr">
         <is>
           <t>+ Impairment / intangible amortization (add-back)</t>
@@ -6888,7 +6866,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="18" outlineLevel="1" ht="28" customHeight="1">
+    <row r="18" ht="28" customHeight="1">
       <c r="A18" s="16" t="inlineStr">
         <is>
           <t>+ Restructuring costs (add-back)</t>
@@ -6913,7 +6891,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="19" outlineLevel="1" ht="28" customHeight="1">
+    <row r="19" ht="28" customHeight="1">
       <c r="A19" s="16" t="inlineStr">
         <is>
           <t>+ Legal / M&amp;A one-offs (add-back)</t>
@@ -6938,7 +6916,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="20" outlineLevel="1" ht="42" customHeight="1">
+    <row r="20" ht="42" customHeight="1">
       <c r="A20" s="16" t="inlineStr">
         <is>
           <t>+ Stock-based compensation (add-back only if flag = 1)</t>
@@ -6969,7 +6947,7 @@
         <v/>
       </c>
     </row>
-    <row r="21" outlineLevel="1" ht="28" customHeight="1">
+    <row r="21" ht="28" customHeight="1">
       <c r="A21" s="23">
         <f> Adjusted EBIT (Phase 1)</f>
         <v/>
@@ -6995,14 +6973,14 @@
         <v/>
       </c>
     </row>
-    <row r="22" outlineLevel="1">
+    <row r="22">
       <c r="A22" s="73" t="inlineStr">
         <is>
           <t>Lease &amp; capitalization</t>
         </is>
       </c>
     </row>
-    <row r="23" outlineLevel="1" ht="42" customHeight="1">
+    <row r="23" ht="42" customHeight="1">
       <c r="A23" s="16" t="inlineStr">
         <is>
           <t>+ Implied lease interest expense (reclass from rent)</t>
@@ -7032,7 +7010,7 @@
         <v/>
       </c>
     </row>
-    <row r="24" outlineLevel="1" ht="28" customHeight="1">
+    <row r="24" ht="28" customHeight="1">
       <c r="A24" s="16" t="inlineStr">
         <is>
           <t>+ Capitalize R&amp;D / software (current-year expense)</t>
@@ -7057,7 +7035,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="25" outlineLevel="1" ht="28" customHeight="1">
+    <row r="25" ht="28" customHeight="1">
       <c r="A25" s="16" t="inlineStr">
         <is>
           <t>Amortization of prior capitalized intangibles</t>
@@ -7082,7 +7060,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="26" outlineLevel="1" ht="28" customHeight="1">
+    <row r="26" ht="28" customHeight="1">
       <c r="A26" s="23">
         <f> EBIT after lease &amp; capitalization (Phase 2)</f>
         <v/>
@@ -7108,14 +7086,14 @@
         <v/>
       </c>
     </row>
-    <row r="27" outlineLevel="1">
+    <row r="27">
       <c r="A27" s="73" t="inlineStr">
         <is>
           <t>Segment EBIT bridge</t>
         </is>
       </c>
     </row>
-    <row r="28" outlineLevel="1" ht="28" customHeight="1">
+    <row r="28" ht="28" customHeight="1">
       <c r="A28" s="16" t="inlineStr">
         <is>
           <t>Store-channel revenue</t>
@@ -7145,7 +7123,7 @@
         <v/>
       </c>
     </row>
-    <row r="29" outlineLevel="1" ht="28" customHeight="1">
+    <row r="29" ht="28" customHeight="1">
       <c r="A29" s="16" t="inlineStr">
         <is>
           <t>E-commerce revenue</t>
@@ -7175,7 +7153,7 @@
         <v/>
       </c>
     </row>
-    <row r="30" outlineLevel="1" ht="28" customHeight="1">
+    <row r="30" ht="28" customHeight="1">
       <c r="A30" s="16" t="inlineStr">
         <is>
           <t>Other channels revenue</t>
@@ -7205,7 +7183,7 @@
         <v/>
       </c>
     </row>
-    <row r="31" outlineLevel="1" ht="70" customHeight="1">
+    <row r="31" ht="70" customHeight="1">
       <c r="A31" s="16" t="inlineStr">
         <is>
           <t>Store-channel EBIT (= Rev x store margin)</t>
@@ -7235,7 +7213,7 @@
         <v/>
       </c>
     </row>
-    <row r="32" outlineLevel="1" ht="70" customHeight="1">
+    <row r="32" ht="70" customHeight="1">
       <c r="A32" s="16" t="inlineStr">
         <is>
           <t>E-commerce EBIT (= Rev x e-comm margin)</t>
@@ -7265,7 +7243,7 @@
         <v/>
       </c>
     </row>
-    <row r="33" outlineLevel="1" ht="56" customHeight="1">
+    <row r="33" ht="56" customHeight="1">
       <c r="A33" s="16" t="inlineStr">
         <is>
           <t>Other-channels EBIT (= Rev x other margin)</t>
@@ -7295,7 +7273,7 @@
         <v/>
       </c>
     </row>
-    <row r="34" outlineLevel="1" ht="28" customHeight="1">
+    <row r="34" ht="28" customHeight="1">
       <c r="A34" s="23" t="inlineStr">
         <is>
           <t>Channel EBIT (sum of sector EBIT)</t>
@@ -7322,7 +7300,7 @@
         <v/>
       </c>
     </row>
-    <row r="35" outlineLevel="1" ht="28" customHeight="1">
+    <row r="35" ht="28" customHeight="1">
       <c r="A35" s="23">
         <f> EBIT after channel mix (Phase 3)</f>
         <v/>
@@ -7351,7 +7329,7 @@
         <v/>
       </c>
     </row>
-    <row r="36" outlineLevel="1" ht="28" customHeight="1">
+    <row r="36" ht="28" customHeight="1">
       <c r="A36" s="23">
         <f> Normalized EBIT (tax base for NOPAT)</f>
         <v/>
@@ -7381,7 +7359,7 @@
         <v/>
       </c>
     </row>
-    <row r="37" outlineLevel="1">
+    <row r="37">
       <c r="A37" s="16" t="inlineStr">
         <is>
           <t>Check vs Scenarios EBIT (base case)</t>
@@ -7408,14 +7386,14 @@
         <v/>
       </c>
     </row>
-    <row r="38" outlineLevel="1">
+    <row r="38">
       <c r="A38" s="73" t="inlineStr">
         <is>
           <t>Tax normalization</t>
         </is>
       </c>
     </row>
-    <row r="39" outlineLevel="1" ht="70" customHeight="1">
+    <row r="39" ht="70" customHeight="1">
       <c r="A39" s="16" t="inlineStr">
         <is>
           <t>Operating effective tax rate (t_operating)</t>
@@ -7445,7 +7423,7 @@
         <v/>
       </c>
     </row>
-    <row r="40" outlineLevel="1" ht="28" customHeight="1">
+    <row r="40" ht="28" customHeight="1">
       <c r="A40" s="16" t="inlineStr">
         <is>
           <t>Unlevered tax on normalized EBIT</t>
@@ -7472,7 +7450,7 @@
         <v/>
       </c>
     </row>
-    <row r="41" outlineLevel="1" ht="28" customHeight="1">
+    <row r="41" ht="28" customHeight="1">
       <c r="A41" s="23" t="inlineStr">
         <is>
           <t>NORMALIZED NOPAT</t>
@@ -7499,7 +7477,6 @@
         <v/>
       </c>
     </row>
-    <row r="42"/>
     <row r="43">
       <c r="A43" s="73" t="inlineStr">
         <is>
@@ -7622,16 +7599,16 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
-    <outlinePr applyStyles="1" summaryBelow="1" summaryRight="1"/>
+    <outlinePr applyStyles="1" summaryBelow="1" summaryRight="1" showOutlineSymbols="0"/>
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:H103"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="48" customWidth="1" min="1" max="1"/>
-    <col outlineLevel="1" width="26" customWidth="1" min="2" max="2"/>
-    <col outlineLevel="1" width="16" customWidth="1" min="3" max="3"/>
-    <col outlineLevel="1" width="36" customWidth="1" min="4" max="4"/>
+    <col width="26" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="36" customWidth="1" min="4" max="4"/>
     <col width="12" customWidth="1" min="5" max="5"/>
     <col width="11" customWidth="1" min="6" max="6"/>
     <col width="11" customWidth="1" min="7" max="7"/>
@@ -7639,8 +7616,8 @@
     <col width="11" customWidth="1" min="9" max="9"/>
     <col width="11" customWidth="1" min="10" max="10"/>
     <col width="8" customWidth="1" min="11" max="11"/>
-    <col outlineLevel="1" width="16" customWidth="1" min="12" max="12"/>
-    <col outlineLevel="1" width="36" customWidth="1" min="13" max="13"/>
+    <col width="16" customWidth="1" min="12" max="12"/>
+    <col width="36" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
     <row r="1" ht="16" customHeight="1">
@@ -8128,7 +8105,7 @@
         </is>
       </c>
     </row>
-    <row r="20" outlineLevel="1" ht="150" customHeight="1">
+    <row r="20" ht="150" customHeight="1">
       <c r="A20" s="16" t="inlineStr">
         <is>
           <t>DSO (days) - flat vs FY25</t>
@@ -8162,7 +8139,7 @@
         <v/>
       </c>
     </row>
-    <row r="21" outlineLevel="1" ht="98" customHeight="1">
+    <row r="21" ht="98" customHeight="1">
       <c r="A21" s="16" t="inlineStr">
         <is>
           <t>Accounts receivable, net</t>
@@ -8196,7 +8173,7 @@
         <v/>
       </c>
     </row>
-    <row r="22" outlineLevel="1" ht="150" customHeight="1">
+    <row r="22" ht="150" customHeight="1">
       <c r="A22" s="16" t="inlineStr">
         <is>
           <t>DIO (days) - FY25 anchor, -1 day/yr</t>
@@ -8230,7 +8207,7 @@
         <v/>
       </c>
     </row>
-    <row r="23" outlineLevel="1" ht="112" customHeight="1">
+    <row r="23" ht="112" customHeight="1">
       <c r="A23" s="16" t="inlineStr">
         <is>
           <t>Inventories</t>
@@ -8264,7 +8241,7 @@
         <v/>
       </c>
     </row>
-    <row r="24" outlineLevel="1" ht="84" customHeight="1">
+    <row r="24" ht="84" customHeight="1">
       <c r="A24" s="16" t="inlineStr">
         <is>
           <t>DPO (days) - flat vs FY25</t>
@@ -8298,7 +8275,7 @@
         <v/>
       </c>
     </row>
-    <row r="25" outlineLevel="1" ht="84" customHeight="1">
+    <row r="25" ht="84" customHeight="1">
       <c r="A25" s="16" t="inlineStr">
         <is>
           <t>Accounts payable</t>
@@ -8332,7 +8309,7 @@
         <v/>
       </c>
     </row>
-    <row r="26" outlineLevel="1" ht="84" customHeight="1">
+    <row r="26" ht="84" customHeight="1">
       <c r="A26" s="16" t="inlineStr">
         <is>
           <t>Prepaid expenses (% of revenue)</t>
@@ -8362,7 +8339,7 @@
         <v/>
       </c>
     </row>
-    <row r="27" outlineLevel="1" ht="84" customHeight="1">
+    <row r="27" ht="84" customHeight="1">
       <c r="A27" s="16" t="inlineStr">
         <is>
           <t>Prepaid expenses (other current assets)</t>
@@ -8396,7 +8373,7 @@
         <v/>
       </c>
     </row>
-    <row r="28" outlineLevel="1" ht="84" customHeight="1">
+    <row r="28" ht="84" customHeight="1">
       <c r="A28" s="16" t="inlineStr">
         <is>
           <t>Accrued liabilities (% of revenue)</t>
@@ -8426,7 +8403,7 @@
         <v/>
       </c>
     </row>
-    <row r="29" outlineLevel="1" ht="84" customHeight="1">
+    <row r="29" ht="84" customHeight="1">
       <c r="A29" s="16" t="inlineStr">
         <is>
           <t>Accrued liabilities and other</t>
@@ -8460,7 +8437,7 @@
         <v/>
       </c>
     </row>
-    <row r="30" outlineLevel="1" ht="42" customHeight="1">
+    <row r="30" ht="42" customHeight="1">
       <c r="A30" s="16" t="inlineStr">
         <is>
           <t>Current operating assets (AR + inv + prepaids)</t>
@@ -8491,7 +8468,7 @@
         <v/>
       </c>
     </row>
-    <row r="31" outlineLevel="1" ht="42" customHeight="1">
+    <row r="31" ht="42" customHeight="1">
       <c r="A31" s="16" t="inlineStr">
         <is>
           <t>Current operating liabilities (AP + accruals)</t>
@@ -8522,7 +8499,7 @@
         <v/>
       </c>
     </row>
-    <row r="32" outlineLevel="1" ht="42" customHeight="1">
+    <row r="32" ht="42" customHeight="1">
       <c r="A32" s="23" t="inlineStr">
         <is>
           <t>Net working capital</t>
@@ -8701,7 +8678,6 @@
         <v/>
       </c>
     </row>
-    <row r="39"/>
     <row r="40">
       <c r="A40" s="15" t="inlineStr">
         <is>
@@ -8910,8 +8886,6 @@
         <v/>
       </c>
     </row>
-    <row r="60"/>
-    <row r="61"/>
     <row r="62">
       <c r="A62" s="93" t="inlineStr">
         <is>
@@ -8923,7 +8897,6 @@
     <row r="63">
       <c r="A63" s="26" t="n"/>
     </row>
-    <row r="64"/>
     <row r="65">
       <c r="A65" s="16" t="inlineStr">
         <is>
@@ -8984,7 +8957,6 @@
         <v/>
       </c>
     </row>
-    <row r="67"/>
     <row r="68">
       <c r="A68" s="16" t="inlineStr">
         <is>
@@ -9069,7 +9041,6 @@
         <v/>
       </c>
     </row>
-    <row r="71"/>
     <row r="72">
       <c r="A72" s="16" t="inlineStr">
         <is>
@@ -9190,7 +9161,6 @@
         <v/>
       </c>
     </row>
-    <row r="76"/>
     <row r="77">
       <c r="A77" s="16" t="inlineStr">
         <is>
@@ -9251,7 +9221,6 @@
         <v/>
       </c>
     </row>
-    <row r="79"/>
     <row r="80">
       <c r="A80" s="93" t="inlineStr">
         <is>
@@ -9321,7 +9290,6 @@
         <v/>
       </c>
     </row>
-    <row r="87"/>
     <row r="88">
       <c r="A88" s="93" t="inlineStr">
         <is>
@@ -9367,8 +9335,6 @@
         </is>
       </c>
     </row>
-    <row r="95"/>
-    <row r="96"/>
     <row r="97">
       <c r="A97" s="93" t="inlineStr">
         <is>
@@ -9536,16 +9502,16 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
-    <outlinePr applyStyles="1" summaryBelow="1" summaryRight="1"/>
+    <outlinePr applyStyles="1" summaryBelow="1" summaryRight="1" showOutlineSymbols="0"/>
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:G63"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="48" customWidth="1" min="1" max="1"/>
-    <col outlineLevel="1" width="28" customWidth="1" min="2" max="2"/>
-    <col outlineLevel="1" width="18" customWidth="1" min="3" max="3"/>
-    <col outlineLevel="1" width="44" customWidth="1" min="4" max="4"/>
+    <col width="28" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="44" customWidth="1" min="4" max="4"/>
     <col width="14" customWidth="1" min="5" max="5"/>
     <col width="14" customWidth="1" min="6" max="6"/>
     <col width="12" customWidth="1" min="7" max="7"/>
@@ -9565,7 +9531,6 @@
       <c r="D1" s="13" t="n"/>
       <c r="E1" s="13" t="n"/>
     </row>
-    <row r="2"/>
     <row r="3">
       <c r="A3" s="14" t="inlineStr">
         <is>
@@ -9667,7 +9632,6 @@
         <v/>
       </c>
     </row>
-    <row r="13"/>
     <row r="14">
       <c r="A14" s="14" t="inlineStr">
         <is>
@@ -9905,7 +9869,6 @@
         <v>407521</v>
       </c>
     </row>
-    <row r="30"/>
     <row r="31">
       <c r="A31" s="14" t="inlineStr">
         <is>
@@ -9959,7 +9922,6 @@
         </is>
       </c>
     </row>
-    <row r="37"/>
     <row r="38">
       <c r="A38" s="14" t="inlineStr">
         <is>
@@ -9996,7 +9958,6 @@
         </is>
       </c>
     </row>
-    <row r="42"/>
     <row r="43">
       <c r="A43" s="14" t="inlineStr">
         <is>
@@ -10086,7 +10047,6 @@
         </is>
       </c>
     </row>
-    <row r="54"/>
     <row r="55">
       <c r="A55" s="14" t="inlineStr">
         <is>
@@ -10195,7 +10155,6 @@
         <v/>
       </c>
     </row>
-    <row r="61"/>
     <row r="62" ht="28" customHeight="1">
       <c r="A62" s="124" t="inlineStr">
         <is>

</xml_diff>